<commit_message>
chore: backup research workflow updates
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1,48 +1,196 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="14175" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI产业链" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AI产业链" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI产业链'!$A$1:$D$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI产业链'!$A$1:$D$97</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="23">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <charset val="134"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Microsoft YaHei"/>
-      <sz val="10"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Microsoft YaHei"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -51,16 +199,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEFF3"/>
+        <fgColor rgb="FFEAEAEA"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAEAEA"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -70,56 +400,327 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9DDE3"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9DDE3"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9DDE3"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9DDE3"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -472,7 +1073,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -482,8 +1082,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D83"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D97"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -492,1833 +1092,2141 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>细分板块</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>公司名称</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>200G EML / InP激光器</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>002384</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>东山精密</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>通过索尔思切入高速光芯片/光模块链条，公开披露100G/200G PAM4 EML相关进展，是200G EML国产映射之一。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>200G EML / InP激光器</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>688498</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>源杰科技</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>100G EML验证、200G EML推进，同时布局CW激光器，属于光芯片上游高弹性标的。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>200G EML / InP激光器</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>688048</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>长光华芯</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>具备EML、CW、PD等光通信芯片矩阵，高功率半导体激光器能力可向AI光通信延展。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>200G EML / InP激光器</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>688313</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>仕佳光子</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CW/DFB及光芯片方向处在送样、小批量阶段，确定性弱于已明确放量公司。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>InP衬底 / 外延</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>002428</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>云南锗业</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>通过云南鑫耀切入InP衬底，A股里InP衬底扩产映射最直接。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>InP衬底 / 外延</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>002975</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>博杰股份</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>通过珠海鼎泰芯源参与InP/GaSb等III-V族化合物衬底，参与度有线索但确定性低于云南锗业。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>低介电电子布 / 电子纱</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>002080</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>中材科技</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>偏高端特种电子布和低介电电子布，AI PCB材料链最硬瓶颈之一。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>低介电电子布 / 电子纱</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>603256</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>宏和科技</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>电子布主业纯度高，高端电子布弹性较强。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>低介电电子布 / 电子纱</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>600176</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>中国巨石</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>电子级玻纤规模龙头，优势在规模和玻纤体系，但AI高端电子布弹性不如纯标的。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>低介电电子布 / 电子纱</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>301526</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>国际复材</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>有电子纱/电子布布局，位置在玻纤和电子材料上游。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>HVLP / 高端铜箔</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>301511</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>德福科技</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>AI PCB高端铜箔主线，HVLP高端布局明确。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>HVLP / 高端铜箔</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>301217</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>铜冠铜箔</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>铜箔平台更稳健，具备高端铜箔布局和客户基础。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>HVLP / 高端铜箔</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>600110</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>诺德股份</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>有高端铜箔布局，但AI PCB主线确定性弱于德福。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>HVLP / 高端铜箔</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>688388</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>嘉元科技</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>偏验证放量弹性，铜箔补涨属性较强但确定性弱于德福。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>CW / UHP激光器</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>688498</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>源杰科技</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>布局CW激光器，硅光/CPO外置光源升级方向受益。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>CW / UHP激光器</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>002384</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>东山精密</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>索尔思体系覆盖高速光源与模块，CW/DFB高功率光源方向有布局。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>CW / UHP激光器</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>688048</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>长光华芯</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>高功率光源能力较强，EML/CW/PD矩阵可覆盖硅光和高速光模块需求。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>CW / UHP激光器</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>688313</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>仕佳光子</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>具备CW/DFB相关布局，但当前仍偏验证和小批量阶段。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>光DSP / 200G SerDes</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>暂无</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>暂无合格A股纯标的</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>这一环节主要由Broadcom、Marvell等海外厂商主导，A股暂不硬凑DSP/SerDes纯标的。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>M8 / M9高速CCL / 半固化片</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>688519</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>南亚新材</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>披露AI服务器、光模块用高速板材料，是高速CCL弹性标的。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>M8 / M9高速CCL / 半固化片</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>600183</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>生益科技</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>平台型CCL龙头，客户和产品覆盖最完整，确定性强。</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>M8 / M9高速CCL / 半固化片</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>603186</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>华正新材</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>聚焦服务器、交换机、光模块相关高频高速材料，弹性看高端材料放量。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>002463</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>沪电股份</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>AI服务器和高速交换机PCB主线，高多层高速板客户和产品验证最直接。</t>
         </is>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>002916</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>深南电路</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>PCB综合龙头，通信、数据中心和封装基板平台完整，AI服务器相关需求拉动明确。</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>300476</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>胜宏科技</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>高多层PCB、HDI和AI服务器/算力硬件方向弹性强，偏高弹性板厂。</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>高速连接器 / 线缆</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>002475</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>立讯精密</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>覆盖高速铜缆、背板连接器、内部/外部互连、光模块、电源和热管理，是铜光电热平台型选手。</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>高速连接器 / 线缆</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>002130</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>沃尔核材</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>偏高速通信线缆，224G、800G、1.6T方向明确，核心看高速线订单和客户验证。</t>
         </is>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>高速连接器 / 线缆</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>688629</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>华丰科技</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>偏高速背板连接器、高速模组和数据中心高速传输连接器，国产AI服务器链条相关度高。</t>
         </is>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>高速电子树脂</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>605589</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>圣泉集团</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>PPO、碳氢、活性酯等树脂平台更宽，材料平台属性强。</t>
         </is>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>高速电子树脂</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>601208</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>东材科技</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>高速电子树脂兑现更直接，AI服务器板级材料收入弹性更清晰。</t>
         </is>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>高速电子树脂</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>603002</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>宏昌电子</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>偏电子级环氧树脂和高频高速材料，位置更偏基础树脂供应。</t>
         </is>
       </c>
     </row>
     <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>TIA / Driver</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>暂无</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>暂无成熟A股纯标的</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>国内有模拟前端、CDR等布局，但尚未形成可明确映射AI光模块主线的成熟A股纯标的。</t>
         </is>
       </c>
     </row>
     <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>液冷</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>002837</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>英维克</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>覆盖冷板、Manifold、快接头、CDU、液冷工质、机房/机柜温控，液冷收入兑现度高。</t>
         </is>
       </c>
     </row>
     <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>液冷</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>301018</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>申菱环境</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>数据中心液冷、CDU、液冷机柜方向明确，AI算力液冷场景相关度高。</t>
         </is>
       </c>
     </row>
     <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>液冷</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>300990</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>同飞股份</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>从工业温控切入数据中心液冷，产品包括CDU、Manifold、预制管路、干冷器、集成冷站、浸没式TANK。</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="37" ht="16.5" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>液冷</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>300499</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>高澜股份</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>覆盖服务器液冷板、Manifold、CDU、TANK等环节，弹性看数据中心液冷订单兑现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>硅光PIC / CPO光引擎</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>000988</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>华工科技</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>华工正源布局CPO、ELSFP、硅光模块，属于硅光/CPO模块平台方向。</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>硅光PIC / CPO光引擎</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>002281</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>光迅科技</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>具备芯片、器件、模块平台，硅光和光电器件能力较完整。</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>硅光PIC / CPO光引擎</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>300394</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>天孚通信</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>偏FAU、POSA、光引擎核心器件，是硅光/CPO耦合和封装环节关键供应商。</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="41" ht="36" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>光模块</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>300308</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>中际旭创</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>高速数通光模块核心龙头，400G/800G/1.6T云数据中心客户放量主线，确定性最强。</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="42" ht="36" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>光模块</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>300502</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>新易盛</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>高速光模块高弹性龙头，800G/1.6T产品与海外云客户需求弹性强。</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>光模块</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>002281</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>光迅科技</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>芯片、器件、模块一体化平台，电信和数通覆盖完整，确定性强但AI数通弹性弱于中际/新易盛。</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44" ht="36" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>法拉第旋光片 / 光隔离器</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>002222</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>福晶科技</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>光通信法拉第旋光片与TGG/TSAG磁光晶体国产替代标的，当前小批量供货，核心看客户验证、扩产和收入占比提升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="36" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>FAU / MT / MPO / 微透镜 / 无源件</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>300394</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>天孚通信</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>偏FAU、POSA、光引擎和高精度光器件，是AI光模块无源器件核心公司。</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>FAU / MT / MPO / 微透镜 / 无源件</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>300570</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>太辰光</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>偏MPO/MTP连接器和光纤连接器，受益于高密度光连接需求。</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="47" ht="36" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>FAU / MT / MPO / 微透镜 / 无源件</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>688167</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>炬光科技</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>偏微光学、V槽、耦合元件等精密光学器件。</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="36" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="48" ht="36" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>光模块封装 / 耦合 / 测试设备</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>300757</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>罗博特科</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>通过ficonTEC参与光子封装、主动耦合和测试设备，是高端光模块设备映射。</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="36" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="49" ht="36" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>光模块封装 / 耦合 / 测试设备</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>688097</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>博众精工</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>披露过400G/800G光模块设备订单，偏自动化装配和测试设备。</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="36" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="50" ht="36" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>光模块封装 / 耦合 / 测试设备</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>603203</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>快克智能</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>涉及光模块AOI、焊接检测等设备，偏检测和精密制造环节。</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="36" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="51" ht="36" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>光模块封装 / 耦合 / 测试设备</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>002957</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>科瑞技术</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>有光模块设备收入，但占比较小，相关度低于罗博特科和博众精工。</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="36" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="52" ht="36" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>电源 / 供电</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>300870</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>欧陆通</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>服务器电源和数据中心电源标的，PSU、高功率服务器电源、液冷PSU方向清晰。</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="36" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="53" ht="36" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>电源 / 供电</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>002851</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>麦格米特</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>AI服务器电源和数据中心供电方案方向明确，重点看验证导入转规模收入。</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="36" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="54" ht="36" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>电源 / 供电</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>002138</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>顺络电子</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>不是PSU整机，偏功率电感、变压器、钽电容等AI服务器供电上游核心元件。</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="36" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>PD / APD / 接收芯片</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>002281</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>光迅科技</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>具备PD/APD及硅光平台能力，光芯片和器件平台属性较强。</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="36" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+    <row r="56" ht="36" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>PD / APD / 接收芯片</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>688048</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>长光华芯</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>具备PIN、PD、VCSEL、EML等光通信芯片矩阵，覆盖发射和接收侧。</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="36" customHeight="1">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="57" ht="36" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>球硅 / 低Df填料</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>688300</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>联瑞新材</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>硅微粉、球形硅微粉主线，低Df填料和封装/覆铜板填料相关度高。</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="36" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="58" ht="36" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>球硅 / 低Df填料</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>300285</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>国瓷材料</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>具备铜板填充材料和陶瓷材料平台，AIPCB相关度偏材料延伸。</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="36" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="59" ht="36" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>球硅 / 低Df填料</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>688733</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>壹石通</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>偏球形氧化铝和封装材料，和AIPCB相关度更间接。</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="36" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="60" ht="36" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>PCB设备</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>301200</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>大族数控</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>覆盖钻孔、曝光、成型、检测等PCB专用设备，是PCB设备主线。</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="36" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
+    <row r="61" ht="36" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>PCB设备</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>688630</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>芯碁微装</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>偏PCB直接成像设备，受益于高精度图形转移需求。</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="36" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
+    <row r="62" ht="36" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>PCB钻针 / 微钻 / 刀具</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>301377</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>鼎泰高科</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>PCB钻针主线，受益于高多层、硬材料和细孔径升级。</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="36" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
+    <row r="63" ht="36" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>PCB钻针 / 微钻 / 刀具</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>000657</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>中钨高新</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>通过金洲公司具备PCB微型刀具产能，偏刀具耗材。</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="36" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
+    <row r="64" ht="36" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>高多层PCB加工设备耗材</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>301200</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>大族数控</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>高多层AIPCB带动钻孔、曝光、成型、检测等设备升级。</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="36" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="65" ht="36" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>高多层PCB加工设备耗材</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>301377</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>鼎泰高科</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>高多层、硬材料、细孔径带动PCB钻针和微钻耗材需求。</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="36" customHeight="1">
-      <c r="A64" s="4" t="inlineStr">
+    <row r="66" ht="36" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>高多层PCB加工设备耗材</t>
         </is>
       </c>
-      <c r="B64" s="5" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>000657</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>中钨高新</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>通过PCB微型刀具产能参与耗材升级，受益于细孔径加工。</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="36" customHeight="1">
-      <c r="A65" s="4" t="inlineStr">
+    <row r="67" ht="36" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>TFLN / 薄膜铌酸锂</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>300620</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>光库科技</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>偏薄膜铌酸锂调制器与光子集成，是TFLN器件方向核心映射。</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="36" customHeight="1">
-      <c r="A66" s="4" t="inlineStr">
+    <row r="68" ht="36" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>TFLN / 薄膜铌酸锂</t>
         </is>
       </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>600330</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>天通股份</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>偏铌酸锂晶体、晶片和材料端，位置更上游。</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="36" customHeight="1">
-      <c r="A67" s="4" t="inlineStr">
+    <row r="69" ht="36" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>散热材料</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>300684</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>中石科技</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>导热界面材料、石墨散热、VC和热管理组件，服务器/数据中心和北美大客户线索明确。</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="36" customHeight="1">
-      <c r="A68" s="4" t="inlineStr">
+    <row r="70" ht="36" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>散热材料</t>
         </is>
       </c>
-      <c r="B68" s="5" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>300602</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>飞荣达</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>电磁屏蔽和热管理材料及器件，覆盖导热石墨膜、散热模组、VC、热管和液冷板。</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="36" customHeight="1">
-      <c r="A69" s="4" t="inlineStr">
+    <row r="71" ht="36" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>散热材料</t>
         </is>
       </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>301489</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>思泉新材</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>热管理材料、散热组件和液冷散热产线，AI服务器、光模块等新场景拓展中，弹性强但兑现需跟踪。</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="36" customHeight="1">
-      <c r="A70" s="4" t="inlineStr">
+    <row r="72" ht="36" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>光模块散热 / 结构件</t>
         </is>
       </c>
-      <c r="B70" s="5" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>300684</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>中石科技</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>偏热管理材料和散热模组，覆盖光模块、服务器和通信设备散热。</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="36" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="73" ht="36" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>光模块散热 / 结构件</t>
         </is>
       </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>301128</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>强瑞技术</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>披露有光模块散热器相关收入，偏结构件和散热部件加工。</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="36" customHeight="1">
-      <c r="A72" s="4" t="inlineStr">
+    <row r="74" ht="36" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>光模块散热 / 结构件</t>
         </is>
       </c>
-      <c r="B72" s="5" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>301489</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>思泉新材</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>偏AI服务器和通信设备热管理材料，弹性较强但兑现仍需跟踪。</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="36" customHeight="1">
-      <c r="A73" s="4" t="inlineStr">
+    <row r="75" ht="36" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>沉铜 / 电镀 / 表面处理药水</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>688603</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>天承科技</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>PCB专用湿电子化学品主线，覆盖沉铜、电镀和表面处理药水。</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="36" customHeight="1">
-      <c r="A74" s="4" t="inlineStr">
+    <row r="76" ht="36" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>沉铜 / 电镀 / 表面处理药水</t>
         </is>
       </c>
-      <c r="B74" s="5" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>002741</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>光华科技</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>覆盖PCB化学品、沉铜、电镀和表面处理，平台更宽但纯度低于天承科技。</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="36" customHeight="1">
-      <c r="A75" s="4" t="inlineStr">
+    <row r="77" ht="36" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
         </is>
       </c>
-      <c r="B75" s="5" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>300576</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>容大感光</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>PCB湿膜、阻焊油墨、干膜相关，是PCB光刻胶/油墨主线。</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="36" customHeight="1">
-      <c r="A76" s="4" t="inlineStr">
+    <row r="78" ht="36" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
         </is>
       </c>
-      <c r="B76" s="5" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>300537</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>广信材料</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>PCB光刻胶占比较高，受益于PCB图形材料国产替代。</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="36" customHeight="1">
-      <c r="A77" s="4" t="inlineStr">
+    <row r="79" ht="16.5" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
         </is>
       </c>
-      <c r="B77" s="5" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>300429</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>强力新材</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>涉及PCB干膜光刻胶材料，相关度低于容大和广信。</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
+    <row r="80" ht="16.5" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>光纤连接 / 线缆配套</t>
         </is>
       </c>
-      <c r="B78" s="5" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>300570</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>太辰光</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>高密度光连接器、MPO/MTP等配套受益于CPO和硅光连接密度提升。</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+    <row r="81" ht="16.5" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>光纤连接 / 线缆配套</t>
         </is>
       </c>
-      <c r="B79" s="5" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>002281</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>光迅科技</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
         <is>
           <t>覆盖无源光器件、光纤阵列和模块平台，配套能力较完整。</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+    <row r="82" ht="16.5" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>光纤连接 / 线缆配套</t>
         </is>
       </c>
-      <c r="B80" s="5" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>300620</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>光库科技</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>保偏连接、光纤器件和铌酸锂相关器件具备协同。</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
+    <row r="83" ht="16.5" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>光纤</t>
         </is>
       </c>
-      <c r="B81" s="5" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>601869</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>长飞光纤</t>
         </is>
       </c>
-      <c r="D81" s="4" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>光纤预制棒、光纤、光缆一体化龙头，光纤板块直接度最高。</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="4" t="inlineStr">
+    <row r="84" ht="16.5" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>光纤</t>
         </is>
       </c>
-      <c r="B82" s="5" t="inlineStr">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>600487</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>亨通光电</t>
         </is>
       </c>
-      <c r="D82" s="4" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>光棒、光纤、光缆、光器件和光通信网络方案平台型龙头。</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr">
+    <row r="85" ht="16.5" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>光纤</t>
         </is>
       </c>
-      <c r="B83" s="5" t="inlineStr">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>600522</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>中天科技</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>光纤光缆、特种光缆和通信网络平台型公司，兼具空芯光纤等新方向弹性。</t>
         </is>
       </c>
     </row>
+    <row r="86" ht="16.5" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>HBM / 高端DRAM</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>688008</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>澜起科技</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>DDR5内存接口芯片、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器高端内存互连核心受益。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="16.5" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>HBM / 高端DRAM</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>300475</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>香农芯创</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>SK海力士高端存储代理及企业级存储业务，受益DDR5/HBM紧缺和云服务客户备货，偏分销弹性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="16.5" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>数据中心电力 / 变压器</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>688676</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>金盘科技</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>数据中心干式变压器和AIDC供电设备方向明确，受益AI数据中心电力设备交付紧张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="16.5" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>数据中心电力 / 变压器</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>002028</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>思源电气</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>变压器、GIS、开关设备和输配电控制平台，受益数据中心并网和全球电力设备紧缺。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="16.5" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>数据中心电力 / 变压器</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>600089</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>特变电工</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>大型变压器、特高压装备和线缆平台，受益电网投资与AI数据中心电力基础设施扩容。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="16.5" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>数据中心电力 / 变压器</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>601179</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>中国西电</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>高压开关、变压器、输配电成套装备平台，受益电网主设备和数据中心并网需求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="16.5" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>先进封装 / CoWoS替代</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>600584</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>长电科技</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>先进封装平台龙头，布局2.5D/3D、Chiplet等，受益国产AI芯片封测升级；不等同台积电CoWoS。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="16.5" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>先进封装 / CoWoS替代</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>002156</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>通富微电</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>绑定高性能计算封测客户，FCBGA、Chiplet、2D+等先进封装扩产，受益AI/HPC封测需求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="16.5" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>FC-BGA / ABF载板</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>002436</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>兴森科技</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>FC-BGA/IC载板国产化主线，客户认证和良率爬坡推进，受益ABF/BT载板紧缺。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="16.5" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD / NAND</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>688525</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>佰维存储</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD、服务器内存和先进封测布局，受益AI服务器带动企业级存储放量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="16.5" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD / NAND</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>301308</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>江波龙</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD和数据中心存储方案，受益AI训练/推理带动高容量SSD需求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD / NAND</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>001309</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>德明利</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>存储模组和SSD控制器/模组链，受益NAND涨价与企业级存储需求，弹性偏周期。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D74"/>
+  <autoFilter ref="A1:D97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: backup latest project state
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -9,7 +9,7 @@
     <sheet name="AI产业链" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI产业链'!$A$1:$D$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI产业链'!$A$1:$D$99</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1082,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2722,88 +2722,88 @@
     <row r="75" ht="36" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>沉铜 / 电镀 / 表面处理药水</t>
+          <t>光模块液冷 / CAGE</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>688603</t>
+          <t>688668</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>天承科技</t>
+          <t>鼎通科技</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>PCB专用湿电子化学品主线，覆盖沉铜、电镀和表面处理药水。</t>
+          <t>液冷CAGE/224G OSFP CAGE方向，募投新增液冷CAGE产能，产品面向高密度数据中心、AI服务器和算力中心，弹性看客户验证和批量交付。</t>
         </is>
       </c>
     </row>
     <row r="76" ht="36" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>沉铜 / 电镀 / 表面处理药水</t>
+          <t>光模块液冷 / CAGE</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>002741</t>
+          <t>301123</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>光华科技</t>
+          <t>奕东电子</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>覆盖PCB化学品、沉铜、电镀和表面处理，平台更宽但纯度低于天承科技。</t>
+          <t>具备光模块CAGE制造经验，液冷板组件已批量出货，推进“连接器+散热”协同的液冷CAGE/光模块液冷方案，弹性看客户导入和液冷模组放量。</t>
         </is>
       </c>
     </row>
     <row r="77" ht="36" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
+          <t>沉铜 / 电镀 / 表面处理药水</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>300576</t>
+          <t>688603</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>容大感光</t>
+          <t>天承科技</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>PCB湿膜、阻焊油墨、干膜相关，是PCB光刻胶/油墨主线。</t>
+          <t>PCB专用湿电子化学品主线，覆盖沉铜、电镀和表面处理药水。</t>
         </is>
       </c>
     </row>
     <row r="78" ht="36" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
+          <t>沉铜 / 电镀 / 表面处理药水</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>300537</t>
+          <t>002741</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>广信材料</t>
+          <t>光华科技</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>PCB光刻胶占比较高，受益于PCB图形材料国产替代。</t>
+          <t>覆盖PCB化学品、沉铜、电镀和表面处理，平台更宽但纯度低于天承科技。</t>
         </is>
       </c>
     </row>
@@ -2815,61 +2815,61 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>300429</t>
+          <t>300576</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>强力新材</t>
+          <t>容大感光</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>涉及PCB干膜光刻胶材料，相关度低于容大和广信。</t>
+          <t>PCB湿膜、阻焊油墨、干膜相关，是PCB光刻胶/油墨主线。</t>
         </is>
       </c>
     </row>
     <row r="80" ht="16.5" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>光纤连接 / 线缆配套</t>
+          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>300570</t>
+          <t>300537</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>太辰光</t>
+          <t>广信材料</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>高密度光连接器、MPO/MTP等配套受益于CPO和硅光连接密度提升。</t>
+          <t>PCB光刻胶占比较高，受益于PCB图形材料国产替代。</t>
         </is>
       </c>
     </row>
     <row r="81" ht="16.5" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>光纤连接 / 线缆配套</t>
+          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>002281</t>
+          <t>300429</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>光迅科技</t>
+          <t>强力新材</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>覆盖无源光器件、光纤阵列和模块平台，配套能力较完整。</t>
+          <t>涉及PCB干膜光刻胶材料，相关度低于容大和广信。</t>
         </is>
       </c>
     </row>
@@ -2881,61 +2881,61 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>300620</t>
+          <t>300570</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>光库科技</t>
+          <t>太辰光</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>保偏连接、光纤器件和铌酸锂相关器件具备协同。</t>
+          <t>高密度光连接器、MPO/MTP等配套受益于CPO和硅光连接密度提升。</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16.5" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>光纤</t>
+          <t>光纤连接 / 线缆配套</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>601869</t>
+          <t>002281</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>长飞光纤</t>
+          <t>光迅科技</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>光纤预制棒、光纤、光缆一体化龙头，光纤板块直接度最高。</t>
+          <t>覆盖无源光器件、光纤阵列和模块平台，配套能力较完整。</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16.5" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>光纤</t>
+          <t>光纤连接 / 线缆配套</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>600487</t>
+          <t>300620</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>亨通光电</t>
+          <t>光库科技</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>光棒、光纤、光缆、光器件和光通信网络方案平台型龙头。</t>
+          <t>保偏连接、光纤器件和铌酸锂相关器件具备协同。</t>
         </is>
       </c>
     </row>
@@ -2947,105 +2947,105 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>600522</t>
+          <t>601869</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>中天科技</t>
+          <t>长飞光纤</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>光纤光缆、特种光缆和通信网络平台型公司，兼具空芯光纤等新方向弹性。</t>
+          <t>光纤预制棒、光纤、光缆一体化龙头，光纤板块直接度最高。</t>
         </is>
       </c>
     </row>
     <row r="86" ht="16.5" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>HBM / 高端DRAM</t>
+          <t>光纤</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>688008</t>
+          <t>600487</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>澜起科技</t>
+          <t>亨通光电</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>DDR5内存接口芯片、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器高端内存互连核心受益。</t>
+          <t>光棒、光纤、光缆、光器件和光通信网络方案平台型龙头。</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16.5" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>HBM / 高端DRAM</t>
+          <t>光纤</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>300475</t>
+          <t>600522</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>香农芯创</t>
+          <t>中天科技</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>SK海力士高端存储代理及企业级存储业务，受益DDR5/HBM紧缺和云服务客户备货，偏分销弹性。</t>
+          <t>光纤光缆、特种光缆和通信网络平台型公司，兼具空芯光纤等新方向弹性。</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16.5" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>数据中心电力 / 变压器</t>
+          <t>HBM / 高端DRAM</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>688676</t>
+          <t>688008</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>金盘科技</t>
+          <t>澜起科技</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>数据中心干式变压器和AIDC供电设备方向明确，受益AI数据中心电力设备交付紧张。</t>
+          <t>DDR5内存接口芯片、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器高端内存互连核心受益。</t>
         </is>
       </c>
     </row>
     <row r="89" ht="16.5" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>数据中心电力 / 变压器</t>
+          <t>HBM / 高端DRAM</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>002028</t>
+          <t>300475</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>香农芯创</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>变压器、GIS、开关设备和输配电控制平台，受益数据中心并网和全球电力设备紧缺。</t>
+          <t>SK海力士高端存储代理及企业级存储业务，受益DDR5/HBM紧缺和云服务客户备货，偏分销弹性。</t>
         </is>
       </c>
     </row>
@@ -3057,17 +3057,17 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>600089</t>
+          <t>688676</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>特变电工</t>
+          <t>金盘科技</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>大型变压器、特高压装备和线缆平台，受益电网投资与AI数据中心电力基础设施扩容。</t>
+          <t>数据中心干式变压器和AIDC供电设备方向明确，受益AI数据中心电力设备交付紧张。</t>
         </is>
       </c>
     </row>
@@ -3079,127 +3079,127 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>601179</t>
+          <t>002028</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>中国西电</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>高压开关、变压器、输配电成套装备平台，受益电网主设备和数据中心并网需求。</t>
+          <t>变压器、GIS、开关设备和输配电控制平台，受益数据中心并网和全球电力设备紧缺。</t>
         </is>
       </c>
     </row>
     <row r="92" ht="16.5" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>数据中心电力 / 变压器</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>600584</t>
+          <t>600089</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>长电科技</t>
+          <t>特变电工</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>先进封装平台龙头，布局2.5D/3D、Chiplet等，受益国产AI芯片封测升级；不等同台积电CoWoS。</t>
+          <t>大型变压器、特高压装备和线缆平台，受益电网投资与AI数据中心电力基础设施扩容。</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16.5" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>数据中心电力 / 变压器</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>002156</t>
+          <t>601179</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>通富微电</t>
+          <t>中国西电</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>绑定高性能计算封测客户，FCBGA、Chiplet、2D+等先进封装扩产，受益AI/HPC封测需求。</t>
+          <t>高压开关、变压器、输配电成套装备平台，受益电网主设备和数据中心并网需求。</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16.5" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA / ABF载板</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>002436</t>
+          <t>600584</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>兴森科技</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA/IC载板国产化主线，客户认证和良率爬坡推进，受益ABF/BT载板紧缺。</t>
+          <t>先进封装平台龙头，布局2.5D/3D、Chiplet等，受益国产AI芯片封测升级；不等同台积电CoWoS。</t>
         </is>
       </c>
     </row>
     <row r="95" ht="16.5" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD / NAND</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>688525</t>
+          <t>002156</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>佰维存储</t>
+          <t>通富微电</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD、服务器内存和先进封测布局，受益AI服务器带动企业级存储放量。</t>
+          <t>绑定高性能计算封测客户，FCBGA、Chiplet、2D+等先进封装扩产，受益AI/HPC封测需求。</t>
         </is>
       </c>
     </row>
     <row r="96" ht="16.5" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD / NAND</t>
+          <t>FC-BGA / ABF载板</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>301308</t>
+          <t>002436</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>江波龙</t>
+          <t>兴森科技</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD和数据中心存储方案，受益AI训练/推理带动高容量SSD需求。</t>
+          <t>FC-BGA/IC载板国产化主线，客户认证和良率爬坡推进，受益ABF/BT载板紧缺。</t>
         </is>
       </c>
     </row>
@@ -3211,22 +3211,66 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
+          <t>688525</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>佰维存储</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD、服务器内存和先进封测布局，受益AI服务器带动企业级存储放量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD / NAND</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>301308</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>江波龙</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD和数据中心存储方案，受益AI训练/推理带动高容量SSD需求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>企业级SSD / NAND</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
           <t>001309</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>德明利</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>存储模组和SSD控制器/模组链，受益NAND涨价与企业级存储需求，弹性偏周期。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D97"/>
+  <autoFilter ref="A1:D99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update AI industry chain workbook
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1082,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D183"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3269,6 +3269,1854 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>国产AI芯片 / 加速卡</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>688256</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>寒武纪</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>云端智能芯片和板卡最直接的A股国产AI算力芯片映射，核心看大客户、订单持续性、生态适配和估值消化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>国产AI芯片 / 加速卡</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>688041</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>CPU+DCU国产高端处理器平台，绑定国产服务器生态，算力国产化确定性强，弹性看DCU放量和软件栈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>国产AI芯片 / 加速卡</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>300474</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>景嘉微</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>GPU+边端侧AI SoC路线，技术弹性强但仍需看通用算力产品商业化、亏损收窄和客户导入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>AI服务器 / ODM / 机架整机</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>601138</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>工业富联</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>A股AI服务器和机架系统ODM最直接映射之一，覆盖云服务商AI服务器、高速网络和系统级整合。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>AI服务器 / ODM / 机架整机</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>000977</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>浪潮信息</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>国内AI服务器和IT基础设施龙头，服务器收入占比高，核心看AI服务器订单、毛利率和现金流质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>AI服务器 / ODM / 机架整机</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>603019</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>中科曙光</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>高端计算机、服务器、存储、液冷和算力服务平台，国产算力基础设施核心公司之一。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>AI服务器 / ODM / 机架整机</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>000938</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>紫光股份</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>新华三体系覆盖AI服务器、数据中心交换机、存储和液冷方案，兼具整机与网络平台属性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>AI网络设备 / 数据中心交换机</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>000938</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>紫光股份</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>新华三数据中心交换机份额靠前，800G智算交换机和无损网络方案是AI集群网络核心映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>AI网络设备 / 数据中心交换机</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>301165</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>锐捷网络</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>数据中心交换机产品受互联网和AI数据中心建设带动，订单交付和毛利率变化需持续跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>AI网络设备 / 数据中心交换机</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>000063</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>中兴通讯</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>连接+算力平台，覆盖AI服务器、存储、数据中心交换机和智算超节点，兼具设备与自研芯片线索。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>以太网交换芯片 / PHY</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>688702</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>盛科通信-U</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>国产以太网交换芯片最直接A股映射，具备高性能端口和Tbps级架构储备，数据中心高端放量仍需验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>以太网交换芯片 / PHY</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>688515</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>裕太微</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>以太网PHY和交换芯片国产化标的，下一代向数据中心等高价值场景延伸，当前更偏观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>CXL / PCIe Retimer / 内存互连</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>688008</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>澜起科技</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>DDR5接口、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器内存互连核心国产映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>CXL / PCIe Retimer / 内存互连</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>暂无成熟A股纯标的</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>高速铜互连 / DAC-AEC / Twinax</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>300913</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>兆龙互连</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>数据中心和AI算力中心高速布线、铜缆组件和连接产品映射，弹性看高速率产品客户导入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>高速铜互连 / DAC-AEC / Twinax</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>300563</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>神宇股份</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>已开发PCIe5.0/6.0/7.0及DAC 56G/112G/224G等高速数据线，属于铜互连高弹性观察标的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>高速铜互连 / DAC-AEC / Twinax</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>002130</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>沃尔核材</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>高速通信线缆和224G/800G/1.6T方向已有表内覆盖，建议在铜互连子环节中单列跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>GPU供电电感 / 磁性材料</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>300811</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>铂科新材</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>芯片电感和金属软磁材料切入AI服务器GPU供电，属于48V/板级供电上游高弹性补充。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>GPU供电电感 / 磁性材料</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>002138</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>顺络电子</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>功率电感、变压器等AI服务器供电上游元件已有表内覆盖，建议和铂科共同跟踪板级供电升级。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>MLCC / 高端被动元件</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>300408</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>三环集团</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>MLCC与陶瓷材料平台，年报提到突破超高容大尺寸产品并加深服务器等客户合作，是Rubin MLCC增量映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>MLCC / 高端被动元件</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>000636</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>风华高科</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>MLCC、电阻、电感等被动元件覆盖AI算力等应用，弹性看高端规格、客户认证和盈利修复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>MLCC / 高端被动元件</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>002138</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>顺络电子</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>功率电感和片式被动元件平台，适合作为AI服务器高可靠被动件和供电元件交叉跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>先进封装材料 / 底填 / EMC</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>688535</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>华海诚科</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>环氧塑封料和电子胶黏剂平台，先进封装材料国产化映射，核心看高端封装客户与收入占比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>先进封装材料 / 底填 / EMC</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>688035</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>德邦科技</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>底部填充胶、固晶、导热、晶圆UV膜等封装材料布局，适配Flip-chip、WLP、SiP、2.5D/3D封装。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>先进封装材料 / 底填 / EMC</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>688300</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>联瑞新材</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>球硅/低Df填料已有表内覆盖，也应归入先进封装和高端塑封材料填料链条交叉跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>300604</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>长川科技</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>半导体测试设备平台，HBM和先进封装拉动测试设备需求，核心看存储/SoC测试订单。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>688200</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>华峰测控</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>模拟、功率、SoC等测试系统平台，受AI芯片国产化和高端SoC测试需求拉动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>688627</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>精智达</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>存储器后道测试、老化、探针卡和HBM/KGSD测试技术推进，是HBM测试国产映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>688661</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>和林微纳</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>测试探针/探针卡耗材方向，属于半导体测试链条精密耗材补充，弹性看高端探针卡导入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>800VDC / HVDC / 机柜供电</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>002851</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>麦格米特</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>AI服务器电源已有表内覆盖，建议在800VDC/HVDC机柜供电子环节中单列观察客户导入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>800VDC / HVDC / 机柜供电</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>002922</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>伊戈尔</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>数据中心移相、油浸、干式变压器和800V直流供电系统布局明确，是机柜供电升级补充标的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>800VDC / HVDC / 机柜供电</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>002335</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>科华数据</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>UPS、HVDC、液冷微模块和预制式电力模组覆盖智算中心供电系统，项目兑现度较高。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>UPS / PDU / 低压配电 / Switchgear</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>002518</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>科士达</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>UPS和数据中心关键基础设施公司，智慧电源和数据中心产品收入占比较高，海外UPS/HVDC需跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>UPS / PDU / 低压配电 / Switchgear</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>002335</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>科华数据</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>数据中心UPS、配电、液冷和微模块综合方案，适合放在电力基础设施核心补缺块。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>UPS / PDU / 低压配电 / Switchgear</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>002706</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>良信股份</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>低压电器和智能配电产品用于智算中心等场景，属于数据中心低压配电与保护器件映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>OCS / 光交换 / 精密光学</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>688195</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>腾景科技</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>精密光学元组件、光纤器件和光测试仪器平台，OCS/CPO相关精密光学为观察方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>OCS / 光交换 / 精密光学</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>300620</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>光库科技</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>保偏光纤器件、铌酸锂和光通信器件平台，可作为OCS/硅光/相干链条交叉观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>OCS / 光交换 / 精密光学</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>300394</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>天孚通信</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>FAU、POSA、光引擎和高精度无源器件已在表内覆盖，也应纳入OCS/CPO精密光学迁移池。</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>601869</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>长飞光纤</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>空芯、多芯、G.654.E和数据中心光联接官方口径增强，但订单和规模收入仍需后续验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>600487</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>亨通光电</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>光纤光缆和特种光纤平台型公司，建议从普通光纤中拆出新型光纤观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>600522</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>中天科技</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>光纤光缆和特种光缆平台，空芯/新型光纤属于中长期技术与交易弹性观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>PCB / HLC / HDI补充</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>688183</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>生益电子</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>高端PCB和智能算力互联核心组件研发投入明确，是AI服务器/高性能计算PCB补充核心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>PCB / HLC / HDI补充</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>002938</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>鹏鼎控股</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>全球PCB龙头，AI云-管-端和AI服务器/光模块PCB布局加速，但A股主体与具体AI收入需继续拆分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>晶圆代工 / 国产先进制程</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>688981</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>中芯国际</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>国产AI芯片制造底座，先进制程与成熟制程并行；受设备、EDA、IP与外部限制约束，不能直接等同先进GPU代工能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>晶圆代工 / 国产先进制程</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>688347</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>华虹公司</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>特色工艺、功率、模拟与嵌入式平台，更多是AI服务器电源、边缘芯片和国产半导体底座映射，先进算力芯片弹性弱于中芯。</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>前道设备 / 国产AI芯片制造</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>002371</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>北方华创</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>刻蚀、薄膜沉积、热处理、清洗等平台型设备龙头，国产晶圆制造CAPEX核心映射；AI链属于制造底座，不是直接下游订单。</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>前道设备 / 国产AI芯片制造</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>688012</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>中微公司</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>刻蚀设备和MOCVD核心平台，先进制程国产设备主线，受益国产AI芯片制造和先进封装扩产。</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>前道设备 / 国产AI芯片制造</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>688072</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>拓荆科技</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>薄膜沉积设备平台，同时向混合键合相关检测/量测延伸，HBM/Chiplet先进封装为中长期弹性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>EDA / IP / ASIC设计服务</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>688521</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>芯原股份</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>半导体IP和芯片定制服务平台，GPU/NPU/视频/接口IP与Chiplet方向相关，适合跟踪国产AI ASIC设计服务景气度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>EDA / IP / ASIC设计服务</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>301269</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>华大九天</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>国产EDA平台核心标的，受益国产芯片设计和制造国产化；AI链映射偏工具层，业绩弹性看授权和客户扩张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>EDA / IP / ASIC设计服务</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>688206</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>概伦电子</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>器件建模、EDA和半导体良率/测试数据分析工具，偏国产EDA补链，交易弹性需看订单兑现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>FC-BGA / ABF载板</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>002916</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>深南电路</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>IC载板与FC-BGA能力建设，兼具PCB与封装基板平台，AI/HPC长期受益但需继续看良率、客户认证和收入占比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>FC-BGA / ABF载板</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>002938</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>鹏鼎控股</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>全球PCB龙头，AI server PCB与IC substrate有体系映射；A股主体与具体AI收入仍需拆分验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>先进封装 / CoWoS替代</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>688362</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>甬矽电子</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>先进封装和系统级封装平台，适合作为AI/HPC封测国产化补充观察，确定性低于长电、通富。</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>先进封装 / CoWoS替代</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>002185</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>华天科技</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>封测平台型公司，具备先进封装布局，更多是国产封测底座映射，AI/HBM收入纯度需跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>688120</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>华海清科</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>CMP、减薄和清洗设备平台，官方年报提到2.5D/RDL把芯片与HBM集成对CMP提出更高要求，是HBM/Chiplet设备映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>688082</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>盛美上海</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>清洗、电镀和面板级先进封装电镀设备，适配RDL/TSV/先进封装湿法制程，核心看封装客户订单放量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>688037</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>芯源微</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>后道先进封装涂胶显影、单片湿法、临时键合/解键合设备，适配超薄晶圆和HBM/Chiplet封装制程。</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>688072</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>拓荆科技</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>混合键合、键合套准量测和键合强度检测等先进封装线索明确，适合作为HBM/3D封装设备观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>300054</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>鼎龙股份</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>CMP抛光垫/抛光液/清洗液、半导体封装PI、PSPI和临时键合胶布局，卡位WLP/2.5D/3D封装材料。</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>688019</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>安集科技</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>CMP抛光液和功能性湿电子化学品平台，先进制程与先进封装共同受益，核心看高端客户份额和新品放量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>300236</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>上海新阳</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>半导体电镀、清洗、Bumping/TSV相关材料，适配先进封装和晶圆级封装工艺。</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>688268</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>华特气体</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>高端特种气体明确提及HBM/TSV刻蚀等应用，属于存储和先进制程耗材映射，弹性看客户认证和放量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>玻璃基板 / TGV / 玻璃中介层</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>603773</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>沃格光电</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>年报把玻璃基板级封装线路载板和TGV用于AI大算力芯片、先进封装、高速传输等方向；当前仍按中长期观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>玻璃基板 / TGV / 玻璃中介层</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>300776</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>帝尔激光</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>年报提到TGV、PCB超快激光加工设备和先进封装装备，属于玻璃基板/高端PCB设备观察。</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>300547</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>川环科技</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>公告披露获得服务器整体解决方案商液冷管路系统项目定点，后续看客户量产、单柜价值量和毛利。</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>300731</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>科创新源</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>通过创源智热布局数据中心散热结构件、液冷板和散热模组，处于客户开拓/认证阶段，弹性强但兑现早期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>002536</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>飞龙股份</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>电子泵、温控阀等液冷热管理部件进入服务器液冷/IDC液冷/AI等场景，项目多但收入纯度需跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>300602</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>飞荣达</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>服务器/数据中心液冷散热、冷板、热管/VC和热管理材料平台，已在散热材料中覆盖，可在液冷部件维度单列。</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>688226</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>威腾电气</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>数据中心相关母线及配电设备受益算力用电提升，年报提到数据中心机柜用智能型直流/交流母线槽。</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>002706</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>良信股份</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>低压配电、智能断路器、智能盘柜面向数据中心等关键配电场景，适合与UPS/PDU/Switchgear共同跟踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>301031</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>中熔电气</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>熔断器和电路保护器件适配高压直流、储能和电力电子，AI机柜配电属于观察映射，需验证数据中心收入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>600745</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>闻泰科技</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>安世半导体分立与功率器件平台，年报提到二极管、MOSFET、保护器件、电源管理IC、GaN FET、SiC MOS在数据中心降耗等领域应用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>605111</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>新洁能</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>SGT/SJ MOSFET、GateDriver、DrMOS等用于服务器电源、CPU/GPU板级供电、PFC/LLC等，AI服务器供电升级弹性明确。</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>688261</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>东微半导</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>高压超级结MOSFET、SiC等功率器件平台，适配高效电源和HVDC方向，但AI数据中心客户需持续验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>600460</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>士兰微</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>功率器件和功率模块平台，偏泛半导体受益，AI服务器电源纯度弱于新洁能/闻泰，需要观察导入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>高端电容 / 固态叠层 / 超级电容</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>002484</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>江海股份</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>MLPC固态叠层高分子电容、超级电容和铝电解平台，IR提到AI服务器研发阶段性成果；核心看批量订单。</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>高端电容 / 固态叠层 / 超级电容</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>603989</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>艾华集团</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>铝电解电容器平台，半年报提及把握AI服务器、数据中心等结构性机遇，适合作为电源电容补充。</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>高端电容 / 固态叠层 / 超级电容</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>600563</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>法拉电子</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>薄膜电容器龙头，覆盖电力电子、储能、智能电网等高压场景，AI数据中心HVDC/电源链为中长期映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>300442</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>润泽科技</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>润泽智算年报披露AIDC/AI算力中心运维、能效和算力服务能力，是下游算力基础设施运营商核心映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>300738</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>奥飞数据</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>半年度报告显示推进大型数据中心/智算中心项目建设交付，受益AI算力需求，需跟踪上架率和客户质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>300383</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>光环新网</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>IDC和云计算平台，半年度报告提到AI驱动下数据中心硬件架构和运维变革；利润波动和项目回款需注意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>600845</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>宝信软件</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>工业智算云和智算中心/云计算节点布局，偏企业级和工业场景算力基础设施映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>HCA / DPU / SmartNIC / RoCE</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>暂无成熟A股纯标的</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>该环节主要由NVIDIA/Mellanox、Broadcom、Marvell、Intel等主导；A股网络设备公司不等同HCA/DPU芯片。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: backup ai chain tracking artifacts
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1082,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:D191"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2436,22 +2436,22 @@
     <row r="62" ht="36" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>PCB钻针 / 微钻 / 刀具</t>
+          <t>PCB电镀设备 / mSAP / IC载板湿制程</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>301377</t>
+          <t>688700</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>鼎泰高科</t>
+          <t>东威科技</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>PCB钻针主线，受益于高多层、硬材料和细孔径升级。</t>
+          <t>PCB垂直连续电镀设备、水平三合一电镀设备和升降式移载VCP覆盖服务器/云存储、高阶HDI、IC载板、BT/ABF载板等，高多层AI PCB与载板扩产带动电镀设备升级。</t>
         </is>
       </c>
     </row>
@@ -2463,39 +2463,39 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>000657</t>
+          <t>301377</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>中钨高新</t>
+          <t>鼎泰高科</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>通过金洲公司具备PCB微型刀具产能，偏刀具耗材。</t>
+          <t>PCB钻针主线，受益于高多层、硬材料和细孔径升级。</t>
         </is>
       </c>
     </row>
     <row r="64" ht="36" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>高多层PCB加工设备耗材</t>
+          <t>PCB钻针 / 微钻 / 刀具</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>301200</t>
+          <t>000657</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>大族数控</t>
+          <t>中钨高新</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>高多层AIPCB带动钻孔、曝光、成型、检测等设备升级。</t>
+          <t>通过金洲公司具备PCB微型刀具产能，偏刀具耗材。</t>
         </is>
       </c>
     </row>
@@ -2507,17 +2507,17 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>301377</t>
+          <t>301200</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>鼎泰高科</t>
+          <t>大族数控</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>高多层、硬材料、细孔径带动PCB钻针和微钻耗材需求。</t>
+          <t>高多层AIPCB带动钻孔、曝光、成型、检测等设备升级。</t>
         </is>
       </c>
     </row>
@@ -2529,39 +2529,39 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>000657</t>
+          <t>301377</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>中钨高新</t>
+          <t>鼎泰高科</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>通过PCB微型刀具产能参与耗材升级，受益于细孔径加工。</t>
+          <t>高多层、硬材料、细孔径带动PCB钻针和微钻耗材需求。</t>
         </is>
       </c>
     </row>
     <row r="67" ht="36" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>TFLN / 薄膜铌酸锂</t>
+          <t>高多层PCB加工设备耗材</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>300620</t>
+          <t>000657</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>光库科技</t>
+          <t>中钨高新</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>偏薄膜铌酸锂调制器与光子集成，是TFLN器件方向核心映射。</t>
+          <t>通过PCB微型刀具产能参与耗材升级，受益于细孔径加工。</t>
         </is>
       </c>
     </row>
@@ -2573,39 +2573,39 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>600330</t>
+          <t>300620</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>天通股份</t>
+          <t>光库科技</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>偏铌酸锂晶体、晶片和材料端，位置更上游。</t>
+          <t>偏薄膜铌酸锂调制器与光子集成，是TFLN器件方向核心映射。</t>
         </is>
       </c>
     </row>
     <row r="69" ht="36" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>散热材料</t>
+          <t>TFLN / 薄膜铌酸锂</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>300684</t>
+          <t>600330</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>中石科技</t>
+          <t>天通股份</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>导热界面材料、石墨散热、VC和热管理组件，服务器/数据中心和北美大客户线索明确。</t>
+          <t>偏铌酸锂晶体、晶片和材料端，位置更上游。</t>
         </is>
       </c>
     </row>
@@ -2617,17 +2617,17 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>300602</t>
+          <t>300684</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>飞荣达</t>
+          <t>中石科技</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>电磁屏蔽和热管理材料及器件，覆盖导热石墨膜、散热模组、VC、热管和液冷板。</t>
+          <t>导热界面材料、石墨散热、VC和热管理组件，服务器/数据中心和北美大客户线索明确。</t>
         </is>
       </c>
     </row>
@@ -2639,39 +2639,39 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>301489</t>
+          <t>300602</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>思泉新材</t>
+          <t>飞荣达</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>热管理材料、散热组件和液冷散热产线，AI服务器、光模块等新场景拓展中，弹性强但兑现需跟踪。</t>
+          <t>电磁屏蔽和热管理材料及器件，覆盖导热石墨膜、散热模组、VC、热管和液冷板。</t>
         </is>
       </c>
     </row>
     <row r="72" ht="36" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>光模块散热 / 结构件</t>
+          <t>散热材料</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>300684</t>
+          <t>301489</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>中石科技</t>
+          <t>思泉新材</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>偏热管理材料和散热模组，覆盖光模块、服务器和通信设备散热。</t>
+          <t>热管理材料、散热组件和液冷散热产线，AI服务器、光模块等新场景拓展中，弹性强但兑现需跟踪。</t>
         </is>
       </c>
     </row>
@@ -2683,17 +2683,17 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>301128</t>
+          <t>300684</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>强瑞技术</t>
+          <t>中石科技</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>披露有光模块散热器相关收入，偏结构件和散热部件加工。</t>
+          <t>偏热管理材料和散热模组，覆盖光模块、服务器和通信设备散热。</t>
         </is>
       </c>
     </row>
@@ -2705,39 +2705,39 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>301489</t>
+          <t>301128</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>思泉新材</t>
+          <t>强瑞技术</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>偏AI服务器和通信设备热管理材料，弹性较强但兑现仍需跟踪。</t>
+          <t>披露有光模块散热器相关收入，偏结构件和散热部件加工。</t>
         </is>
       </c>
     </row>
     <row r="75" ht="36" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>光模块液冷 / CAGE</t>
+          <t>光模块散热 / 结构件</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>688668</t>
+          <t>301489</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>鼎通科技</t>
+          <t>思泉新材</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>液冷CAGE/224G OSFP CAGE方向，募投新增液冷CAGE产能，产品面向高密度数据中心、AI服务器和算力中心，弹性看客户验证和批量交付。</t>
+          <t>偏AI服务器和通信设备热管理材料，弹性较强但兑现仍需跟踪。</t>
         </is>
       </c>
     </row>
@@ -2749,39 +2749,39 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>301123</t>
+          <t>688668</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>奕东电子</t>
+          <t>鼎通科技</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>具备光模块CAGE制造经验，液冷板组件已批量出货，推进“连接器+散热”协同的液冷CAGE/光模块液冷方案，弹性看客户导入和液冷模组放量。</t>
+          <t>液冷CAGE/224G OSFP CAGE方向，募投新增液冷CAGE产能，产品面向高密度数据中心、AI服务器和算力中心，弹性看客户验证和批量交付。</t>
         </is>
       </c>
     </row>
     <row r="77" ht="36" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>沉铜 / 电镀 / 表面处理药水</t>
+          <t>光模块液冷 / CAGE</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>688603</t>
+          <t>301123</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>天承科技</t>
+          <t>奕东电子</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>PCB专用湿电子化学品主线，覆盖沉铜、电镀和表面处理药水。</t>
+          <t>具备光模块CAGE制造经验，液冷板组件已批量出货，推进“连接器+散热”协同的液冷CAGE/光模块液冷方案，弹性看客户导入和液冷模组放量。</t>
         </is>
       </c>
     </row>
@@ -2793,39 +2793,39 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>002741</t>
+          <t>688603</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>光华科技</t>
+          <t>天承科技</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>覆盖PCB化学品、沉铜、电镀和表面处理，平台更宽但纯度低于天承科技。</t>
+          <t>PCB专用湿电子化学品主线，覆盖沉铜、电镀和表面处理药水。</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16.5" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
+          <t>沉铜 / 电镀 / 表面处理药水</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>300576</t>
+          <t>002741</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>容大感光</t>
+          <t>光华科技</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>PCB湿膜、阻焊油墨、干膜相关，是PCB光刻胶/油墨主线。</t>
+          <t>覆盖PCB化学品、沉铜、电镀和表面处理，平台更宽但纯度低于天承科技。</t>
         </is>
       </c>
     </row>
@@ -2837,17 +2837,17 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>300537</t>
+          <t>300576</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>广信材料</t>
+          <t>容大感光</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>PCB光刻胶占比较高，受益于PCB图形材料国产替代。</t>
+          <t>PCB湿膜、阻焊油墨、干膜相关，是PCB光刻胶/油墨主线。</t>
         </is>
       </c>
     </row>
@@ -2859,39 +2859,39 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>300429</t>
+          <t>300537</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>强力新材</t>
+          <t>广信材料</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>涉及PCB干膜光刻胶材料，相关度低于容大和广信。</t>
+          <t>PCB光刻胶占比较高，受益于PCB图形材料国产替代。</t>
         </is>
       </c>
     </row>
     <row r="82" ht="16.5" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>光纤连接 / 线缆配套</t>
+          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>300570</t>
+          <t>300429</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>太辰光</t>
+          <t>强力新材</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>高密度光连接器、MPO/MTP等配套受益于CPO和硅光连接密度提升。</t>
+          <t>涉及PCB干膜光刻胶材料，相关度低于容大和广信。</t>
         </is>
       </c>
     </row>
@@ -2903,17 +2903,17 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>002281</t>
+          <t>300570</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>光迅科技</t>
+          <t>太辰光</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>覆盖无源光器件、光纤阵列和模块平台，配套能力较完整。</t>
+          <t>高密度光连接器、MPO/MTP等配套受益于CPO和硅光连接密度提升。</t>
         </is>
       </c>
     </row>
@@ -2925,39 +2925,39 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>300620</t>
+          <t>002281</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>光库科技</t>
+          <t>光迅科技</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>保偏连接、光纤器件和铌酸锂相关器件具备协同。</t>
+          <t>覆盖无源光器件、光纤阵列和模块平台，配套能力较完整。</t>
         </is>
       </c>
     </row>
     <row r="85" ht="16.5" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>光纤</t>
+          <t>光纤连接 / 线缆配套</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>601869</t>
+          <t>300620</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>长飞光纤</t>
+          <t>光库科技</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>光纤预制棒、光纤、光缆一体化龙头，光纤板块直接度最高。</t>
+          <t>保偏连接、光纤器件和铌酸锂相关器件具备协同。</t>
         </is>
       </c>
     </row>
@@ -2969,17 +2969,17 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>600487</t>
+          <t>601869</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>亨通光电</t>
+          <t>长飞光纤</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>光棒、光纤、光缆、光器件和光通信网络方案平台型龙头。</t>
+          <t>光纤预制棒、光纤、光缆一体化龙头，光纤板块直接度最高。</t>
         </is>
       </c>
     </row>
@@ -2991,39 +2991,39 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>600522</t>
+          <t>600487</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>中天科技</t>
+          <t>亨通光电</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>光纤光缆、特种光缆和通信网络平台型公司，兼具空芯光纤等新方向弹性。</t>
+          <t>光棒、光纤、光缆、光器件和光通信网络方案平台型龙头。</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16.5" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>HBM / 高端DRAM</t>
+          <t>光纤</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>688008</t>
+          <t>600522</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>澜起科技</t>
+          <t>中天科技</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>DDR5内存接口芯片、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器高端内存互连核心受益。</t>
+          <t>光纤光缆、特种光缆和通信网络平台型公司，兼具空芯光纤等新方向弹性。</t>
         </is>
       </c>
     </row>
@@ -3035,39 +3035,39 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>300475</t>
+          <t>688008</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>香农芯创</t>
+          <t>澜起科技</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>SK海力士高端存储代理及企业级存储业务，受益DDR5/HBM紧缺和云服务客户备货，偏分销弹性。</t>
+          <t>DDR5内存接口芯片、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器高端内存互连核心受益。</t>
         </is>
       </c>
     </row>
     <row r="90" ht="16.5" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>数据中心电力 / 变压器</t>
+          <t>HBM / 高端DRAM</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>688676</t>
+          <t>300475</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>金盘科技</t>
+          <t>香农芯创</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>数据中心干式变压器和AIDC供电设备方向明确，受益AI数据中心电力设备交付紧张。</t>
+          <t>SK海力士高端存储代理及企业级存储业务，受益DDR5/HBM紧缺和云服务客户备货，偏分销弹性。</t>
         </is>
       </c>
     </row>
@@ -3079,17 +3079,17 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>002028</t>
+          <t>688676</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>金盘科技</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>变压器、GIS、开关设备和输配电控制平台，受益数据中心并网和全球电力设备紧缺。</t>
+          <t>数据中心干式变压器和AIDC供电设备方向明确，受益AI数据中心电力设备交付紧张。</t>
         </is>
       </c>
     </row>
@@ -3101,17 +3101,17 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>600089</t>
+          <t>002028</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>特变电工</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>大型变压器、特高压装备和线缆平台，受益电网投资与AI数据中心电力基础设施扩容。</t>
+          <t>变压器、GIS、开关设备和输配电控制平台，受益数据中心并网和全球电力设备紧缺。</t>
         </is>
       </c>
     </row>
@@ -3123,39 +3123,39 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>601179</t>
+          <t>600089</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>中国西电</t>
+          <t>特变电工</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>高压开关、变压器、输配电成套装备平台，受益电网主设备和数据中心并网需求。</t>
+          <t>大型变压器、特高压装备和线缆平台，受益电网投资与AI数据中心电力基础设施扩容。</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16.5" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>数据中心电力 / 变压器</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>600584</t>
+          <t>601179</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>长电科技</t>
+          <t>中国西电</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>先进封装平台龙头，布局2.5D/3D、Chiplet等，受益国产AI芯片封测升级；不等同台积电CoWoS。</t>
+          <t>高压开关、变压器、输配电成套装备平台，受益电网主设备和数据中心并网需求。</t>
         </is>
       </c>
     </row>
@@ -3167,61 +3167,61 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>002156</t>
+          <t>600584</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>通富微电</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>绑定高性能计算封测客户，FCBGA、Chiplet、2D+等先进封装扩产，受益AI/HPC封测需求。</t>
+          <t>先进封装平台龙头，布局2.5D/3D、Chiplet等，受益国产AI芯片封测升级；不等同台积电CoWoS。</t>
         </is>
       </c>
     </row>
     <row r="96" ht="16.5" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA / ABF载板</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>002436</t>
+          <t>002156</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>兴森科技</t>
+          <t>通富微电</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA/IC载板国产化主线，客户认证和良率爬坡推进，受益ABF/BT载板紧缺。</t>
+          <t>绑定高性能计算封测客户，FCBGA、Chiplet、2D+等先进封装扩产，受益AI/HPC封测需求。</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD / NAND</t>
+          <t>FC-BGA / ABF载板</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>688525</t>
+          <t>002436</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>佰维存储</t>
+          <t>兴森科技</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD、服务器内存和先进封测布局，受益AI服务器带动企业级存储放量。</t>
+          <t>FC-BGA/IC载板国产化主线，客户认证和良率爬坡推进，受益ABF/BT载板紧缺。</t>
         </is>
       </c>
     </row>
@@ -3233,17 +3233,17 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>301308</t>
+          <t>688525</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>江波龙</t>
+          <t>佰维存储</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD和数据中心存储方案，受益AI训练/推理带动高容量SSD需求。</t>
+          <t>企业级SSD、服务器内存和先进封测布局，受益AI服务器带动企业级存储放量。</t>
         </is>
       </c>
     </row>
@@ -3255,39 +3255,39 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>001309</t>
+          <t>301308</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>德明利</t>
+          <t>江波龙</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>存储模组和SSD控制器/模组链，受益NAND涨价与企业级存储需求，弹性偏周期。</t>
+          <t>企业级SSD和数据中心存储方案，受益AI训练/推理带动高容量SSD需求。</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>国产AI芯片 / 加速卡</t>
+          <t>企业级SSD / NAND</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>688256</t>
+          <t>001309</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>寒武纪</t>
+          <t>德明利</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>云端智能芯片和板卡最直接的A股国产AI算力芯片映射，核心看大客户、订单持续性、生态适配和估值消化。</t>
+          <t>存储模组和SSD控制器/模组链，受益NAND涨价与企业级存储需求，弹性偏周期。</t>
         </is>
       </c>
     </row>
@@ -3299,17 +3299,17 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>688041</t>
+          <t>688256</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>海光信息</t>
+          <t>寒武纪</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>CPU+DCU国产高端处理器平台，绑定国产服务器生态，算力国产化确定性强，弹性看DCU放量和软件栈。</t>
+          <t>云端智能芯片和板卡最直接的A股国产AI算力芯片映射，核心看大客户、订单持续性、生态适配和估值消化。</t>
         </is>
       </c>
     </row>
@@ -3321,39 +3321,39 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>300474</t>
+          <t>688041</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>景嘉微</t>
+          <t>海光信息</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>GPU+边端侧AI SoC路线，技术弹性强但仍需看通用算力产品商业化、亏损收窄和客户导入。</t>
+          <t>CPU+DCU国产高端处理器平台，绑定国产服务器生态，算力国产化确定性强，弹性看DCU放量和软件栈。</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>AI服务器 / ODM / 机架整机</t>
+          <t>国产AI芯片 / 加速卡</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>601138</t>
+          <t>300474</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>景嘉微</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>A股AI服务器和机架系统ODM最直接映射之一，覆盖云服务商AI服务器、高速网络和系统级整合。</t>
+          <t>GPU+边端侧AI SoC路线，技术弹性强但仍需看通用算力产品商业化、亏损收窄和客户导入。</t>
         </is>
       </c>
     </row>
@@ -3365,17 +3365,17 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>000977</t>
+          <t>601138</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>浪潮信息</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>国内AI服务器和IT基础设施龙头，服务器收入占比高，核心看AI服务器订单、毛利率和现金流质量。</t>
+          <t>A股AI服务器和机架系统ODM最直接映射之一，覆盖云服务商AI服务器、高速网络和系统级整合。</t>
         </is>
       </c>
     </row>
@@ -3387,17 +3387,17 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>603019</t>
+          <t>000977</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>中科曙光</t>
+          <t>浪潮信息</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>高端计算机、服务器、存储、液冷和算力服务平台，国产算力基础设施核心公司之一。</t>
+          <t>国内AI服务器和IT基础设施龙头，服务器收入占比高，核心看AI服务器订单、毛利率和现金流质量。</t>
         </is>
       </c>
     </row>
@@ -3409,24 +3409,24 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>000938</t>
+          <t>603019</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>紫光股份</t>
+          <t>中科曙光</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>新华三体系覆盖AI服务器、数据中心交换机、存储和液冷方案，兼具整机与网络平台属性。</t>
+          <t>高端计算机、服务器、存储、液冷和算力服务平台，国产算力基础设施核心公司之一。</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>AI网络设备 / 数据中心交换机</t>
+          <t>AI服务器 / ODM / 机架整机</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>新华三数据中心交换机份额靠前，800G智算交换机和无损网络方案是AI集群网络核心映射。</t>
+          <t>新华三体系覆盖AI服务器、数据中心交换机、存储和液冷方案，兼具整机与网络平台属性。</t>
         </is>
       </c>
     </row>
@@ -3453,17 +3453,17 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>301165</t>
+          <t>000938</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>锐捷网络</t>
+          <t>紫光股份</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>数据中心交换机产品受互联网和AI数据中心建设带动，订单交付和毛利率变化需持续跟踪。</t>
+          <t>新华三数据中心交换机份额靠前，800G智算交换机和无损网络方案是AI集群网络核心映射。</t>
         </is>
       </c>
     </row>
@@ -3475,39 +3475,39 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>000063</t>
+          <t>301165</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>中兴通讯</t>
+          <t>锐捷网络</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>连接+算力平台，覆盖AI服务器、存储、数据中心交换机和智算超节点，兼具设备与自研芯片线索。</t>
+          <t>数据中心交换机产品受互联网和AI数据中心建设带动，订单交付和毛利率变化需持续跟踪。</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>以太网交换芯片 / PHY</t>
+          <t>AI网络设备 / 数据中心交换机</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>688702</t>
+          <t>000063</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>盛科通信-U</t>
+          <t>中兴通讯</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>国产以太网交换芯片最直接A股映射，具备高性能端口和Tbps级架构储备，数据中心高端放量仍需验证。</t>
+          <t>连接+算力平台，覆盖AI服务器、存储、数据中心交换机和智算超节点，兼具设备与自研芯片线索。</t>
         </is>
       </c>
     </row>
@@ -3519,39 +3519,39 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>688515</t>
+          <t>688702</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>裕太微</t>
+          <t>盛科通信-U</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>以太网PHY和交换芯片国产化标的，下一代向数据中心等高价值场景延伸，当前更偏观察。</t>
+          <t>国产以太网交换芯片最直接A股映射，具备高性能端口和Tbps级架构储备，数据中心高端放量仍需验证。</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>CXL / PCIe Retimer / 内存互连</t>
+          <t>以太网交换芯片 / PHY</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>688008</t>
+          <t>688515</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>澜起科技</t>
+          <t>裕太微</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>DDR5接口、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器内存互连核心国产映射。</t>
+          <t>以太网PHY和交换芯片国产化标的，下一代向数据中心等高价值场景延伸，当前更偏观察。</t>
         </is>
       </c>
     </row>
@@ -3563,61 +3563,61 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>688008</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>澜起科技</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
+          <t>DDR5接口、MRCD/MDB、CKD、PCIe Retimer和CXL布局，AI服务器内存互连核心国产映射。</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>高速铜互连 / DAC-AEC / Twinax</t>
+          <t>CXL / PCIe Retimer / 内存互连</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>300913</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>兆龙互连</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>数据中心和AI算力中心高速布线、铜缆组件和连接产品映射，弹性看高速率产品客户导入。</t>
+          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>高速铜互连 / DAC-AEC / Twinax</t>
+          <t>低抖动时钟源 / 高端晶振</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>300563</t>
+          <t>603738</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>神宇股份</t>
+          <t>泰晶科技</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>已开发PCIe5.0/6.0/7.0及DAC 56G/112G/224G等高速数据线，属于铜互连高弹性观察标的。</t>
+          <t>石英晶振与硅振双路线，高基频低抖动差分振荡器切入AI数据中心、AI服务器、光模块和高速互连时钟源需求；2025年报披露312.5MHz差分输出温补振荡器、低抖动可编程振荡器及625MHz/1250MHz等MEMS/BAW方向，先按高端时钟源观察，核心看客户设计导入和规模收入。</t>
         </is>
       </c>
     </row>
@@ -3629,112 +3629,112 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>002130</t>
+          <t>300913</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>沃尔核材</t>
+          <t>兆龙互连</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>高速通信线缆和224G/800G/1.6T方向已有表内覆盖，建议在铜互连子环节中单列跟踪。</t>
+          <t>数据中心和AI算力中心高速布线、铜缆组件和连接产品映射，弹性看高速率产品客户导入。</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>GPU供电电感 / 磁性材料</t>
+          <t>高速铜互连 / DAC-AEC / Twinax</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>300811</t>
+          <t>300563</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>铂科新材</t>
+          <t>神宇股份</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>芯片电感和金属软磁材料切入AI服务器GPU供电，属于48V/板级供电上游高弹性补充。</t>
+          <t>已开发PCIe5.0/6.0/7.0及DAC 56G/112G/224G等高速数据线，属于铜互连高弹性观察标的。</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>GPU供电电感 / 磁性材料</t>
+          <t>高速铜互连 / DAC-AEC / Twinax</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>002138</t>
+          <t>002130</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>顺络电子</t>
+          <t>沃尔核材</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>功率电感、变压器等AI服务器供电上游元件已有表内覆盖，建议和铂科共同跟踪板级供电升级。</t>
+          <t>高速通信线缆和224G/800G/1.6T方向已有表内覆盖，建议在铜互连子环节中单列跟踪。</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>MLCC / 高端被动元件</t>
+          <t>高速铜互连 / DAC-AEC / Twinax</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>300408</t>
+          <t>688800</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>三环集团</t>
+          <t>瑞可达</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>MLCC与陶瓷材料平台，年报提到突破超高容大尺寸产品并加深服务器等客户合作，是Rubin MLCC增量映射。</t>
+          <t>募集说明书定义AEC/DAC/ACC高速线缆主要用于数据中心、高性能计算和电信网络，同时覆盖高速板对板、高速I/O、SFP+和CAGE连接器；与旭创体系有AEC方向合作线索。</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>MLCC / 高端被动元件</t>
+          <t>GPU供电电感 / 磁性材料</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>000636</t>
+          <t>300811</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>风华高科</t>
+          <t>铂科新材</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>MLCC、电阻、电感等被动元件覆盖AI算力等应用，弹性看高端规格、客户认证和盈利修复。</t>
+          <t>芯片电感和金属软磁材料切入AI服务器GPU供电，属于48V/板级供电上游高弹性补充。</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>MLCC / 高端被动元件</t>
+          <t>GPU供电电感 / 磁性材料</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -3749,139 +3749,139 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>功率电感和片式被动元件平台，适合作为AI服务器高可靠被动件和供电元件交叉跟踪。</t>
+          <t>功率电感、变压器等AI服务器供电上游元件已有表内覆盖，建议和铂科共同跟踪板级供电升级。</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>先进封装材料 / 底填 / EMC</t>
+          <t>MLCC / 高端被动元件</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>688535</t>
+          <t>300408</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>华海诚科</t>
+          <t>三环集团</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>环氧塑封料和电子胶黏剂平台，先进封装材料国产化映射，核心看高端封装客户与收入占比。</t>
+          <t>MLCC与陶瓷材料平台，年报提到突破超高容大尺寸产品并加深服务器等客户合作，是Rubin MLCC增量映射。</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>先进封装材料 / 底填 / EMC</t>
+          <t>MLCC / 高端被动元件</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>688035</t>
+          <t>000636</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>德邦科技</t>
+          <t>风华高科</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>底部填充胶、固晶、导热、晶圆UV膜等封装材料布局，适配Flip-chip、WLP、SiP、2.5D/3D封装。</t>
+          <t>MLCC、电阻、电感等被动元件覆盖AI算力等应用，弹性看高端规格、客户认证和盈利修复。</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>先进封装材料 / 底填 / EMC</t>
+          <t>MLCC / 高端被动元件</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>688300</t>
+          <t>002138</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>联瑞新材</t>
+          <t>顺络电子</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>球硅/低Df填料已有表内覆盖，也应归入先进封装和高端塑封材料填料链条交叉跟踪。</t>
+          <t>功率电感和片式被动元件平台，适合作为AI服务器高可靠被动件和供电元件交叉跟踪。</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>先进封装材料 / 底填 / EMC</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>300604</t>
+          <t>688535</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>长川科技</t>
+          <t>华海诚科</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备平台，HBM和先进封装拉动测试设备需求，核心看存储/SoC测试订单。</t>
+          <t>环氧塑封料和电子胶黏剂平台，先进封装材料国产化映射，核心看高端封装客户与收入占比。</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>先进封装材料 / 底填 / EMC</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>688200</t>
+          <t>688035</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>华峰测控</t>
+          <t>德邦科技</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>模拟、功率、SoC等测试系统平台，受AI芯片国产化和高端SoC测试需求拉动。</t>
+          <t>底部填充胶、固晶、导热、晶圆UV膜等封装材料布局，适配Flip-chip、WLP、SiP、2.5D/3D封装。</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>先进封装材料 / 底填 / EMC</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>688627</t>
+          <t>688300</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>精智达</t>
+          <t>联瑞新材</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>存储器后道测试、老化、探针卡和HBM/KGSD测试技术推进，是HBM测试国产映射。</t>
+          <t>球硅/低Df填料已有表内覆盖，也应归入先进封装和高端塑封材料填料链条交叉跟踪。</t>
         </is>
       </c>
     </row>
@@ -3893,1225 +3893,1401 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>688661</t>
+          <t>300604</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>和林微纳</t>
+          <t>长川科技</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>测试探针/探针卡耗材方向，属于半导体测试链条精密耗材补充，弹性看高端探针卡导入。</t>
+          <t>半导体测试设备平台，HBM和先进封装拉动测试设备需求，核心看存储/SoC测试订单。</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>800VDC / HVDC / 机柜供电</t>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>002851</t>
+          <t>688200</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>麦格米特</t>
+          <t>华峰测控</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>AI服务器电源已有表内覆盖，建议在800VDC/HVDC机柜供电子环节中单列观察客户导入。</t>
+          <t>模拟、功率、SoC等测试系统平台，受AI芯片国产化和高端SoC测试需求拉动。</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>800VDC / HVDC / 机柜供电</t>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>002922</t>
+          <t>688627</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>伊戈尔</t>
+          <t>精智达</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>数据中心移相、油浸、干式变压器和800V直流供电系统布局明确，是机柜供电升级补充标的。</t>
+          <t>存储器后道测试、老化、探针卡和HBM/KGSD测试技术推进，是HBM测试国产映射。</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>800VDC / HVDC / 机柜供电</t>
+          <t>半导体测试设备 / HBM测试 / 探针</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>002335</t>
+          <t>688661</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>科华数据</t>
+          <t>和林微纳</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>UPS、HVDC、液冷微模块和预制式电力模组覆盖智算中心供电系统，项目兑现度较高。</t>
+          <t>测试探针/探针卡耗材方向，属于半导体测试链条精密耗材补充，弹性看高端探针卡导入。</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>UPS / PDU / 低压配电 / Switchgear</t>
+          <t>半导体量测 / 缺陷检测 / 良率管理</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>002518</t>
+          <t>688361</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>科士达</t>
+          <t>中科飞测</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>UPS和数据中心关键基础设施公司，智慧电源和数据中心产品收入占比较高，海外UPS/HVDC需跟踪。</t>
+          <t>检测+量测设备平台，年报披露面向先进逻辑、先进存储及HBM 2.5D/3D封装提供光学、电子束、X光良率管理解决方案，是AI芯片/HBM制造良率节点补充。</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>UPS / PDU / 低压配电 / Switchgear</t>
+          <t>半导体量测 / 缺陷检测 / 良率管理</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>002335</t>
+          <t>300567</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>科华数据</t>
+          <t>精测电子</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>数据中心UPS、配电、液冷和微模块综合方案，适合放在电力基础设施核心补缺块。</t>
+          <t>半导体前道量检测设备、电子束设备和HBM BI测试系统均有披露，适合补入先进存储/HBM测试与量测节点；需持续看半导体业务收入占比和订单兑现。</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>UPS / PDU / 低压配电 / Switchgear</t>
+          <t>800VDC / HVDC / 机柜供电</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>002706</t>
+          <t>002851</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>良信股份</t>
+          <t>麦格米特</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>低压电器和智能配电产品用于智算中心等场景，属于数据中心低压配电与保护器件映射。</t>
+          <t>AI服务器电源已有表内覆盖，建议在800VDC/HVDC机柜供电子环节中单列观察客户导入。</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>OCS / 光交换 / 精密光学</t>
+          <t>800VDC / HVDC / 机柜供电</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>688195</t>
+          <t>002922</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>腾景科技</t>
+          <t>伊戈尔</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>精密光学元组件、光纤器件和光测试仪器平台，OCS/CPO相关精密光学为观察方向。</t>
+          <t>数据中心移相、油浸、干式变压器和800V直流供电系统布局明确，是机柜供电升级补充标的。</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>OCS / 光交换 / 精密光学</t>
+          <t>800VDC / HVDC / 机柜供电</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>300620</t>
+          <t>002335</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>光库科技</t>
+          <t>科华数据</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>保偏光纤器件、铌酸锂和光通信器件平台，可作为OCS/硅光/相干链条交叉观察。</t>
+          <t>UPS、HVDC、液冷微模块和预制式电力模组覆盖智算中心供电系统，项目兑现度较高。</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>OCS / 光交换 / 精密光学</t>
+          <t>UPS / PDU / 低压配电 / Switchgear</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>300394</t>
+          <t>002518</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>天孚通信</t>
+          <t>科士达</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>FAU、POSA、光引擎和高精度无源器件已在表内覆盖，也应纳入OCS/CPO精密光学迁移池。</t>
+          <t>UPS和数据中心关键基础设施公司，智慧电源和数据中心产品收入占比较高，海外UPS/HVDC需跟踪。</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+          <t>UPS / PDU / 低压配电 / Switchgear</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>601869</t>
+          <t>002335</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>长飞光纤</t>
+          <t>科华数据</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>空芯、多芯、G.654.E和数据中心光联接官方口径增强，但订单和规模收入仍需后续验证。</t>
+          <t>数据中心UPS、配电、液冷和微模块综合方案，适合放在电力基础设施核心补缺块。</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+          <t>UPS / PDU / 低压配电 / Switchgear</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>600487</t>
+          <t>002706</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>亨通光电</t>
+          <t>良信股份</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>光纤光缆和特种光纤平台型公司，建议从普通光纤中拆出新型光纤观察。</t>
+          <t>低压电器和智能配电产品用于智算中心等场景，属于数据中心低压配电与保护器件映射。</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+          <t>OCS / 光交换 / 精密光学</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>600522</t>
+          <t>688195</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>中天科技</t>
+          <t>腾景科技</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>光纤光缆和特种光缆平台，空芯/新型光纤属于中长期技术与交易弹性观察。</t>
+          <t>精密光学元组件、光纤器件和光测试仪器平台，OCS/CPO相关精密光学为观察方向。</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>PCB / HLC / HDI补充</t>
+          <t>OCS / 光交换 / 精密光学</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>688183</t>
+          <t>300620</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>生益电子</t>
+          <t>光库科技</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>高端PCB和智能算力互联核心组件研发投入明确，是AI服务器/高性能计算PCB补充核心。</t>
+          <t>保偏光纤器件、铌酸锂和光通信器件平台，可作为OCS/硅光/相干链条交叉观察。</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>PCB / HLC / HDI补充</t>
+          <t>OCS / 光交换 / 精密光学</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>002938</t>
+          <t>300394</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>鹏鼎控股</t>
+          <t>天孚通信</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>全球PCB龙头，AI云-管-端和AI服务器/光模块PCB布局加速，但A股主体与具体AI收入需继续拆分。</t>
+          <t>FAU、POSA、光引擎和高精度无源器件已在表内覆盖，也应纳入OCS/CPO精密光学迁移池。</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>晶圆代工 / 国产先进制程</t>
+          <t>空芯 / 多芯 / G.654.E新型光纤</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>688981</t>
+          <t>601869</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>中芯国际</t>
+          <t>长飞光纤</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>国产AI芯片制造底座，先进制程与成熟制程并行；受设备、EDA、IP与外部限制约束，不能直接等同先进GPU代工能力。</t>
+          <t>空芯、多芯、G.654.E和数据中心光联接官方口径增强，但订单和规模收入仍需后续验证。</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>晶圆代工 / 国产先进制程</t>
+          <t>空芯 / 多芯 / G.654.E新型光纤</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>688347</t>
+          <t>600487</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>华虹公司</t>
+          <t>亨通光电</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>特色工艺、功率、模拟与嵌入式平台，更多是AI服务器电源、边缘芯片和国产半导体底座映射，先进算力芯片弹性弱于中芯。</t>
+          <t>光纤光缆和特种光纤平台型公司，建议从普通光纤中拆出新型光纤观察。</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>前道设备 / 国产AI芯片制造</t>
+          <t>空芯 / 多芯 / G.654.E新型光纤</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>002371</t>
+          <t>600522</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>北方华创</t>
+          <t>中天科技</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>刻蚀、薄膜沉积、热处理、清洗等平台型设备龙头，国产晶圆制造CAPEX核心映射；AI链属于制造底座，不是直接下游订单。</t>
+          <t>光纤光缆和特种光缆平台，空芯/新型光纤属于中长期技术与交易弹性观察。</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>前道设备 / 国产AI芯片制造</t>
+          <t>PCB / HLC / HDI补充</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>688012</t>
+          <t>688183</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>中微公司</t>
+          <t>生益电子</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>刻蚀设备和MOCVD核心平台，先进制程国产设备主线，受益国产AI芯片制造和先进封装扩产。</t>
+          <t>高端PCB和智能算力互联核心组件研发投入明确，是AI服务器/高性能计算PCB补充核心。</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>前道设备 / 国产AI芯片制造</t>
+          <t>PCB / HLC / HDI补充</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>688072</t>
+          <t>002938</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>拓荆科技</t>
+          <t>鹏鼎控股</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>薄膜沉积设备平台，同时向混合键合相关检测/量测延伸，HBM/Chiplet先进封装为中长期弹性。</t>
+          <t>全球PCB龙头，AI云-管-端和AI服务器/光模块PCB布局加速，但A股主体与具体AI收入需继续拆分。</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>EDA / IP / ASIC设计服务</t>
+          <t>晶圆代工 / 国产先进制程</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>688521</t>
+          <t>688981</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>芯原股份</t>
+          <t>中芯国际</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>半导体IP和芯片定制服务平台，GPU/NPU/视频/接口IP与Chiplet方向相关，适合跟踪国产AI ASIC设计服务景气度。</t>
+          <t>国产AI芯片制造底座，先进制程与成熟制程并行；受设备、EDA、IP与外部限制约束，不能直接等同先进GPU代工能力。</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>EDA / IP / ASIC设计服务</t>
+          <t>晶圆代工 / 国产先进制程</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>301269</t>
+          <t>688347</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>华大九天</t>
+          <t>华虹公司</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>国产EDA平台核心标的，受益国产芯片设计和制造国产化；AI链映射偏工具层，业绩弹性看授权和客户扩张。</t>
+          <t>特色工艺、功率、模拟与嵌入式平台，更多是AI服务器电源、边缘芯片和国产半导体底座映射，先进算力芯片弹性弱于中芯。</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>EDA / IP / ASIC设计服务</t>
+          <t>前道设备 / 国产AI芯片制造</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>688206</t>
+          <t>002371</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>概伦电子</t>
+          <t>北方华创</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>器件建模、EDA和半导体良率/测试数据分析工具，偏国产EDA补链，交易弹性需看订单兑现。</t>
+          <t>刻蚀、薄膜沉积、热处理、清洗等平台型设备龙头，国产晶圆制造CAPEX核心映射；AI链属于制造底座，不是直接下游订单。</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA / ABF载板</t>
+          <t>前道设备 / 国产AI芯片制造</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>002916</t>
+          <t>688012</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>深南电路</t>
+          <t>中微公司</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>IC载板与FC-BGA能力建设，兼具PCB与封装基板平台，AI/HPC长期受益但需继续看良率、客户认证和收入占比。</t>
+          <t>刻蚀设备和MOCVD核心平台，先进制程国产设备主线，受益国产AI芯片制造和先进封装扩产。</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA / ABF载板</t>
+          <t>前道设备 / 国产AI芯片制造</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>002938</t>
+          <t>688072</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>鹏鼎控股</t>
+          <t>拓荆科技</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>全球PCB龙头，AI server PCB与IC substrate有体系映射；A股主体与具体AI收入仍需拆分验证。</t>
+          <t>薄膜沉积设备平台，同时向混合键合相关检测/量测延伸，HBM/Chiplet先进封装为中长期弹性。</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>EDA / IP / ASIC设计服务</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>688362</t>
+          <t>688521</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>甬矽电子</t>
+          <t>芯原股份</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>先进封装和系统级封装平台，适合作为AI/HPC封测国产化补充观察，确定性低于长电、通富。</t>
+          <t>半导体IP和芯片定制服务平台，GPU/NPU/视频/接口IP与Chiplet方向相关，适合跟踪国产AI ASIC设计服务景气度。</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>EDA / IP / ASIC设计服务</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>002185</t>
+          <t>301269</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>华天科技</t>
+          <t>华大九天</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>封测平台型公司，具备先进封装布局，更多是国产封测底座映射，AI/HBM收入纯度需跟踪。</t>
+          <t>国产EDA平台核心标的，受益国产芯片设计和制造国产化；AI链映射偏工具层，业绩弹性看授权和客户扩张。</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>EDA / IP / ASIC设计服务</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>688120</t>
+          <t>688206</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>华海清科</t>
+          <t>概伦电子</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>CMP、减薄和清洗设备平台，官方年报提到2.5D/RDL把芯片与HBM集成对CMP提出更高要求，是HBM/Chiplet设备映射。</t>
+          <t>器件建模、EDA和半导体良率/测试数据分析工具，偏国产EDA补链，交易弹性需看订单兑现。</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>FC-BGA / ABF载板</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>688082</t>
+          <t>002916</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>盛美上海</t>
+          <t>深南电路</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>清洗、电镀和面板级先进封装电镀设备，适配RDL/TSV/先进封装湿法制程，核心看封装客户订单放量。</t>
+          <t>IC载板与FC-BGA能力建设，兼具PCB与封装基板平台，AI/HPC长期受益但需继续看良率、客户认证和收入占比。</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>FC-BGA / ABF载板</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>688037</t>
+          <t>002938</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>芯源微</t>
+          <t>鹏鼎控股</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>后道先进封装涂胶显影、单片湿法、临时键合/解键合设备，适配超薄晶圆和HBM/Chiplet封装制程。</t>
+          <t>全球PCB龙头，AI server PCB与IC substrate有体系映射；A股主体与具体AI收入仍需拆分验证。</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>688072</t>
+          <t>688362</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>拓荆科技</t>
+          <t>甬矽电子</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>混合键合、键合套准量测和键合强度检测等先进封装线索明确，适合作为HBM/3D封装设备观察。</t>
+          <t>先进封装和系统级封装平台，适合作为AI/HPC封测国产化补充观察，确定性低于长电、通富。</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>300054</t>
+          <t>002185</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>鼎龙股份</t>
+          <t>华天科技</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>CMP抛光垫/抛光液/清洗液、半导体封装PI、PSPI和临时键合胶布局，卡位WLP/2.5D/3D封装材料。</t>
+          <t>封测平台型公司，具备先进封装布局，更多是国产封测底座映射，AI/HBM收入纯度需跟踪。</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>688019</t>
+          <t>688120</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>安集科技</t>
+          <t>华海清科</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>CMP抛光液和功能性湿电子化学品平台，先进制程与先进封装共同受益，核心看高端客户份额和新品放量。</t>
+          <t>CMP、减薄和清洗设备平台，官方年报提到2.5D/RDL把芯片与HBM集成对CMP提出更高要求，是HBM/Chiplet设备映射。</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>300236</t>
+          <t>688082</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>上海新阳</t>
+          <t>盛美上海</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>半导体电镀、清洗、Bumping/TSV相关材料，适配先进封装和晶圆级封装工艺。</t>
+          <t>清洗、电镀和面板级先进封装电镀设备，适配RDL/TSV/先进封装湿法制程，核心看封装客户订单放量。</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>688268</t>
+          <t>688037</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>华特气体</t>
+          <t>芯源微</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>高端特种气体明确提及HBM/TSV刻蚀等应用，属于存储和先进制程耗材映射，弹性看客户认证和放量。</t>
+          <t>后道先进封装涂胶显影、单片湿法、临时键合/解键合设备，适配超薄晶圆和HBM/Chiplet封装制程。</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>玻璃基板 / TGV / 玻璃中介层</t>
+          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>603773</t>
+          <t>688072</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>沃格光电</t>
+          <t>拓荆科技</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>年报把玻璃基板级封装线路载板和TGV用于AI大算力芯片、先进封装、高速传输等方向；当前仍按中长期观察。</t>
+          <t>混合键合、键合套准量测和键合强度检测等先进封装线索明确，适合作为HBM/3D封装设备观察。</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>玻璃基板 / TGV / 玻璃中介层</t>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>300776</t>
+          <t>300054</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>帝尔激光</t>
+          <t>鼎龙股份</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>年报提到TGV、PCB超快激光加工设备和先进封装装备，属于玻璃基板/高端PCB设备观察。</t>
+          <t>CMP抛光垫/抛光液/清洗液、半导体封装PI、PSPI和临时键合胶布局，卡位WLP/2.5D/3D封装材料。</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>300547</t>
+          <t>688019</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>川环科技</t>
+          <t>安集科技</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>公告披露获得服务器整体解决方案商液冷管路系统项目定点，后续看客户量产、单柜价值量和毛利。</t>
+          <t>CMP抛光液和功能性湿电子化学品平台，先进制程与先进封装共同受益，核心看高端客户份额和新品放量。</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>300731</t>
+          <t>300236</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>科创新源</t>
+          <t>上海新阳</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>通过创源智热布局数据中心散热结构件、液冷板和散热模组，处于客户开拓/认证阶段，弹性强但兑现早期。</t>
+          <t>半导体电镀、清洗、Bumping/TSV相关材料，适配先进封装和晶圆级封装工艺。</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>先进封装工艺材料 / CMP / PI / 特气</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>002536</t>
+          <t>688268</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>飞龙股份</t>
+          <t>华特气体</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>电子泵、温控阀等液冷热管理部件进入服务器液冷/IDC液冷/AI等场景，项目多但收入纯度需跟踪。</t>
+          <t>高端特种气体明确提及HBM/TSV刻蚀等应用，属于存储和先进制程耗材映射，弹性看客户认证和放量。</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>先进封装电镀液 / TSV-TGV添加剂</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>300602</t>
+          <t>688720</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>飞荣达</t>
+          <t>艾森股份</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>服务器/数据中心液冷散热、冷板、热管/VC和热管理材料平台，已在散热材料中覆盖，可在液冷部件维度单列。</t>
+          <t>年报披露HBM3E、Chiplet 3D堆叠、CoWoS-L等带动高纯电镀液、TSV/TGV添加剂需求，RDL/Bumping/TSV全工艺材料方案覆盖国内多数封装厂。</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+          <t>玻璃基板 / TGV / 玻璃中介层</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>688226</t>
+          <t>603773</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>威腾电气</t>
+          <t>沃格光电</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>数据中心相关母线及配电设备受益算力用电提升，年报提到数据中心机柜用智能型直流/交流母线槽。</t>
+          <t>年报把玻璃基板级封装线路载板和TGV用于AI大算力芯片、先进封装、高速传输等方向；当前仍按中长期观察。</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+          <t>玻璃基板 / TGV / 玻璃中介层</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>002706</t>
+          <t>300776</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>良信股份</t>
+          <t>帝尔激光</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>低压配电、智能断路器、智能盘柜面向数据中心等关键配电场景，适合与UPS/PDU/Switchgear共同跟踪。</t>
+          <t>年报提到TGV、PCB超快激光加工设备和先进封装装备，属于玻璃基板/高端PCB设备观察。</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>301031</t>
+          <t>300547</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>中熔电气</t>
+          <t>川环科技</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>熔断器和电路保护器件适配高压直流、储能和电力电子，AI机柜配电属于观察映射，需验证数据中心收入。</t>
+          <t>公告披露获得服务器整体解决方案商液冷管路系统项目定点，后续看客户量产、单柜价值量和毛利。</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>600745</t>
+          <t>300731</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>科创新源</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>安世半导体分立与功率器件平台，年报提到二极管、MOSFET、保护器件、电源管理IC、GaN FET、SiC MOS在数据中心降耗等领域应用。</t>
+          <t>通过创源智热布局数据中心散热结构件、液冷板和散热模组，处于客户开拓/认证阶段，弹性强但兑现早期。</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>605111</t>
+          <t>002536</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>新洁能</t>
+          <t>飞龙股份</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>SGT/SJ MOSFET、GateDriver、DrMOS等用于服务器电源、CPU/GPU板级供电、PFC/LLC等，AI服务器供电升级弹性明确。</t>
+          <t>电子泵、温控阀等液冷热管理部件进入服务器液冷/IDC液冷/AI等场景，项目多但收入纯度需跟踪。</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>688261</t>
+          <t>300602</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>东微半导</t>
+          <t>飞荣达</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>高压超级结MOSFET、SiC等功率器件平台，适配高效电源和HVDC方向，但AI数据中心客户需持续验证。</t>
+          <t>服务器/数据中心液冷散热、冷板、热管/VC和热管理材料平台，已在散热材料中覆盖，可在液冷部件维度单列。</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>液冷快接头 / UQD / 流体连接器</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>600460</t>
+          <t>002179</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>士兰微</t>
+          <t>中航光电</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>功率器件和功率模块平台，偏泛半导体受益，AI服务器电源纯度弱于新洁能/闻泰，需要观察导入。</t>
+          <t>年报列示流体连接器、流体传输管路、液冷机箱、液冷板、液冷源等液冷解决方案，应用于数据中心、超算、储能等高端装备，是液冷互连和流体连接器补缺核心。</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>高端电容 / 固态叠层 / 超级电容</t>
+          <t>液冷快接头 / UQD / 流体连接器</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>002484</t>
+          <t>688800</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>江海股份</t>
+          <t>瑞可达</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>MLPC固态叠层高分子电容、超级电容和铝电解平台，IR提到AI服务器研发阶段性成果；核心看批量订单。</t>
+          <t>面向AI与数据中心通信领域提供UQD冷却连接方案，服务器液冷UQD连接器和高速铜缆/AEC共同构成连接+冷却双线弹性。</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>高端电容 / 固态叠层 / 超级电容</t>
+          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>603989</t>
+          <t>688226</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>艾华集团</t>
+          <t>威腾电气</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>铝电解电容器平台，半年报提及把握AI服务器、数据中心等结构性机遇，适合作为电源电容补充。</t>
+          <t>数据中心相关母线及配电设备受益算力用电提升，年报提到数据中心机柜用智能型直流/交流母线槽。</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>高端电容 / 固态叠层 / 超级电容</t>
+          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>600563</t>
+          <t>002706</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>法拉电子</t>
+          <t>良信股份</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>薄膜电容器龙头，覆盖电力电子、储能、智能电网等高压场景，AI数据中心HVDC/电源链为中长期映射。</t>
+          <t>低压配电、智能断路器、智能盘柜面向数据中心等关键配电场景，适合与UPS/PDU/Switchgear共同跟踪。</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>300442</t>
+          <t>301031</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>中熔电气</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>润泽智算年报披露AIDC/AI算力中心运维、能效和算力服务能力，是下游算力基础设施运营商核心映射。</t>
+          <t>熔断器和电路保护器件适配高压直流、储能和电力电子，AI机柜配电属于观察映射，需验证数据中心收入。</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>300738</t>
+          <t>600745</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>奥飞数据</t>
+          <t>闻泰科技</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>半年度报告显示推进大型数据中心/智算中心项目建设交付，受益AI算力需求，需跟踪上架率和客户质量。</t>
+          <t>安世半导体分立与功率器件平台，年报提到二极管、MOSFET、保护器件、电源管理IC、GaN FET、SiC MOS在数据中心降耗等领域应用。</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>300383</t>
+          <t>605111</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>光环新网</t>
+          <t>新洁能</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>IDC和云计算平台，半年度报告提到AI驱动下数据中心硬件架构和运维变革；利润波动和项目回款需注意。</t>
+          <t>SGT/SJ MOSFET、GateDriver、DrMOS等用于服务器电源、CPU/GPU板级供电、PFC/LLC等，AI服务器供电升级弹性明确。</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>600845</t>
+          <t>688261</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>宝信软件</t>
+          <t>东微半导</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>工业智算云和智算中心/云计算节点布局，偏企业级和工业场景算力基础设施映射。</t>
+          <t>高压超级结MOSFET、SiC等功率器件平台，适配高效电源和HVDC方向，但AI数据中心客户需持续验证。</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
+          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>600460</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>士兰微</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>功率器件和功率模块平台，偏泛半导体受益，AI服务器电源纯度弱于新洁能/闻泰，需要观察导入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>高端电容 / 固态叠层 / 超级电容</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>002484</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>江海股份</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>MLPC固态叠层高分子电容、超级电容和铝电解平台，IR提到AI服务器研发阶段性成果；核心看批量订单。</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>高端电容 / 固态叠层 / 超级电容</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>603989</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>艾华集团</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>铝电解电容器平台，半年报提及把握AI服务器、数据中心等结构性机遇，适合作为电源电容补充。</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>高端电容 / 固态叠层 / 超级电容</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>600563</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>法拉电子</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>薄膜电容器龙头，覆盖电力电子、储能、智能电网等高压场景，AI数据中心HVDC/电源链为中长期映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>300442</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>润泽科技</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>润泽智算年报披露AIDC/AI算力中心运维、能效和算力服务能力，是下游算力基础设施运营商核心映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>300738</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>奥飞数据</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>半年度报告显示推进大型数据中心/智算中心项目建设交付，受益AI算力需求，需跟踪上架率和客户质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>300383</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>光环新网</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>IDC和云计算平台，半年度报告提到AI驱动下数据中心硬件架构和运维变革；利润波动和项目回款需注意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 智算中心 / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>600845</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>宝信软件</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>工业智算云和智算中心/云计算节点布局，偏企业级和工业场景算力基础设施映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
           <t>HCA / DPU / SmartNIC / RoCE</t>
         </is>
       </c>
-      <c r="B183" s="3" t="inlineStr">
+      <c r="B191" s="3" t="inlineStr">
         <is>
           <t>暂无</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>暂无成熟A股纯标的</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>该环节主要由NVIDIA/Mellanox、Broadcom、Marvell、Intel等主导；A股网络设备公司不等同HCA/DPU芯片。</t>
         </is>

</xml_diff>

<commit_message>
chore: update AI industry chain workbook
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1082,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D191"/>
+  <dimension ref="A1:D195"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1534,7 +1534,7 @@
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>M8 / M9高速CCL / 半固化片</t>
+          <t>M8 / M9高速CCL</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1556,7 +1556,7 @@
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>M8 / M9高速CCL / 半固化片</t>
+          <t>M8 / M9高速CCL</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1578,7 +1578,7 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>M8 / M9高速CCL / 半固化片</t>
+          <t>M8 / M9高速CCL</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2062,7 +2062,7 @@
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>FAU / MT / MPO / 微透镜 / 无源件</t>
+          <t>FAU / MT</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -2084,7 +2084,7 @@
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>FAU / MT / MPO / 微透镜 / 无源件</t>
+          <t>FAU / MT</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>FAU / MT / MPO / 微透镜 / 无源件</t>
+          <t>FAU / MT</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2128,7 +2128,7 @@
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>光模块封装 / 耦合 / 测试设备</t>
+          <t>光模块封装 / 耦合</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2150,7 +2150,7 @@
     <row r="49" ht="36" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>光模块封装 / 耦合 / 测试设备</t>
+          <t>光模块封装 / 耦合</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2172,7 +2172,7 @@
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>光模块封装 / 耦合 / 测试设备</t>
+          <t>光模块封装 / 耦合</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2194,7 +2194,7 @@
     <row r="51" ht="36" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>光模块封装 / 耦合 / 测试设备</t>
+          <t>光模块封装 / 耦合</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2282,7 +2282,7 @@
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>PD / APD / 接收芯片</t>
+          <t>PD / APD</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
     <row r="56" ht="36" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PD / APD / 接收芯片</t>
+          <t>PD / APD</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -2436,7 +2436,7 @@
     <row r="62" ht="36" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>PCB电镀设备 / mSAP / IC载板湿制程</t>
+          <t>PCB电镀设备 / mSAP</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -2458,7 +2458,7 @@
     <row r="63" ht="36" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>PCB钻针 / 微钻 / 刀具</t>
+          <t>PCB钻针 / 微钻</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <row r="64" ht="36" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>PCB钻针 / 微钻 / 刀具</t>
+          <t>PCB钻针 / 微钻</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -2788,7 +2788,7 @@
     <row r="78" ht="36" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>沉铜 / 电镀 / 表面处理药水</t>
+          <t>沉铜 / 电镀</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="79" ht="16.5" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>沉铜 / 电镀 / 表面处理药水</t>
+          <t>沉铜 / 电镀</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -2832,7 +2832,7 @@
     <row r="80" ht="16.5" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
+          <t>干膜 / 阻焊油墨</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -2854,7 +2854,7 @@
     <row r="81" ht="16.5" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
+          <t>干膜 / 阻焊油墨</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -2876,7 +2876,7 @@
     <row r="82" ht="16.5" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>干膜 / 阻焊油墨 / PCB光刻胶</t>
+          <t>干膜 / 阻焊油墨</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -3360,7 +3360,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>AI服务器 / ODM / 机架整机</t>
+          <t>AI服务器 / ODM</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -3382,7 +3382,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>AI服务器 / ODM / 机架整机</t>
+          <t>AI服务器 / ODM</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -3404,7 +3404,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>AI服务器 / ODM / 机架整机</t>
+          <t>AI服务器 / ODM</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>AI服务器 / ODM / 机架整机</t>
+          <t>AI服务器 / ODM</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3558,7 +3558,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>CXL / PCIe Retimer / 内存互连</t>
+          <t>CXL / PCIe Retimer</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>CXL / PCIe Retimer / 内存互连</t>
+          <t>CXL / PCIe Retimer</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -3624,7 +3624,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>高速铜互连 / DAC-AEC / Twinax</t>
+          <t>高速铜互连 / DAC-AEC</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -3646,7 +3646,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>高速铜互连 / DAC-AEC / Twinax</t>
+          <t>高速铜互连 / DAC-AEC</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -3668,7 +3668,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>高速铜互连 / DAC-AEC / Twinax</t>
+          <t>高速铜互连 / DAC-AEC</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -3690,7 +3690,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>高速铜互连 / DAC-AEC / Twinax</t>
+          <t>高速铜互连 / DAC-AEC</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -3822,7 +3822,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>先进封装材料 / 底填 / EMC</t>
+          <t>先进封装材料 / 底填</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3844,7 +3844,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>先进封装材料 / 底填 / EMC</t>
+          <t>先进封装材料 / 底填</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>先进封装材料 / 底填 / EMC</t>
+          <t>先进封装材料 / 底填</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -3888,7 +3888,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>半导体测试设备 / HBM测试</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -3910,7 +3910,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>半导体测试设备 / HBM测试</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -3932,7 +3932,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>半导体测试设备 / HBM测试</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -3954,7 +3954,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备 / HBM测试 / 探针</t>
+          <t>半导体测试设备 / HBM测试</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -3976,7 +3976,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>半导体量测 / 缺陷检测 / 良率管理</t>
+          <t>半导体量测 / 缺陷检测</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -3998,7 +3998,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>半导体量测 / 缺陷检测 / 良率管理</t>
+          <t>半导体量测 / 缺陷检测</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -4020,7 +4020,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>800VDC / HVDC / 机柜供电</t>
+          <t>800VDC / HVDC</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -4042,7 +4042,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>800VDC / HVDC / 机柜供电</t>
+          <t>800VDC / HVDC</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -4064,7 +4064,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>800VDC / HVDC / 机柜供电</t>
+          <t>800VDC / HVDC</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -4086,7 +4086,7 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>UPS / PDU / 低压配电 / Switchgear</t>
+          <t>UPS / PDU</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -4108,7 +4108,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>UPS / PDU / 低压配电 / Switchgear</t>
+          <t>UPS / PDU</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4130,7 +4130,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>UPS / PDU / 低压配电 / Switchgear</t>
+          <t>UPS / PDU</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4152,7 +4152,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>OCS / 光交换 / 精密光学</t>
+          <t>OCS / 光交换</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -4174,7 +4174,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>OCS / 光交换 / 精密光学</t>
+          <t>OCS / 光交换</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -4196,7 +4196,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>OCS / 光交换 / 精密光学</t>
+          <t>OCS / 光交换</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -4218,7 +4218,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+          <t>空芯 / 多芯</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
@@ -4240,7 +4240,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+          <t>空芯 / 多芯</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -4262,7 +4262,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>空芯 / 多芯 / G.654.E新型光纤</t>
+          <t>空芯 / 多芯</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4284,7 +4284,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>PCB / HLC / HDI补充</t>
+          <t>PCB / HLC</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -4306,7 +4306,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>PCB / HLC / HDI补充</t>
+          <t>PCB / HLC</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -4372,922 +4372,1010 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>前道设备 / 国产AI芯片制造</t>
+          <t>半导体洁净室 / 厂务工程</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>002371</t>
+          <t>603929</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>北方华创</t>
+          <t>亚翔集成</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>刻蚀、薄膜沉积、热处理、清洗等平台型设备龙头，国产晶圆制造CAPEX核心映射；AI链属于制造底座，不是直接下游订单。</t>
+          <t>半导体洁净室系统集成核心标的，2025年报披露电子行业-半导体收入占比较高，受益国产晶圆制造、存储、封测与海外半导体产能扩张；定位为AI芯片制造前序工程配套，不是GPU/光模块等核心器件。</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>前道设备 / 国产AI芯片制造</t>
+          <t>半导体洁净室 / 厂务工程</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>688012</t>
+          <t>601133</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>中微公司</t>
+          <t>柏诚股份</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>刻蚀设备和MOCVD核心平台，先进制程国产设备主线，受益国产AI芯片制造和先进封装扩产。</t>
+          <t>洁净室系统集成平台，半导体及泛半导体洁净室是高科技产业前序性投入，受益晶圆厂、先进封装、显示和高端制造扩产；弹性看订单质量、项目毛利率和回款。</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>前道设备 / 国产AI芯片制造</t>
+          <t>半导体洁净室 / 厂务工程</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>688072</t>
+          <t>603163</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>拓荆科技</t>
+          <t>圣晖集成</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>薄膜沉积设备平台，同时向混合键合相关检测/量测延伸，HBM/Chiplet先进封装为中长期弹性。</t>
+          <t>洁净室系统集成和二次配工程公司，IC半导体、封测、高阶PCB和东南亚扩产映射清晰；属于半导体资本开支和AI边缘应用扩产配套，需跟踪新签订单、在手订单和毛利率。</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>EDA / IP / ASIC设计服务</t>
+          <t>前道设备 / 国产AI芯片制造</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>688521</t>
+          <t>002371</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>芯原股份</t>
+          <t>北方华创</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>半导体IP和芯片定制服务平台，GPU/NPU/视频/接口IP与Chiplet方向相关，适合跟踪国产AI ASIC设计服务景气度。</t>
+          <t>刻蚀、薄膜沉积、热处理、清洗等平台型设备龙头，国产晶圆制造CAPEX核心映射；AI链属于制造底座，不是直接下游订单。</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>EDA / IP / ASIC设计服务</t>
+          <t>前道设备 / 国产AI芯片制造</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>301269</t>
+          <t>688012</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>华大九天</t>
+          <t>中微公司</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>国产EDA平台核心标的，受益国产芯片设计和制造国产化；AI链映射偏工具层，业绩弹性看授权和客户扩张。</t>
+          <t>刻蚀设备和MOCVD核心平台，先进制程国产设备主线，受益国产AI芯片制造和先进封装扩产。</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>EDA / IP / ASIC设计服务</t>
+          <t>前道设备 / 国产AI芯片制造</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>688206</t>
+          <t>688072</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>概伦电子</t>
+          <t>拓荆科技</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>器件建模、EDA和半导体良率/测试数据分析工具，偏国产EDA补链，交易弹性需看订单兑现。</t>
+          <t>薄膜沉积设备平台，同时向混合键合相关检测/量测延伸，HBM/Chiplet先进封装为中长期弹性。</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA / ABF载板</t>
+          <t>EDA / IP</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>002916</t>
+          <t>688521</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>深南电路</t>
+          <t>芯原股份</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>IC载板与FC-BGA能力建设，兼具PCB与封装基板平台，AI/HPC长期受益但需继续看良率、客户认证和收入占比。</t>
+          <t>半导体IP和芯片定制服务平台，GPU/NPU/视频/接口IP与Chiplet方向相关，适合跟踪国产AI ASIC设计服务景气度。</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>FC-BGA / ABF载板</t>
+          <t>EDA / IP</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>002938</t>
+          <t>301269</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>鹏鼎控股</t>
+          <t>华大九天</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>全球PCB龙头，AI server PCB与IC substrate有体系映射；A股主体与具体AI收入仍需拆分验证。</t>
+          <t>国产EDA平台核心标的，受益国产芯片设计和制造国产化；AI链映射偏工具层，业绩弹性看授权和客户扩张。</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>EDA / IP</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>688362</t>
+          <t>688206</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>甬矽电子</t>
+          <t>概伦电子</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>先进封装和系统级封装平台，适合作为AI/HPC封测国产化补充观察，确定性低于长电、通富。</t>
+          <t>器件建模、EDA和半导体良率/测试数据分析工具，偏国产EDA补链，交易弹性需看订单兑现。</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>先进封装 / CoWoS替代</t>
+          <t>FC-BGA / ABF载板</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>002185</t>
+          <t>002916</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>华天科技</t>
+          <t>深南电路</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>封测平台型公司，具备先进封装布局，更多是国产封测底座映射，AI/HBM收入纯度需跟踪。</t>
+          <t>IC载板与FC-BGA能力建设，兼具PCB与封装基板平台，AI/HPC长期受益但需继续看良率、客户认证和收入占比。</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>FC-BGA / ABF载板</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>688120</t>
+          <t>002938</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>华海清科</t>
+          <t>鹏鼎控股</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>CMP、减薄和清洗设备平台，官方年报提到2.5D/RDL把芯片与HBM集成对CMP提出更高要求，是HBM/Chiplet设备映射。</t>
+          <t>全球PCB龙头，AI server PCB与IC substrate有体系映射；A股主体与具体AI收入仍需拆分验证。</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>688082</t>
+          <t>688362</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>盛美上海</t>
+          <t>甬矽电子</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>清洗、电镀和面板级先进封装电镀设备，适配RDL/TSV/先进封装湿法制程，核心看封装客户订单放量。</t>
+          <t>先进封装和系统级封装平台，适合作为AI/HPC封测国产化补充观察，确定性低于长电、通富。</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>先进封装 / CoWoS替代</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>688037</t>
+          <t>002185</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>芯源微</t>
+          <t>华天科技</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>后道先进封装涂胶显影、单片湿法、临时键合/解键合设备，适配超薄晶圆和HBM/Chiplet封装制程。</t>
+          <t>封测平台型公司，具备先进封装布局，更多是国产封测底座映射，AI/HBM收入纯度需跟踪。</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>先进封装设备 / Hybrid bonding / TSV / CMP</t>
+          <t>先进封装设备 / Hybrid bonding</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>688072</t>
+          <t>688120</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>拓荆科技</t>
+          <t>华海清科</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>混合键合、键合套准量测和键合强度检测等先进封装线索明确，适合作为HBM/3D封装设备观察。</t>
+          <t>CMP、减薄和清洗设备平台，官方年报提到2.5D/RDL把芯片与HBM集成对CMP提出更高要求，是HBM/Chiplet设备映射。</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装设备 / Hybrid bonding</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>300054</t>
+          <t>688082</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>鼎龙股份</t>
+          <t>盛美上海</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>CMP抛光垫/抛光液/清洗液、半导体封装PI、PSPI和临时键合胶布局，卡位WLP/2.5D/3D封装材料。</t>
+          <t>清洗、电镀和面板级先进封装电镀设备，适配RDL/TSV/先进封装湿法制程，核心看封装客户订单放量。</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装设备 / Hybrid bonding</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>688019</t>
+          <t>688037</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>安集科技</t>
+          <t>芯源微</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>CMP抛光液和功能性湿电子化学品平台，先进制程与先进封装共同受益，核心看高端客户份额和新品放量。</t>
+          <t>后道先进封装涂胶显影、单片湿法、临时键合/解键合设备，适配超薄晶圆和HBM/Chiplet封装制程。</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装设备 / Hybrid bonding</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>300236</t>
+          <t>688072</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>上海新阳</t>
+          <t>拓荆科技</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>半导体电镀、清洗、Bumping/TSV相关材料，适配先进封装和晶圆级封装工艺。</t>
+          <t>混合键合、键合套准量测和键合强度检测等先进封装线索明确，适合作为HBM/3D封装设备观察。</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>先进封装工艺材料 / CMP / PI / 特气</t>
+          <t>先进封装工艺材料 / CMP</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>688268</t>
+          <t>300054</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>华特气体</t>
+          <t>鼎龙股份</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>高端特种气体明确提及HBM/TSV刻蚀等应用，属于存储和先进制程耗材映射，弹性看客户认证和放量。</t>
+          <t>CMP抛光垫/抛光液/清洗液、半导体封装PI、PSPI和临时键合胶布局，卡位WLP/2.5D/3D封装材料。</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>先进封装电镀液 / TSV-TGV添加剂</t>
+          <t>先进封装工艺材料 / CMP</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>688720</t>
+          <t>688019</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>艾森股份</t>
+          <t>安集科技</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>年报披露HBM3E、Chiplet 3D堆叠、CoWoS-L等带动高纯电镀液、TSV/TGV添加剂需求，RDL/Bumping/TSV全工艺材料方案覆盖国内多数封装厂。</t>
+          <t>CMP抛光液和功能性湿电子化学品平台，先进制程与先进封装共同受益，核心看高端客户份额和新品放量。</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>玻璃基板 / TGV / 玻璃中介层</t>
+          <t>先进封装工艺材料 / CMP</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>603773</t>
+          <t>300236</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>沃格光电</t>
+          <t>上海新阳</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>年报把玻璃基板级封装线路载板和TGV用于AI大算力芯片、先进封装、高速传输等方向；当前仍按中长期观察。</t>
+          <t>半导体电镀、清洗、Bumping/TSV相关材料，适配先进封装和晶圆级封装工艺。</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>玻璃基板 / TGV / 玻璃中介层</t>
+          <t>先进封装工艺材料 / CMP</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>300776</t>
+          <t>688268</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>帝尔激光</t>
+          <t>华特气体</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>年报提到TGV、PCB超快激光加工设备和先进封装装备，属于玻璃基板/高端PCB设备观察。</t>
+          <t>高端特种气体明确提及HBM/TSV刻蚀等应用，属于存储和先进制程耗材映射，弹性看客户认证和放量。</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>先进封装电镀液 / TSV-TGV添加剂</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>300547</t>
+          <t>688720</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>川环科技</t>
+          <t>艾森股份</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>公告披露获得服务器整体解决方案商液冷管路系统项目定点，后续看客户量产、单柜价值量和毛利。</t>
+          <t>年报披露HBM3E、Chiplet 3D堆叠、CoWoS-L等带动高纯电镀液、TSV/TGV添加剂需求，RDL/Bumping/TSV全工艺材料方案覆盖国内多数封装厂。</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>玻璃基板 / TGV</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>300731</t>
+          <t>603773</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>科创新源</t>
+          <t>沃格光电</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>通过创源智热布局数据中心散热结构件、液冷板和散热模组，处于客户开拓/认证阶段，弹性强但兑现早期。</t>
+          <t>年报把玻璃基板级封装线路载板和TGV用于AI大算力芯片、先进封装、高速传输等方向；当前仍按中长期观察。</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>玻璃基板 / TGV</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>002536</t>
+          <t>300776</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>飞龙股份</t>
+          <t>帝尔激光</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>电子泵、温控阀等液冷热管理部件进入服务器液冷/IDC液冷/AI等场景，项目多但收入纯度需跟踪。</t>
+          <t>年报提到TGV、PCB超快激光加工设备和先进封装装备，属于玻璃基板/高端PCB设备观察。</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>液冷管路 / 泵阀 / 快接头 / 冷板</t>
+          <t>液冷管路 / 泵阀</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>300602</t>
+          <t>300547</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>飞荣达</t>
+          <t>川环科技</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>服务器/数据中心液冷散热、冷板、热管/VC和热管理材料平台，已在散热材料中覆盖，可在液冷部件维度单列。</t>
+          <t>公告披露获得服务器整体解决方案商液冷管路系统项目定点，后续看客户量产、单柜价值量和毛利。</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>液冷快接头 / UQD / 流体连接器</t>
+          <t>液冷管路 / 泵阀</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>002179</t>
+          <t>300731</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>中航光电</t>
+          <t>科创新源</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>年报列示流体连接器、流体传输管路、液冷机箱、液冷板、液冷源等液冷解决方案，应用于数据中心、超算、储能等高端装备，是液冷互连和流体连接器补缺核心。</t>
+          <t>通过创源智热布局数据中心散热结构件、液冷板和散热模组，处于客户开拓/认证阶段，弹性强但兑现早期。</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>液冷快接头 / UQD / 流体连接器</t>
+          <t>液冷管路 / 泵阀</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>688800</t>
+          <t>002536</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>瑞可达</t>
+          <t>飞龙股份</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>面向AI与数据中心通信领域提供UQD冷却连接方案，服务器液冷UQD连接器和高速铜缆/AEC共同构成连接+冷却双线弹性。</t>
+          <t>电子泵、温控阀等液冷热管理部件进入服务器液冷/IDC液冷/AI等场景，项目多但收入纯度需跟踪。</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+          <t>液冷管路 / 泵阀</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>688226</t>
+          <t>300602</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>威腾电气</t>
+          <t>飞荣达</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>数据中心相关母线及配电设备受益算力用电提升，年报提到数据中心机柜用智能型直流/交流母线槽。</t>
+          <t>服务器/数据中心液冷散热、冷板、热管/VC和热管理材料平台，已在散热材料中覆盖，可在液冷部件维度单列。</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+          <t>液冷快接头 / UQD</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>002706</t>
+          <t>002179</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>良信股份</t>
+          <t>中航光电</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>低压配电、智能断路器、智能盘柜面向数据中心等关键配电场景，适合与UPS/PDU/Switchgear共同跟踪。</t>
+          <t>年报列示流体连接器、流体传输管路、液冷机箱、液冷板、液冷源等液冷解决方案，应用于数据中心、超算、储能等高端装备，是液冷互连和流体连接器补缺核心。</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>母线槽 / Busway / 机柜PDU / 低压配电</t>
+          <t>液冷快接头 / UQD</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>301031</t>
+          <t>688800</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>中熔电气</t>
+          <t>瑞可达</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>熔断器和电路保护器件适配高压直流、储能和电力电子，AI机柜配电属于观察映射，需验证数据中心收入。</t>
+          <t>面向AI与数据中心通信领域提供UQD冷却连接方案，服务器液冷UQD连接器和高速铜缆/AEC共同构成连接+冷却双线弹性。</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>母线槽 / Busway</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>600745</t>
+          <t>688226</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>威腾电气</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>安世半导体分立与功率器件平台，年报提到二极管、MOSFET、保护器件、电源管理IC、GaN FET、SiC MOS在数据中心降耗等领域应用。</t>
+          <t>数据中心相关母线及配电设备受益算力用电提升，年报提到数据中心机柜用智能型直流/交流母线槽。</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>母线槽 / Busway</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>605111</t>
+          <t>002706</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>新洁能</t>
+          <t>良信股份</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>SGT/SJ MOSFET、GateDriver、DrMOS等用于服务器电源、CPU/GPU板级供电、PFC/LLC等，AI服务器供电升级弹性明确。</t>
+          <t>低压配电、智能断路器、智能盘柜面向数据中心等关键配电场景，适合与UPS/PDU/Switchgear共同跟踪。</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>母线槽 / Busway</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>688261</t>
+          <t>301031</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>东微半导</t>
+          <t>中熔电气</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>高压超级结MOSFET、SiC等功率器件平台，适配高效电源和HVDC方向，但AI数据中心客户需持续验证。</t>
+          <t>熔断器和电路保护器件适配高压直流、储能和电力电子，AI机柜配电属于观察映射，需验证数据中心收入。</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>功率半导体 / GaN / SiC / MOSFET / DrMOS</t>
+          <t>功率半导体 / GaN</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>600460</t>
+          <t>600745</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>士兰微</t>
+          <t>闻泰科技</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>功率器件和功率模块平台，偏泛半导体受益，AI服务器电源纯度弱于新洁能/闻泰，需要观察导入。</t>
+          <t>安世半导体分立与功率器件平台，年报提到二极管、MOSFET、保护器件、电源管理IC、GaN FET、SiC MOS在数据中心降耗等领域应用。</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>高端电容 / 固态叠层 / 超级电容</t>
+          <t>功率半导体 / GaN</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>002484</t>
+          <t>605111</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>江海股份</t>
+          <t>新洁能</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>MLPC固态叠层高分子电容、超级电容和铝电解平台，IR提到AI服务器研发阶段性成果；核心看批量订单。</t>
+          <t>SGT/SJ MOSFET、GateDriver、DrMOS等用于服务器电源、CPU/GPU板级供电、PFC/LLC等，AI服务器供电升级弹性明确。</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>高端电容 / 固态叠层 / 超级电容</t>
+          <t>功率半导体 / GaN</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>603989</t>
+          <t>688261</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>艾华集团</t>
+          <t>东微半导</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>铝电解电容器平台，半年报提及把握AI服务器、数据中心等结构性机遇，适合作为电源电容补充。</t>
+          <t>高压超级结MOSFET、SiC等功率器件平台，适配高效电源和HVDC方向，但AI数据中心客户需持续验证。</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>高端电容 / 固态叠层 / 超级电容</t>
+          <t>功率半导体 / GaN</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>600563</t>
+          <t>600460</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>法拉电子</t>
+          <t>士兰微</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>薄膜电容器龙头，覆盖电力电子、储能、智能电网等高压场景，AI数据中心HVDC/电源链为中长期映射。</t>
+          <t>功率器件和功率模块平台，偏泛半导体受益，AI服务器电源纯度弱于新洁能/闻泰，需要观察导入。</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>高端电容 / 固态叠层</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>300442</t>
+          <t>002484</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>江海股份</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>润泽智算年报披露AIDC/AI算力中心运维、能效和算力服务能力，是下游算力基础设施运营商核心映射。</t>
+          <t>MLPC固态叠层高分子电容、超级电容和铝电解平台，IR提到AI服务器研发阶段性成果；核心看批量订单。</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>高端电容 / 固态叠层</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>300738</t>
+          <t>603989</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>奥飞数据</t>
+          <t>艾华集团</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>半年度报告显示推进大型数据中心/智算中心项目建设交付，受益AI算力需求，需跟踪上架率和客户质量。</t>
+          <t>铝电解电容器平台，半年报提及把握AI服务器、数据中心等结构性机遇，适合作为电源电容补充。</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>高端电容 / 固态叠层</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>300383</t>
+          <t>600563</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>光环新网</t>
+          <t>法拉电子</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>IDC和云计算平台，半年度报告提到AI驱动下数据中心硬件架构和运维变革；利润波动和项目回款需注意。</t>
+          <t>薄膜电容器龙头，覆盖电力电子、储能、智能电网等高压场景，AI数据中心HVDC/电源链为中长期映射。</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>IDC / 智算中心 / 算力基础设施</t>
+          <t>IDC / 算力基础设施</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>600845</t>
+          <t>300442</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>宝信软件</t>
+          <t>润泽科技</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>工业智算云和智算中心/云计算节点布局，偏企业级和工业场景算力基础设施映射。</t>
+          <t>润泽智算年报披露AIDC/AI算力中心运维、能效和算力服务能力，是下游算力基础设施运营商核心映射。</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>HCA / DPU / SmartNIC / RoCE</t>
+          <t>IDC / 算力基础设施</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
+          <t>300738</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>奥飞数据</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>半年度报告显示推进大型数据中心/智算中心项目建设交付，受益AI算力需求，需跟踪上架率和客户质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>300383</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>光环新网</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>IDC和云计算平台，半年度报告提到AI驱动下数据中心硬件架构和运维变革；利润波动和项目回款需注意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>600845</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>宝信软件</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>工业智算云和智算中心/云计算节点布局，偏企业级和工业场景算力基础设施映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>IDC / 算力基础设施</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>300857</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>协创数据</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>智能算力产品及服务、云算力租赁、算力服务器/集群交付和企业级SSD共同驱动；定位为下游算力服务/基础设施运营商，非GPU、光模块、PCB等上游硬瓶颈。核心跟踪客户验收计费、算力利用率、服务器采购资本开支、现金流和融资节奏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>HCA / DPU</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
           <t>暂无</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>暂无成熟A股纯标的</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>该环节主要由NVIDIA/Mellanox、Broadcom、Marvell、Intel等主导；A股网络设备公司不等同HCA/DPU芯片。</t>
         </is>

</xml_diff>

<commit_message>
chore: update AI chain WF6 entries
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1089,7 +1089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E384"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/业绩快报显示电子特种气体是公司主要收入来源，AI等新一代信息技术提升先进芯片、显示面板硬件需求，带动电子特气增长；主线保留半导体电子特气，需跟踪成熟品价格竞争和新产品放量节奏。</t>
+          <t>证据强：2025年报披露公司超高纯WF6用于集成电路CVD并具备2000吨/年产能，招股书披露产品纯度达6N以上、可满足不同制程需求，客户覆盖台积电、美光、SK海力士等海内外晶圆厂；AI链条来自先进芯片/存储扩产对CVD钨沉积电子特气需求的拉动。高端确定性强于一般电子特气平台，需跟踪海外新增订单公告、6N/7N价格、钨粉成本及成熟品竞争。</t>
         </is>
       </c>
       <c r="E251" s="6" t="inlineStr">
@@ -7856,17 +7856,17 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>688106</t>
+          <t>600378</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>金宏气体</t>
+          <t>昊华科技</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露电子特种气体国内市占率约2.81%，电子大宗载气提纯、现场制气及多个半导体/显示项目持续导入；但公司2025年增收不增利、应收较高，主板块由单一电子特气扩为半导体电子气体。</t>
+          <t>证据中强：昊华气体官网披露电子级六氟化钨5N产品，公开互动口径称WF6产能约600吨/年；AI链条来自先进制程/存储芯片CVD钨沉积用电子特气需求，确定性和客户验证透明度弱于中船特气，需跟踪6N升级、客户认证、出口订单和钨粉成本传导。</t>
         </is>
       </c>
       <c r="E252" s="6" t="inlineStr">
@@ -7878,22 +7878,22 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>半导体前驱体材料</t>
+          <t>半导体电子特气</t>
         </is>
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>300346</t>
+          <t>688106</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>南大光电</t>
+          <t>金宏气体</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司围绕先进前驱体、电子特气、光刻胶及配套材料三大核心半导体材料发展，业绩连续增长；光刻胶有产业化突破但收入规模仍需跟踪，主线从光刻胶/ALD-CVD前驱体重复标签收敛为半导体前驱体材料。</t>
+          <t>证据中强：2025年报披露电子特种气体国内市占率约2.81%，电子大宗载气提纯、现场制气及多个半导体/显示项目持续导入；但公司2025年增收不增利、应收较高，主板块由单一电子特气扩为半导体电子气体。</t>
         </is>
       </c>
       <c r="E253" s="6" t="inlineStr">
@@ -7905,22 +7905,22 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>半导体高纯金属靶材</t>
+          <t>半导体前驱体材料</t>
         </is>
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>300666</t>
+          <t>300346</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>江丰电子</t>
+          <t>南大光电</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示公司核心产品为超高纯金属溅射靶材，覆盖先进制程及存储、逻辑、功率等客户，半导体靶材收入占比高；HBM TSV金属材料属于先进封装/存储升级延伸，证据仍弱于靶材主业，合并删减“HBM TSV金属材料”重复行。</t>
+          <t>证据中强：2025年报显示公司围绕先进前驱体、电子特气、光刻胶及配套材料三大核心半导体材料发展，业绩连续增长；光刻胶有产业化突破但收入规模仍需跟踪，主线从光刻胶/ALD-CVD前驱体重复标签收敛为半导体前驱体材料。</t>
         </is>
       </c>
       <c r="E254" s="6" t="inlineStr">
@@ -7937,17 +7937,17 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>600206</t>
+          <t>300666</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>有研新材</t>
+          <t>江丰电子</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦电子薄膜及贵金属材料等新材料，集成电路及半导体薄膜材料国产化需求持续；高纯金属靶材是更确定主线，HBM TSV金属材料属于先进存储/封装延伸，当前公开证据不足以作为主板块。</t>
+          <t>证据强：2025年报显示公司核心产品为超高纯金属溅射靶材，覆盖先进制程及存储、逻辑、功率等客户，半导体靶材收入占比高；HBM TSV金属材料属于先进封装/存储升级延伸，证据仍弱于靶材主业，合并删减“HBM TSV金属材料”重复行。</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
@@ -7959,22 +7959,22 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>半导体先进陶瓷部件</t>
+          <t>半导体高纯金属靶材</t>
         </is>
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>301611</t>
+          <t>600206</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>珂玛科技</t>
+          <t>有研新材</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以半导体先进陶瓷零部件为核心，陶瓷加热器已大批量交付，静电卡盘8/12英寸产品通过客户验证并小规模量产；静电卡盘弹性清晰但收入仍小，主板块由单一静电卡盘修正为半导体先进陶瓷部件。</t>
+          <t>证据中强：2025年报披露公司聚焦电子薄膜及贵金属材料等新材料，集成电路及半导体薄膜材料国产化需求持续；高纯金属靶材是更确定主线，HBM TSV金属材料属于先进存储/封装延伸，当前公开证据不足以作为主板块。</t>
         </is>
       </c>
       <c r="E256" s="6" t="inlineStr">
@@ -7986,22 +7986,22 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>碳化硅衬底</t>
+          <t>半导体先进陶瓷部件</t>
         </is>
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>688234</t>
+          <t>301611</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>天岳先进</t>
+          <t>珂玛科技</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营碳化硅衬底，导电型SiC衬底全球份额27.6%、8英寸份额51.3%；AI数据中心拉动SiC材料应用是中长期变量，但2025收入下滑并亏损，需跟踪价格和产能利用率。</t>
+          <t>证据中强：2025年报披露公司以半导体先进陶瓷零部件为核心，陶瓷加热器已大批量交付，静电卡盘8/12英寸产品通过客户验证并小规模量产；静电卡盘弹性清晰但收入仍小，主板块由单一静电卡盘修正为半导体先进陶瓷部件。</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
@@ -8013,22 +8013,22 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>内存接口芯片</t>
+          <t>碳化硅衬底</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>688008</t>
+          <t>688234</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>澜起科技</t>
+          <t>天岳先进</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>DDR5 RCD/DB、MRCD/MDB、CKD是AI服务器高带宽内存互连核心节点，PCIe Retimer、CXL MXC扩展高速互连第二曲线；主板块收敛为内存接口芯片，HBM、DDR5 SPD、SOCAMM、CXL和CXL内存扩展模组均并入备注或删除，避免误当存储模组/HBM厂商。风险是海外竞争、服务器平台迭代和新品放量节奏。证据A。</t>
+          <t>证据强：2025年报披露公司主营碳化硅衬底，导电型SiC衬底全球份额27.6%、8英寸份额51.3%；AI数据中心拉动SiC材料应用是中长期变量，但2025收入下滑并亏损，需跟踪价格和产能利用率。</t>
         </is>
       </c>
       <c r="E258" s="6" t="inlineStr">
@@ -8040,22 +8040,22 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>DDR5 SPD</t>
+          <t>内存接口芯片</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>688123</t>
+          <t>688008</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>聚辰股份</t>
+          <t>澜起科技</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>公司具备DDR2/3/4/5内存模组配套SPD、TS等芯片产品，DDR5 SPD受益AI服务器内存模组数量提升，是明确的小芯片弹性节点；主板块保留DDR5 SPD，SOCAMM作为下游内存模组形态并入备注，不单列。风险是DDR5渗透节奏、客户导入、EEPROM周期和价格竞争。证据A。</t>
+          <t>DDR5 RCD/DB、MRCD/MDB、CKD是AI服务器高带宽内存互连核心节点，PCIe Retimer、CXL MXC扩展高速互连第二曲线；主板块收敛为内存接口芯片，HBM、DDR5 SPD、SOCAMM、CXL和CXL内存扩展模组均并入备注或删除，避免误当存储模组/HBM厂商。风险是海外竞争、服务器平台迭代和新品放量节奏。证据A。</t>
         </is>
       </c>
       <c r="E259" s="6" t="inlineStr">
@@ -8067,22 +8067,22 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>高端存储分销</t>
+          <t>DDR5 SPD</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>300475</t>
+          <t>688123</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>香农芯创</t>
+          <t>聚辰股份</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>公司以SK海力士核心代理分销为基本盘，向国内云服务器龙头和大型ODM提供存储解决方案；HBM/DDR5紧缺带来强周期弹性，但本质不是HBM制造商。自主海普存储企业级SSD/DRAM开始贡献增量。主板块由HBM改为高端存储分销，风险是存储价格周期、供应商授权、分销毛利和库存。证据A/B。</t>
+          <t>公司具备DDR2/3/4/5内存模组配套SPD、TS等芯片产品，DDR5 SPD受益AI服务器内存模组数量提升，是明确的小芯片弹性节点；主板块保留DDR5 SPD，SOCAMM作为下游内存模组形态并入备注，不单列。风险是DDR5渗透节奏、客户导入、EEPROM周期和价格竞争。证据A。</t>
         </is>
       </c>
       <c r="E260" s="6" t="inlineStr">
@@ -8094,22 +8094,22 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>企业级存储模组</t>
+          <t>高端存储分销</t>
         </is>
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>688525</t>
+          <t>300475</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>佰维存储</t>
+          <t>香农芯创</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>公司企业级存储方案覆盖PCIe/SATA SSD、DDR4/DDR5 RDIMM和CXL内存扩展模组，服务数据中心、服务器和AI工作负载；主板块由DDR5 SPD改为企业级存储模组，SOCAMM、企业级SSD、SSD主控、UFS、晶圆级封测和CXL并入备注或降级。风险是NAND/DRAM价格周期、库存、客户认证和自研控制器/封测兑现。证据B。</t>
+          <t>公司以SK海力士核心代理分销为基本盘，向国内云服务器龙头和大型ODM提供存储解决方案；HBM/DDR5紧缺带来强周期弹性，但本质不是HBM制造商。自主海普存储企业级SSD/DRAM开始贡献增量。主板块由HBM改为高端存储分销，风险是存储价格周期、供应商授权、分销毛利和库存。证据A/B。</t>
         </is>
       </c>
       <c r="E261" s="6" t="inlineStr">
@@ -8126,17 +8126,17 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>301308</t>
+          <t>688525</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>江波龙</t>
+          <t>佰维存储</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>公司企业级eSSD和RDIMM已在互联网、运营商等客户完成验证并批量出货，SOCAMM2、CXL内存扩展、MRDIMM等构成AI服务器存储升级可选项；主板块由SOCAMM改为企业级存储模组，端侧UFS、eMMC、SSD主控、SPU、HLC-iSA、mSSD和CXL并入备注。SOCAMM2仍需收入贡献验证。证据A/B。</t>
+          <t>公司企业级存储方案覆盖PCIe/SATA SSD、DDR4/DDR5 RDIMM和CXL内存扩展模组，服务数据中心、服务器和AI工作负载；主板块由DDR5 SPD改为企业级存储模组，SOCAMM、企业级SSD、SSD主控、UFS、晶圆级封测和CXL并入备注或降级。风险是NAND/DRAM价格周期、库存、客户认证和自研控制器/封测兑现。证据B。</t>
         </is>
       </c>
       <c r="E262" s="6" t="inlineStr">
@@ -8148,22 +8148,22 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD</t>
+          <t>企业级存储模组</t>
         </is>
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>001309</t>
+          <t>301308</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>德明利</t>
+          <t>江波龙</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露AI浪潮下公司加快向高容量、高性能固态硬盘拓展，重点聚焦QLC NAND企业级应用方向；自研主控是能力基础，但表格保留最贴近收入承载的“企业级SSD”，删减企业级SSD主控、QLC SSD、AI场景化存储方案重复行。风险是存储价格周期和经营现金流波动。</t>
+          <t>公司企业级eSSD和RDIMM已在互联网、运营商等客户完成验证并批量出货，SOCAMM2、CXL内存扩展、MRDIMM等构成AI服务器存储升级可选项；主板块由SOCAMM改为企业级存储模组，端侧UFS、eMMC、SSD主控、SPU、HLC-iSA、mSSD和CXL并入备注。SOCAMM2仍需收入贡献验证。证据A/B。</t>
         </is>
       </c>
       <c r="E263" s="6" t="inlineStr">
@@ -8175,22 +8175,22 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD主控</t>
+          <t>企业级SSD</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>300672</t>
+          <t>001309</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>国科微</t>
+          <t>德明利</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>证据中偏弱：公司固态存储主控芯片实现国产替代，同时布局端侧AI、车载电子、智慧视觉等多条芯片线；AI数据中心企业级SSD客户、收入占比和订单仍未充分披露，保留为SSD主控国产替代观察，基本面需关注2025亏损后毛利修复和研发投入转化。</t>
+          <t>证据中强：2025年报摘要披露AI浪潮下公司加快向高容量、高性能固态硬盘拓展，重点聚焦QLC NAND企业级应用方向；自研主控是能力基础，但表格保留最贴近收入承载的“企业级SSD”，删减企业级SSD主控、QLC SSD、AI场景化存储方案重复行。风险是存储价格周期和经营现金流波动。</t>
         </is>
       </c>
       <c r="E264" s="6" t="inlineStr">
@@ -8207,17 +8207,17 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>688449</t>
+          <t>300672</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>联芸科技</t>
+          <t>国科微</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露SSD主控覆盖SATA、PCIe3.0/4.0/5.0，企业级PCIe Gen5 SSD主控已进入量产测试阶段，并规划PCIe Gen6/Gen7切入数据中心；删减UFS主控重复行，UFS偏终端嵌入式，AI算力弹性以企业级SSD主控为主。</t>
+          <t>证据中偏弱：公司固态存储主控芯片实现国产替代，同时布局端侧AI、车载电子、智慧视觉等多条芯片线；AI数据中心企业级SSD客户、收入占比和订单仍未充分披露，保留为SSD主控国产替代观察，基本面需关注2025亏损后毛利修复和研发投入转化。</t>
         </is>
       </c>
       <c r="E265" s="6" t="inlineStr">
@@ -8229,22 +8229,22 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>AI存储</t>
+          <t>企业级SSD主控</t>
         </is>
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>300302</t>
+          <t>688449</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>同有科技</t>
+          <t>联芸科技</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露高端存储在AI智算中心、高性能计算等核心场景推进，NVMe/RDMA高性能分布式文件存储用于智算领域高并发、低延迟需求；主板块保留AI存储，跟踪标杆方案复制、国产化替代和毛利率。</t>
+          <t>证据强：2025年报披露SSD主控覆盖SATA、PCIe3.0/4.0/5.0，企业级PCIe Gen5 SSD主控已进入量产测试阶段，并规划PCIe Gen6/Gen7切入数据中心；删减UFS主控重复行，UFS偏终端嵌入式，AI算力弹性以企业级SSD主控为主。</t>
         </is>
       </c>
       <c r="E266" s="6" t="inlineStr">
@@ -8256,30 +8256,34 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>HBF高带宽闪存</t>
+          <t>AI存储</t>
         </is>
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>300302</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>同有科技</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>德明利2025半年报提到闪迪HBF结合3D NAND与HBM、适合读取密集型AI推理任务；A股暂无成熟高带宽闪存纯标的。</t>
-        </is>
-      </c>
-      <c r="E267" s="6" t="n"/>
+          <t>证据强：2025年报披露高端存储在AI智算中心、高性能计算等核心场景推进，NVMe/RDMA高性能分布式文件存储用于智算领域高并发、低延迟需求；主板块保留AI存储，跟踪标杆方案复制、国产化替代和毛利率。</t>
+        </is>
+      </c>
+      <c r="E267" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>Nearline HDD</t>
+          <t>HBF高带宽闪存</t>
         </is>
       </c>
       <c r="B268" s="3" t="inlineStr">
@@ -8294,7 +8298,7 @@
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>希捷和西部数据官方披露AI数据增长推动数据中心exabyte级低成本存储需求；近线HDD仍主要由海外双寡头主导。</t>
+          <t>德明利2025半年报提到闪迪HBF结合3D NAND与HBM、适合读取密集型AI推理任务；A股暂无成熟高带宽闪存纯标的。</t>
         </is>
       </c>
       <c r="E268" s="6" t="n"/>
@@ -8302,7 +8306,7 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>HAMR-ePMR高容量HDD</t>
+          <t>Nearline HDD</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr">
@@ -8317,7 +8321,7 @@
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>希捷披露HAMR Mozaic放量，西部数据披露40TB UltraSMR ePMR验证和HAMR 100TB路线；A股暂无成熟HDD主线标的。</t>
+          <t>希捷和西部数据官方披露AI数据增长推动数据中心exabyte级低成本存储需求；近线HDD仍主要由海外双寡头主导。</t>
         </is>
       </c>
       <c r="E269" s="6" t="n"/>
@@ -8325,7 +8329,7 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>高带宽HDD</t>
+          <t>HAMR-ePMR高容量HDD</t>
         </is>
       </c>
       <c r="B270" s="3" t="inlineStr">
@@ -8340,7 +8344,7 @@
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>西部数据2026 Innovation Day披露High Bandwidth Drive与Dual Pivot提升HDD带宽/IO，服务AI温冷数据层，A股暂无对应纯标的。</t>
+          <t>希捷披露HAMR Mozaic放量，西部数据披露40TB UltraSMR ePMR验证和HAMR 100TB路线；A股暂无成熟HDD主线标的。</t>
         </is>
       </c>
       <c r="E270" s="6" t="n"/>
@@ -8348,7 +8352,7 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>CXL</t>
+          <t>高带宽HDD</t>
         </is>
       </c>
       <c r="B271" s="3" t="inlineStr">
@@ -8363,7 +8367,7 @@
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
+          <t>西部数据2026 Innovation Day披露High Bandwidth Drive与Dual Pivot提升HDD带宽/IO，服务AI温冷数据层，A股暂无对应纯标的。</t>
         </is>
       </c>
       <c r="E271" s="6" t="n"/>
@@ -8371,22 +8375,22 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>CXL内存扩展模组</t>
+          <t>CXL</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
           <t>暂无成熟A股纯标的</t>
         </is>
       </c>
-      <c r="C272" s="2" t="inlineStr">
-        <is>
-          <t>CXL Switch暂无成熟A股纯标的</t>
-        </is>
-      </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>CXL交换/池化控制仍主要由Marvell等海外厂商推进，A股目前缺成熟CXL Switch纯标的。</t>
+          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
         </is>
       </c>
       <c r="E272" s="6" t="n"/>
@@ -8394,49 +8398,45 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>HBM BI</t>
+          <t>CXL内存扩展模组</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>300567</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>精测电子</t>
+          <t>CXL Switch暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>检测设备平台，2025年报摘要披露推出JH5520 HBM BI测试系统以满足HBM高端存储测试需求，半导体量检测覆盖前道、后道电测和先进封装；主板块改为HBM BI，PCB AOI、半导体量测和先进封装X-Ray并入备注，风险是半导体业务收入占比、客户认证和设备订单兑现。证据A/B。</t>
-        </is>
-      </c>
-      <c r="E273" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>CXL交换/池化控制仍主要由Marvell等海外厂商推进，A股目前缺成熟CXL Switch纯标的。</t>
+        </is>
+      </c>
+      <c r="E273" s="6" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>AI服务器整机</t>
+          <t>HBM BI</t>
         </is>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>603019</t>
+          <t>300567</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>中科曙光</t>
+          <t>精测电子</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心是高端计算机、智能计算和算力服务，2025年报披露继续围绕AI算力、液冷散热、高速互联等核心领域投入；AI存储和推理板卡只是配套能力，删减AI存储、AI推理板卡、AI服务器ODM重复行，保留更准确的AI服务器整机/智算底座定位。</t>
+          <t>检测设备平台，2025年报摘要披露推出JH5520 HBM BI测试系统以满足HBM高端存储测试需求，半导体量检测覆盖前道、后道电测和先进封装；主板块改为HBM BI，PCB AOI、半导体量测和先进封装X-Ray并入备注，风险是半导体业务收入占比、客户认证和设备订单兑现。证据A/B。</t>
         </is>
       </c>
       <c r="E274" s="6" t="inlineStr">
@@ -8453,17 +8453,17 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>000977</t>
+          <t>603019</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>浪潮信息</t>
+          <t>中科曙光</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露总营收1647.82亿元、同比增长43.25%，主要由服务器产品销售增长驱动；存储交换类收入占比小，删减AI存储重复行，主板块改为AI服务器整机。风险是服务器高增但毛利率偏低，GPU/核心器件供应和价格压力影响利润弹性。</t>
+          <t>证据中强：公司核心是高端计算机、智能计算和算力服务，2025年报披露继续围绕AI算力、液冷散热、高速互联等核心领域投入；AI存储和推理板卡只是配套能力，删减AI存储、AI推理板卡、AI服务器ODM重复行，保留更准确的AI服务器整机/智算底座定位。</t>
         </is>
       </c>
       <c r="E275" s="6" t="inlineStr">
@@ -8480,17 +8480,17 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>000034</t>
+          <t>000977</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>神州数码</t>
+          <t>浪潮信息</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露AI相关业务收入330.3亿元、同比增长47.7%，神州鲲泰服务器基于鲲鹏CPU+昇腾NPU支持DeepSeek等大模型私有化部署，并开放国产技术栈AI智算OpenLab；主线是国产算力整机和方案。</t>
+          <t>证据强：2025年报披露总营收1647.82亿元、同比增长43.25%，主要由服务器产品销售增长驱动；存储交换类收入占比小，删减AI存储重复行，主板块改为AI服务器整机。风险是服务器高增但毛利率偏低，GPU/核心器件供应和价格压力影响利润弹性。</t>
         </is>
       </c>
       <c r="E276" s="6" t="inlineStr">
@@ -8507,17 +8507,17 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>002261</t>
+          <t>000034</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>拓维信息</t>
+          <t>神州数码</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露公司基于“鲲鹏+昇腾AI”算力底座，推出中心侧高性能服务器、推理服务器和边端终端侧产品；主板块从国产AI服务器收敛为昇腾AI服务器，风险是收入下滑、利润体量仍小。</t>
+          <t>证据中强：2025年报披露AI相关业务收入330.3亿元、同比增长47.7%，神州鲲泰服务器基于鲲鹏CPU+昇腾NPU支持DeepSeek等大模型私有化部署，并开放国产技术栈AI智算OpenLab；主线是国产算力整机和方案。</t>
         </is>
       </c>
       <c r="E277" s="6" t="inlineStr">
@@ -8529,22 +8529,22 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>AI服务器ODM</t>
+          <t>AI服务器整机</t>
         </is>
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>601138</t>
+          <t>002261</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>拓维信息</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司与全球头部客户协同下一代AI服务器及液冷技术，云服务商AI服务器收入同比大增，GPU与ASIC方案产品快速增长；删减“AI服务器机柜”重复行，机柜/液冷作为ODM系统能力纳入备注。</t>
+          <t>证据中：2025年报摘要披露公司基于“鲲鹏+昇腾AI”算力底座，推出中心侧高性能服务器、推理服务器和边端终端侧产品；主板块从国产AI服务器收敛为昇腾AI服务器，风险是收入下滑、利润体量仍小。</t>
         </is>
       </c>
       <c r="E278" s="6" t="inlineStr">
@@ -8561,17 +8561,17 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>603296</t>
+          <t>601138</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>华勤技术</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露华勤数据中心业务形成AI服务器、通用服务器、交换机等全栈产品组合，数据中心业务收入754.75亿元、同比增长51.93%；主板块保留AI服务器ODM，AI PC和终端ODM作为附属受益。</t>
+          <t>证据强：2025年报披露公司与全球头部客户协同下一代AI服务器及液冷技术，云服务商AI服务器收入同比大增，GPU与ASIC方案产品快速增长；删减“AI服务器机柜”重复行，机柜/液冷作为ODM系统能力纳入备注。</t>
         </is>
       </c>
       <c r="E279" s="6" t="inlineStr">
@@ -8583,22 +8583,22 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>算力服务器结构件</t>
+          <t>AI服务器ODM</t>
         </is>
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>002965</t>
+          <t>603296</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>祥鑫科技</t>
+          <t>华勤技术</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>证据中弱：2025年报披露公司在通信设备领域可供应通讯插箱、交换机箱、算力服务器等产品和服务，但汽车业务仍占收入主体且净利润下滑；主板块由AI服务器机柜收敛为算力服务器结构件，AI订单强度需继续验证。</t>
+          <t>证据强：2025年报披露华勤数据中心业务形成AI服务器、通用服务器、交换机等全栈产品组合，数据中心业务收入754.75亿元、同比增长51.93%；主板块保留AI服务器ODM，AI PC和终端ODM作为附属受益。</t>
         </is>
       </c>
       <c r="E280" s="6" t="inlineStr">
@@ -8610,22 +8610,22 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>智能算力产品及服务</t>
+          <t>算力服务器结构件</t>
         </is>
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>300857</t>
+          <t>002965</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>协创数据</t>
+          <t>祥鑫科技</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露智能算力产品及服务收入27.61亿元、同比增长1727.17%、占总收入22.57%，成为第二大收入支柱；原IDC标签不准确，改为智能算力产品及服务。</t>
+          <t>证据中弱：2025年报披露公司在通信设备领域可供应通讯插箱、交换机箱、算力服务器等产品和服务，但汽车业务仍占收入主体且净利润下滑；主板块由AI服务器机柜收敛为算力服务器结构件，AI订单强度需继续验证。</t>
         </is>
       </c>
       <c r="E281" s="6" t="inlineStr">
@@ -8637,22 +8637,22 @@
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>国产AI加速芯片</t>
+          <t>智能算力产品及服务</t>
         </is>
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>688256</t>
+          <t>300857</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>寒武纪</t>
+          <t>协创数据</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司云边端智能芯片及板卡矩阵，云端产品线面向服务器和数据中心AI处理，收入大增并首次全年盈利；删减“AI推理板卡”重复行，板卡是产品形态，主板块归入国产AI加速芯片。</t>
+          <t>证据强：2025年报披露智能算力产品及服务收入27.61亿元、同比增长1727.17%、占总收入22.57%，成为第二大收入支柱；原IDC标签不准确，改为智能算力产品及服务。</t>
         </is>
       </c>
       <c r="E282" s="6" t="inlineStr">
@@ -8664,22 +8664,22 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>国产CPU-DCU芯片</t>
+          <t>国产AI加速芯片</t>
         </is>
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>688041</t>
+          <t>688256</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>海光信息</t>
+          <t>寒武纪</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及公开资料显示海光坚持CPU+DCU双芯战略，DCU软件栈适配大模型训练推理并在多行业场景落地；删减“AI推理板卡”重复行，核心价值在国产高端处理器和DCU算力平台。</t>
+          <t>证据强：2025年报披露公司云边端智能芯片及板卡矩阵，云端产品线面向服务器和数据中心AI处理，收入大增并首次全年盈利；删减“AI推理板卡”重复行，板卡是产品形态，主板块归入国产AI加速芯片。</t>
         </is>
       </c>
       <c r="E283" s="6" t="inlineStr">
@@ -8691,22 +8691,22 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>国产GPU芯片</t>
+          <t>国产CPU-DCU芯片</t>
         </is>
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>300474</t>
+          <t>688041</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>景嘉微</t>
+          <t>海光信息</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司推进“高性能GPU+边端侧AI SoC芯片”双轮驱动，景宏系列智算模块及整机产品瞄准AI训练和推理；删减“AI推理板卡”重复行，当前仍以国产GPU芯片为主线，亏损和商业化规模是主要风险。</t>
+          <t>证据强：2025年报及公开资料显示海光坚持CPU+DCU双芯战略，DCU软件栈适配大模型训练推理并在多行业场景落地；删减“AI推理板卡”重复行，核心价值在国产高端处理器和DCU算力平台。</t>
         </is>
       </c>
       <c r="E284" s="6" t="inlineStr">
@@ -8718,22 +8718,22 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>AI推理芯片</t>
+          <t>国产GPU芯片</t>
         </is>
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>688343</t>
+          <t>300474</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>云天励飞</t>
+          <t>景嘉微</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司构建应用、算法、芯片全栈能力，自研AI推理芯片适配国产大模型、操作系统和推理框架，并推出大模型一体机；一体机为产品化形态，主板块保留AI推理芯片。</t>
+          <t>证据中：2025年报披露公司推进“高性能GPU+边端侧AI SoC芯片”双轮驱动，景宏系列智算模块及整机产品瞄准AI训练和推理；删减“AI推理板卡”重复行，当前仍以国产GPU芯片为主线，亏损和商业化规模是主要风险。</t>
         </is>
       </c>
       <c r="E285" s="6" t="inlineStr">
@@ -8745,22 +8745,22 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>智算网络设备</t>
+          <t>AI推理芯片</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>000938</t>
+          <t>688343</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>紫光股份</t>
+          <t>云天励飞</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>证据强：新华三深度覆盖云、网、安、算、存、端，但公司披露中国数据中心交换机份额居前，并在智算网络、800G/CPO交换机和AI算力基础设施上持续推进；删减AI存储、AI服务器ODM重复行，主板块保留最能体现差异化和份额优势的智算交换机。</t>
+          <t>证据中强：2025年报披露公司构建应用、算法、芯片全栈能力，自研AI推理芯片适配国产大模型、操作系统和推理框架，并推出大模型一体机；一体机为产品化形态，主板块保留AI推理芯片。</t>
         </is>
       </c>
       <c r="E286" s="6" t="inlineStr">
@@ -8777,17 +8777,17 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>301165</t>
+          <t>000938</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>锐捷网络</t>
+          <t>紫光股份</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI智算中心网络方案已服务中国移动、阿里、字节、百度、腾讯等训练/推理大模型场景，数据中心交换机订单加速交付；IDC数据显示中国数据中心交换机市占率第三。</t>
+          <t>证据强：新华三深度覆盖云、网、安、算、存、端，但公司披露中国数据中心交换机份额居前，并在智算网络、800G/CPO交换机和AI算力基础设施上持续推进；删减AI存储、AI服务器ODM重复行，主板块保留最能体现差异化和份额优势的智算交换机。</t>
         </is>
       </c>
       <c r="E287" s="6" t="inlineStr">
@@ -8804,17 +8804,17 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>000063</t>
+          <t>301165</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>中兴通讯</t>
+          <t>锐捷网络</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及公司新闻披露算力业务收入同比约150%，服务器及存储同比超200%，数据中心产品同比增长；公司以自研AI大容量交换芯片支撑智算超节点和万卡级智算中心，主板块从交换机扩展为智算网络设备。</t>
+          <t>证据强：2025年报披露AI智算中心网络方案已服务中国移动、阿里、字节、百度、腾讯等训练/推理大模型场景，数据中心交换机订单加速交付；IDC数据显示中国数据中心交换机市占率第三。</t>
         </is>
       </c>
       <c r="E288" s="6" t="inlineStr">
@@ -8826,22 +8826,22 @@
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>以太网交换芯片</t>
+          <t>智算网络设备</t>
         </is>
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>688702</t>
+          <t>000063</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>盛科通信-U</t>
+          <t>中兴通讯</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营以太网交换芯片及配套产品，交换芯片收入8.31亿元、占营收72.26%，交换机收入占比较低；删减“智算交换机”重复行，保留最能体现价值量的以太网交换芯片，风险是亏损扩大和高端产品放量节奏。</t>
+          <t>证据强：2025年报及公司新闻披露算力业务收入同比约150%，服务器及存储同比超200%，数据中心产品同比增长；公司以自研AI大容量交换芯片支撑智算超节点和万卡级智算中心，主板块从交换机扩展为智算网络设备。</t>
         </is>
       </c>
       <c r="E289" s="6" t="inlineStr">
@@ -8853,22 +8853,22 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>以太网PHY-交换芯片</t>
+          <t>以太网交换芯片</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>688515</t>
+          <t>688702</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>裕太微</t>
+          <t>盛科通信-U</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注高速有线通信芯片，网通PHY、交换机芯片、网卡芯片已规模量产，网通类产品销量约1.4亿颗，并向数据中心与基站等高价值场景延伸；AI数据中心直接收入仍需跟踪。</t>
+          <t>证据中强：2025年报披露公司主营以太网交换芯片及配套产品，交换芯片收入8.31亿元、占营收72.26%，交换机收入占比较低；删减“智算交换机”重复行，保留最能体现价值量的以太网交换芯片，风险是亏损扩大和高端产品放量节奏。</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
@@ -8880,30 +8880,34 @@
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>PCIe Switch</t>
+          <t>以太网PHY-交换芯片</t>
         </is>
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>688515</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>裕太微</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>GPU集群内PCIe Switch、NVSwitch和高端交换ASIC主要由NVIDIA、Broadcom、Microchip、Astera等海外厂商主导，A股不硬凑。</t>
-        </is>
-      </c>
-      <c r="E291" s="6" t="n"/>
+          <t>证据中：2025年报披露公司专注高速有线通信芯片，网通PHY、交换机芯片、网卡芯片已规模量产，网通类产品销量约1.4亿颗，并向数据中心与基站等高价值场景延伸；AI数据中心直接收入仍需跟踪。</t>
+        </is>
+      </c>
+      <c r="E291" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>BMC</t>
+          <t>PCIe Switch</t>
         </is>
       </c>
       <c r="B292" s="3" t="inlineStr">
@@ -8918,7 +8922,7 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>AI服务器BMC/远程管理芯片以海外和台湾厂商为主，A股目前缺成熟纯标的，先列系统级空白。</t>
+          <t>GPU集群内PCIe Switch、NVSwitch和高端交换ASIC主要由NVIDIA、Broadcom、Microchip、Astera等海外厂商主导，A股不硬凑。</t>
         </is>
       </c>
       <c r="E292" s="6" t="n"/>
@@ -8926,49 +8930,45 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>Edge BMC管理芯片</t>
+          <t>BMC</t>
         </is>
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>688595</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>芯海科技</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露面向边缘计算及服务器市场的轻量级edge BMC管理芯片已上市并量产销售，同时EC芯片在AI PC量产；保留BMC但改为Edge BMC管理芯片，风险是公司仍亏损且BMC收入规模未单列。</t>
-        </is>
-      </c>
-      <c r="E293" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>AI服务器BMC/远程管理芯片以海外和台湾厂商为主，A股目前缺成熟纯标的，先列系统级空白。</t>
+        </is>
+      </c>
+      <c r="E293" s="6" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>低抖动时钟源</t>
+          <t>Edge BMC管理芯片</t>
         </is>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>603738</t>
+          <t>688595</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>泰晶科技</t>
+          <t>芯海科技</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露公司开发面向AI数据中心基础设施的312.5MHz差分输出温补振荡器和低抖动可编程振荡器，满足AI数据中心、3.2T光模块、AI算力等需求；主板块保留低抖动时钟源。</t>
+          <t>证据中：2025年报摘要披露面向边缘计算及服务器市场的轻量级edge BMC管理芯片已上市并量产销售，同时EC芯片在AI PC量产；保留BMC但改为Edge BMC管理芯片，风险是公司仍亏损且BMC收入规模未单列。</t>
         </is>
       </c>
       <c r="E294" s="6" t="inlineStr">
@@ -8980,22 +8980,22 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>高频晶振</t>
+          <t>低抖动时钟源</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>300460</t>
+          <t>603738</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>惠伦晶体</t>
+          <t>泰晶科技</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>证据弱：2025半年报披露公司主营石英晶体元器件，高频产品和服务器等领域方案商认证具备基础支撑价值；但2025年仍亏损且未见明确AI服务器低抖动订单，主板块由低抖动时钟源降级为高频晶振观察。</t>
+          <t>证据中强：2025年报/半年报披露公司开发面向AI数据中心基础设施的312.5MHz差分输出温补振荡器和低抖动可编程振荡器，满足AI数据中心、3.2T光模块、AI算力等需求；主板块保留低抖动时钟源。</t>
         </is>
       </c>
       <c r="E295" s="6" t="inlineStr">
@@ -9007,22 +9007,22 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>IDC</t>
+          <t>高频晶振</t>
         </is>
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>600845</t>
+          <t>300460</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>宝信软件</t>
+          <t>惠伦晶体</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>工业软件和IDC双主业，宝之云IDC、华北基地、人工智能算力资源池等资产构成算力基础设施运营侧真实映射；DCIM不是公司最核心的AI受益解释。主板块由DCIM改为IDC，原IDC重复行合并删除。风险是钢铁行业软件需求承压、IDC资本开支和上架率、电力成本、AI算力资源池回报周期。证据A/B。</t>
+          <t>证据弱：2025半年报披露公司主营石英晶体元器件，高频产品和服务器等领域方案商认证具备基础支撑价值；但2025年仍亏损且未见明确AI服务器低抖动订单，主板块由低抖动时钟源降级为高频晶振观察。</t>
         </is>
       </c>
       <c r="E296" s="6" t="inlineStr">
@@ -9034,22 +9034,22 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>AIDC智算中心</t>
+          <t>IDC</t>
         </is>
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>300442</t>
+          <t>600845</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>宝信软件</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示AIDC收入25.1亿元、占总收入44.24%，新增交付算力规模220MW且含单体100MW智算中心；合并IDC/算力中心运维，主线改为AIDC智算中心。</t>
+          <t>工业软件和IDC双主业，宝之云IDC、华北基地、人工智能算力资源池等资产构成算力基础设施运营侧真实映射；DCIM不是公司最核心的AI受益解释。主板块由DCIM改为IDC，原IDC重复行合并删除。风险是钢铁行业软件需求承压、IDC资本开支和上架率、电力成本、AI算力资源池回报周期。证据A/B。</t>
         </is>
       </c>
       <c r="E297" s="6" t="inlineStr">
@@ -9061,22 +9061,22 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>IDC及算力租赁</t>
+          <t>AIDC智算中心</t>
         </is>
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>300738</t>
+          <t>300442</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>奥飞数据</t>
+          <t>润泽科技</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露业务为IDC及互联网综合服务，报告期新项目投产并继续推进算力租赁和相关设备销售；AI链受益来自机柜上架和算力需求，保留IDC及算力租赁。</t>
+          <t>证据强：2025年报显示AIDC收入25.1亿元、占总收入44.24%，新增交付算力规模220MW且含单体100MW智算中心；合并IDC/算力中心运维，主线改为AIDC智算中心。</t>
         </is>
       </c>
       <c r="E298" s="6" t="inlineStr">
@@ -9088,22 +9088,22 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>IDC云计算基础设施</t>
+          <t>IDC及算力租赁</t>
         </is>
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>300383</t>
+          <t>300738</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>光环新网</t>
+          <t>奥飞数据</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露主营仍是IDC及云计算，AI爆发带动数据中心与云计算需求，并与格灵深瞳合作AI+行业智算云；直接算力运营收入未充分拆分，保留IDC云计算基础设施。</t>
+          <t>证据中：2025年报披露业务为IDC及互联网综合服务，报告期新项目投产并继续推进算力租赁和相关设备销售；AI链受益来自机柜上架和算力需求，保留IDC及算力租赁。</t>
         </is>
       </c>
       <c r="E299" s="6" t="inlineStr">
@@ -9115,22 +9115,22 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>算力中心运维</t>
+          <t>IDC云计算基础设施</t>
         </is>
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>002929</t>
+          <t>300383</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>润建股份</t>
+          <t>光环新网</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露算力网络业务增长、算力中心管理运维和智算云服务推进，但AI及算力收入占比仍较小且归母净利下滑；保留算力中心运维并下调盈利确定性。</t>
+          <t>证据中：2025年报披露主营仍是IDC及云计算，AI爆发带动数据中心与云计算需求，并与格灵深瞳合作AI+行业智算云；直接算力运营收入未充分拆分，保留IDC云计算基础设施。</t>
         </is>
       </c>
       <c r="E300" s="6" t="inlineStr">
@@ -9142,22 +9142,22 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>算力设备交付运维</t>
+          <t>算力中心运维</t>
         </is>
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>301085</t>
+          <t>002929</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>亚康股份</t>
+          <t>润建股份</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露向富士康、英业达、华勤、浪潮等算力服务器制造商提供交付及售后维保，并从传统数据中心向AI智算中心运维升级；公司亏损，主线为算力设备交付运维。</t>
+          <t>证据中：2025年报披露算力网络业务增长、算力中心管理运维和智算云服务推进，但AI及算力收入占比仍较小且归母净利下滑；保留算力中心运维并下调盈利确定性。</t>
         </is>
       </c>
       <c r="E301" s="6" t="inlineStr">
@@ -9169,22 +9169,22 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>AI智能终端ODM</t>
+          <t>算力设备交付运维</t>
         </is>
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>603341</t>
+          <t>301085</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>龙旗科技</t>
+          <t>亚康股份</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露AI PC实现全平台产品设计与量产落地并获得全球头部客户订单，智能眼镜实现多场景、多品类规模化量产，AIoT业务覆盖智能手表/手环和智能眼镜；主板块从智能终端ODM细化为AI智能终端ODM。风险是手机/平板仍占大盘，新业务弹性需看AI PC、智能眼镜收入占比和毛利。</t>
+          <t>证据中：2025年报摘要披露向富士康、英业达、华勤、浪潮等算力服务器制造商提供交付及售后维保，并从传统数据中心向AI智算中心运维升级；公司亏损，主线为算力设备交付运维。</t>
         </is>
       </c>
       <c r="E302" s="6" t="inlineStr">
@@ -9196,22 +9196,22 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>端侧AI SoC</t>
+          <t>AI智能终端ODM</t>
         </is>
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>603893</t>
+          <t>603341</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>瑞芯微</t>
+          <t>龙旗科技</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/半年报披露智能应用处理器为核心收入来源，RK3588/RK3576等SoC和自研NPU支持端侧模型、AIoT多场景落地；主板块从“端侧AI处理器”规范为“端侧AI SoC”，跟踪高端SoC新品、客户导入和AIoT需求持续性。</t>
+          <t>证据中强：2025年报披露AI PC实现全平台产品设计与量产落地并获得全球头部客户订单，智能眼镜实现多场景、多品类规模化量产，AIoT业务覆盖智能手表/手环和智能眼镜；主板块从智能终端ODM细化为AI智能终端ODM。风险是手机/平板仍占大盘，新业务弹性需看AI PC、智能眼镜收入占比和毛利。</t>
         </is>
       </c>
       <c r="E303" s="6" t="inlineStr">
@@ -9228,17 +9228,17 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>300458</t>
+          <t>603893</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>全志科技</t>
+          <t>瑞芯微</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司实现CPU、GPU、NPU、DSP及RISC-V协处理器复杂异构芯片规模化量产，智能终端应用处理器是核心业务；删减AI眼镜应用处理器重复行，AI眼镜只是下游应用之一，主板块保留端侧AI SoC。</t>
+          <t>证据强：2025年报/半年报披露智能应用处理器为核心收入来源，RK3588/RK3576等SoC和自研NPU支持端侧模型、AIoT多场景落地；主板块从“端侧AI处理器”规范为“端侧AI SoC”，跟踪高端SoC新品、客户导入和AIoT需求持续性。</t>
         </is>
       </c>
       <c r="E304" s="6" t="inlineStr">
@@ -9255,17 +9255,17 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>688099</t>
+          <t>300458</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>晶晨股份</t>
+          <t>全志科技</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露智能多媒体及显示SoC仍是核心收入来源，AIoT SoC收入16.40亿元、同比增长8.50%，AIoT SoC集成NPU、DSP、视觉处理单元、ISP及编解码器并获Google EDLA认证；主板块从端侧AIoT SoC收敛为端侧AI SoC，跟踪端侧大模型适配、头部客户新品和经营现金流修复。</t>
+          <t>证据中强：2025年报披露公司实现CPU、GPU、NPU、DSP及RISC-V协处理器复杂异构芯片规模化量产，智能终端应用处理器是核心业务；删减AI眼镜应用处理器重复行，AI眼镜只是下游应用之一，主板块保留端侧AI SoC。</t>
         </is>
       </c>
       <c r="E305" s="6" t="inlineStr">
@@ -9277,22 +9277,22 @@
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜主控SoC</t>
+          <t>端侧AI SoC</t>
         </is>
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>688608</t>
+          <t>688099</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>恒玄科技</t>
+          <t>晶晨股份</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
+          <t>证据中强：2025年报披露智能多媒体及显示SoC仍是核心收入来源，AIoT SoC收入16.40亿元、同比增长8.50%，AIoT SoC集成NPU、DSP、视觉处理单元、ISP及编解码器并获Google EDLA认证；主板块从端侧AIoT SoC收敛为端侧AI SoC，跟踪端侧大模型适配、头部客户新品和经营现金流修复。</t>
         </is>
       </c>
       <c r="E306" s="6" t="inlineStr">
@@ -9304,22 +9304,22 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>智能穿戴SoC</t>
+          <t>AI眼镜主控SoC</t>
         </is>
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>688049</t>
+          <t>688608</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>炬芯科技</t>
+          <t>恒玄科技</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
+          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
         </is>
       </c>
       <c r="E307" s="6" t="inlineStr">
@@ -9331,22 +9331,22 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>端侧音视频SoC</t>
+          <t>智能穿戴SoC</t>
         </is>
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>688332</t>
+          <t>688049</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>中科蓝讯</t>
+          <t>炬芯科技</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
+          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
         </is>
       </c>
       <c r="E308" s="6" t="inlineStr">
@@ -9358,22 +9358,22 @@
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>端侧AI MCU</t>
+          <t>端侧音视频SoC</t>
         </is>
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>688018</t>
+          <t>688332</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>乐鑫科技</t>
+          <t>中科蓝讯</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
+          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
         </is>
       </c>
       <c r="E309" s="6" t="inlineStr">
@@ -9385,22 +9385,22 @@
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>端侧AI蜂窝模组</t>
+          <t>端侧AI MCU</t>
         </is>
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>603236</t>
+          <t>688018</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>移远通信</t>
+          <t>乐鑫科技</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
+          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
         </is>
       </c>
       <c r="E310" s="6" t="inlineStr">
@@ -9412,22 +9412,22 @@
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>高算力智能模组</t>
+          <t>端侧AI蜂窝模组</t>
         </is>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>002881</t>
+          <t>603236</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>美格智能</t>
+          <t>移远通信</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
+          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
         </is>
       </c>
       <c r="E311" s="6" t="inlineStr">
@@ -9439,22 +9439,22 @@
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>端侧AI模组</t>
+          <t>高算力智能模组</t>
         </is>
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>300638</t>
+          <t>002881</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>广和通</t>
+          <t>美格智能</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
+          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
         </is>
       </c>
       <c r="E312" s="6" t="inlineStr">
@@ -9466,22 +9466,22 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>AIOS端侧智能</t>
+          <t>端侧AI模组</t>
         </is>
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>300496</t>
+          <t>300638</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>中科创达</t>
+          <t>广和通</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
+          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
         </is>
       </c>
       <c r="E313" s="6" t="inlineStr">
@@ -9493,22 +9493,22 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>AR光波导</t>
+          <t>AIOS端侧智能</t>
         </is>
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>002273</t>
+          <t>300496</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>水晶光电</t>
+          <t>中科创达</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
+          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
         </is>
       </c>
       <c r="E314" s="6" t="inlineStr">
@@ -9520,22 +9520,22 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜光学模组</t>
+          <t>AR光波导</t>
         </is>
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>300433</t>
+          <t>002273</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>蓝思科技</t>
+          <t>水晶光电</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
+          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
         </is>
       </c>
       <c r="E315" s="6" t="inlineStr">
@@ -9547,22 +9547,22 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>AR投影光机</t>
+          <t>AI眼镜光学模组</t>
         </is>
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>688010</t>
+          <t>300433</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>福光股份</t>
+          <t>蓝思科技</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
+          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
         </is>
       </c>
       <c r="E316" s="6" t="inlineStr">
@@ -9574,22 +9574,22 @@
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>硅基OLED微显示</t>
+          <t>AR投影光机</t>
         </is>
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>688496</t>
+          <t>688010</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>清越科技</t>
+          <t>福光股份</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
+          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
         </is>
       </c>
       <c r="E317" s="6" t="inlineStr">
@@ -9601,22 +9601,22 @@
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED光机</t>
+          <t>硅基OLED微显示</t>
         </is>
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>300296</t>
+          <t>688496</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>利亚德</t>
+          <t>清越科技</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
+          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
         </is>
       </c>
       <c r="E318" s="6" t="inlineStr">
@@ -9628,22 +9628,22 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED微显示</t>
+          <t>AI眼镜MicroLED光机</t>
         </is>
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>300323</t>
+          <t>300296</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>京东方华灿</t>
+          <t>利亚德</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
+          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
         </is>
       </c>
       <c r="E319" s="6" t="inlineStr">
@@ -9655,22 +9655,22 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MicroLED芯片</t>
+          <t>AI眼镜MicroLED微显示</t>
         </is>
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>600703</t>
+          <t>300323</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>三安光电</t>
+          <t>京东方华灿</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
+          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
         </is>
       </c>
       <c r="E320" s="6" t="inlineStr">
@@ -9682,22 +9682,22 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>OLED-MicroLED显示</t>
+          <t>MicroLED芯片</t>
         </is>
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>002387</t>
+          <t>600703</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>维信诺</t>
+          <t>三安光电</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
+          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
         </is>
       </c>
       <c r="E321" s="6" t="inlineStr">
@@ -9709,22 +9709,22 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜CIS</t>
+          <t>OLED-MicroLED显示</t>
         </is>
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>688213</t>
+          <t>002387</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>思特威</t>
+          <t>维信诺</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
+          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
         </is>
       </c>
       <c r="E322" s="6" t="inlineStr">
@@ -9741,17 +9741,17 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>688728</t>
+          <t>688213</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>格科微</t>
+          <t>思特威</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
+          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
         </is>
       </c>
       <c r="E323" s="6" t="inlineStr">
@@ -9763,22 +9763,22 @@
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜视觉算法</t>
+          <t>AI眼镜CIS</t>
         </is>
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>688088</t>
+          <t>688728</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>虹软科技</t>
+          <t>格科微</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
+          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
         </is>
       </c>
       <c r="E324" s="6" t="inlineStr">
@@ -9790,22 +9790,22 @@
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜模拟芯片</t>
+          <t>AI眼镜视觉算法</t>
         </is>
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>688798</t>
+          <t>688088</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>艾为电子</t>
+          <t>虹软科技</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
+          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
         </is>
       </c>
       <c r="E325" s="6" t="inlineStr">
@@ -9817,22 +9817,22 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜声学传感器</t>
+          <t>AI眼镜模拟芯片</t>
         </is>
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>688286</t>
+          <t>688798</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>敏芯股份</t>
+          <t>艾为电子</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
+          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
         </is>
       </c>
       <c r="E326" s="6" t="inlineStr">
@@ -9844,22 +9844,22 @@
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>消费锂电池</t>
+          <t>AI眼镜声学传感器</t>
         </is>
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>688772</t>
+          <t>688286</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>珠海冠宇</t>
+          <t>敏芯股份</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
+          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
         </is>
       </c>
       <c r="E327" s="6" t="inlineStr">
@@ -9871,22 +9871,22 @@
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜电池</t>
+          <t>消费锂电池</t>
         </is>
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>001283</t>
+          <t>688772</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>豪鹏科技</t>
+          <t>珠海冠宇</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
+          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
         </is>
       </c>
       <c r="E328" s="6" t="inlineStr">
@@ -9898,22 +9898,22 @@
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜结构件</t>
+          <t>AI智能眼镜电池</t>
         </is>
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>300115</t>
+          <t>001283</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>长盈精密</t>
+          <t>豪鹏科技</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
+          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
         </is>
       </c>
       <c r="E329" s="6" t="inlineStr">
@@ -9925,22 +9925,22 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜整机</t>
+          <t>AI眼镜结构件</t>
         </is>
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>002241</t>
+          <t>300115</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>歌尔股份</t>
+          <t>长盈精密</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
+          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
         </is>
       </c>
       <c r="E330" s="6" t="inlineStr">
@@ -9952,22 +9952,22 @@
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>AI终端精密功能件</t>
+          <t>AI智能眼镜整机</t>
         </is>
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>002600</t>
+          <t>002241</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>领益智造</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
+          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
         </is>
       </c>
       <c r="E331" s="6" t="inlineStr">
@@ -9979,22 +9979,22 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>机器人3D视觉</t>
+          <t>AI终端精密功能件</t>
         </is>
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>688322</t>
+          <t>002600</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>奥比中光</t>
+          <t>领益智造</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
+          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
         </is>
       </c>
       <c r="E332" s="6" t="inlineStr">
@@ -10006,22 +10006,22 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>机器人力传感器</t>
+          <t>机器人3D视觉</t>
         </is>
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>603662</t>
+          <t>688322</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>柯力传感</t>
+          <t>奥比中光</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
+          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
         </is>
       </c>
       <c r="E333" s="6" t="inlineStr">
@@ -10038,17 +10038,17 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>301413</t>
+          <t>603662</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>安培龙</t>
+          <t>柯力传感</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
+          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
         </is>
       </c>
       <c r="E334" s="6" t="inlineStr">
@@ -10065,17 +10065,17 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>300354</t>
+          <t>301413</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>东华测试</t>
+          <t>安培龙</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
+          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
         </is>
       </c>
       <c r="E335" s="6" t="inlineStr">
@@ -10087,22 +10087,22 @@
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>机器人电子皮肤</t>
+          <t>机器人力传感器</t>
         </is>
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>300007</t>
+          <t>300354</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>汉威科技</t>
+          <t>东华测试</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
+          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
         </is>
       </c>
       <c r="E336" s="6" t="inlineStr">
@@ -10114,22 +10114,22 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>机器人谐波减速器</t>
+          <t>机器人电子皮肤</t>
         </is>
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>688017</t>
+          <t>300007</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>绿的谐波</t>
+          <t>汉威科技</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
+          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
         </is>
       </c>
       <c r="E337" s="6" t="inlineStr">
@@ -10141,22 +10141,22 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>机器人精密减速器</t>
+          <t>机器人谐波减速器</t>
         </is>
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>002896</t>
+          <t>688017</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>中大力德</t>
+          <t>绿的谐波</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
+          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
         </is>
       </c>
       <c r="E338" s="6" t="inlineStr">
@@ -10173,17 +10173,17 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>002472</t>
+          <t>002896</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>双环传动</t>
+          <t>中大力德</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
+          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
         </is>
       </c>
       <c r="E339" s="6" t="inlineStr">
@@ -10195,22 +10195,22 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>行星滚柱丝杠</t>
+          <t>机器人精密减速器</t>
         </is>
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>603667</t>
+          <t>002472</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>五洲新春</t>
+          <t>双环传动</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
+          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
         </is>
       </c>
       <c r="E340" s="6" t="inlineStr">
@@ -10227,17 +10227,17 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>601100</t>
+          <t>603667</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>恒立液压</t>
+          <t>五洲新春</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
+          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
         </is>
       </c>
       <c r="E341" s="6" t="inlineStr">
@@ -10254,17 +10254,17 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>688678</t>
+          <t>601100</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>福立旺</t>
+          <t>恒立液压</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
+          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
         </is>
       </c>
       <c r="E342" s="6" t="inlineStr">
@@ -10281,17 +10281,17 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>603009</t>
+          <t>688678</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>北特科技</t>
+          <t>福立旺</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
+          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
         </is>
       </c>
       <c r="E343" s="6" t="inlineStr">
@@ -10303,22 +10303,22 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>机器人执行器</t>
+          <t>行星滚柱丝杠</t>
         </is>
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>601689</t>
+          <t>603009</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>拓普集团</t>
+          <t>北特科技</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
+          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
         </is>
       </c>
       <c r="E344" s="6" t="inlineStr">
@@ -10330,22 +10330,22 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>机器人伺服驱动</t>
+          <t>机器人执行器</t>
         </is>
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>300124</t>
+          <t>601689</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>汇川技术</t>
+          <t>拓普集团</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
+          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
         </is>
       </c>
       <c r="E345" s="6" t="inlineStr">
@@ -10357,22 +10357,22 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>机器人驱控系统</t>
+          <t>机器人伺服驱动</t>
         </is>
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>002979</t>
+          <t>300124</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>雷赛智能</t>
+          <t>汇川技术</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
+          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
         </is>
       </c>
       <c r="E346" s="6" t="inlineStr">
@@ -10384,22 +10384,22 @@
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>空心杯电机</t>
+          <t>机器人驱控系统</t>
         </is>
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>603728</t>
+          <t>002979</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>鸣志电器</t>
+          <t>雷赛智能</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
+          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
         </is>
       </c>
       <c r="E347" s="6" t="inlineStr">
@@ -10411,22 +10411,22 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>行业大模型+Agent平台</t>
+          <t>空心杯电机</t>
         </is>
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>300229</t>
+          <t>603728</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>拓尔思</t>
+          <t>鸣志电器</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
+          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
         </is>
       </c>
       <c r="E348" s="6" t="inlineStr">
@@ -10438,22 +10438,22 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>行业大模型训推一体</t>
+          <t>行业大模型+Agent平台</t>
         </is>
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>688327</t>
+          <t>300229</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>云从科技</t>
+          <t>拓尔思</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
+          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
         </is>
       </c>
       <c r="E349" s="6" t="inlineStr">
@@ -10465,22 +10465,22 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>国产算力大模型底座</t>
+          <t>行业大模型训推一体</t>
         </is>
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>002230</t>
+          <t>688327</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>科大讯飞</t>
+          <t>云从科技</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
         </is>
       </c>
       <c r="E350" s="6" t="inlineStr">
@@ -10492,22 +10492,22 @@
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>企业AI平台</t>
+          <t>国产算力大模型底座</t>
         </is>
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>600588</t>
+          <t>002230</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>用友网络</t>
+          <t>科大讯飞</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
+          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
         </is>
       </c>
       <c r="E351" s="6" t="inlineStr">
@@ -10519,22 +10519,22 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>企业级AI应用平台</t>
+          <t>企业AI平台</t>
         </is>
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>300170</t>
+          <t>600588</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>汉得信息</t>
+          <t>用友网络</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
+          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
         </is>
       </c>
       <c r="E352" s="6" t="inlineStr">
@@ -10546,22 +10546,22 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>行业AI智能体平台</t>
+          <t>企业级AI应用平台</t>
         </is>
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>301236</t>
+          <t>300170</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>软通动力</t>
+          <t>汉得信息</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
         </is>
       </c>
       <c r="E353" s="6" t="inlineStr">
@@ -10573,22 +10573,22 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>制造业AI智能体平台</t>
+          <t>行业AI智能体平台</t>
         </is>
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>300378</t>
+          <t>301236</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>鼎捷数智</t>
+          <t>软通动力</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
         </is>
       </c>
       <c r="E354" s="6" t="inlineStr">
@@ -10600,22 +10600,22 @@
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>行业AI交付</t>
+          <t>制造业AI智能体平台</t>
         </is>
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>002649</t>
+          <t>300378</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>博彦科技</t>
+          <t>鼎捷数智</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
+          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
         </is>
       </c>
       <c r="E355" s="6" t="inlineStr">
@@ -10627,22 +10627,22 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>AI数据基础设施软件</t>
+          <t>行业AI交付</t>
         </is>
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>688031</t>
+          <t>002649</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>星环科技</t>
+          <t>博彦科技</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
         </is>
       </c>
       <c r="E356" s="6" t="inlineStr">
@@ -10654,22 +10654,22 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>向量数据库</t>
+          <t>AI数据基础设施软件</t>
         </is>
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>603138</t>
+          <t>688031</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>海量数据</t>
+          <t>星环科技</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
+          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
         </is>
       </c>
       <c r="E357" s="6" t="inlineStr">
@@ -10681,22 +10681,22 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>AI数据库</t>
+          <t>向量数据库</t>
         </is>
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>688692</t>
+          <t>603138</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>达梦数据</t>
+          <t>海量数据</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
+          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
         </is>
       </c>
       <c r="E358" s="6" t="inlineStr">
@@ -10708,22 +10708,22 @@
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>多模态训练数据</t>
+          <t>AI数据库</t>
         </is>
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>688787</t>
+          <t>688692</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>海天瑞声</t>
+          <t>达梦数据</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
+          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
         </is>
       </c>
       <c r="E359" s="6" t="inlineStr">
@@ -10735,22 +10735,22 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>中文数据语料</t>
+          <t>多模态训练数据</t>
         </is>
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>688228</t>
+          <t>688787</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>开普云</t>
+          <t>海天瑞声</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
+          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
         </is>
       </c>
       <c r="E360" s="6" t="inlineStr">
@@ -10762,22 +10762,22 @@
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>AI安全</t>
+          <t>中文数据语料</t>
         </is>
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>002439</t>
+          <t>688228</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>启明星辰</t>
+          <t>开普云</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
+          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
         </is>
       </c>
       <c r="E361" s="6" t="inlineStr">
@@ -10794,17 +10794,17 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>300454</t>
+          <t>002439</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>深信服</t>
+          <t>启明星辰</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
+          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
         </is>
       </c>
       <c r="E362" s="6" t="inlineStr">
@@ -10821,17 +10821,17 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>688561</t>
+          <t>300454</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>奇安信</t>
+          <t>深信服</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
+          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
         </is>
       </c>
       <c r="E363" s="6" t="inlineStr">
@@ -10848,17 +10848,17 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>688023</t>
+          <t>688561</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>安恒信息</t>
+          <t>奇安信</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
+          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
         </is>
       </c>
       <c r="E364" s="6" t="inlineStr">
@@ -10875,17 +10875,17 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>601360</t>
+          <t>688023</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>三六零</t>
+          <t>安恒信息</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
+          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
         </is>
       </c>
       <c r="E365" s="6" t="inlineStr">
@@ -10902,17 +10902,17 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>300369</t>
+          <t>601360</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>绿盟科技</t>
+          <t>三六零</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
+          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
         </is>
       </c>
       <c r="E366" s="6" t="inlineStr">
@@ -10924,22 +10924,22 @@
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>AI办公Agent</t>
+          <t>AI安全</t>
         </is>
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>688111</t>
+          <t>300369</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>金山办公</t>
+          <t>绿盟科技</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
+          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
         </is>
       </c>
       <c r="E367" s="6" t="inlineStr">
@@ -10951,22 +10951,22 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>PDF文档AI</t>
+          <t>AI办公Agent</t>
         </is>
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>688095</t>
+          <t>688111</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>福昕软件</t>
+          <t>金山办公</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
+          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
         </is>
       </c>
       <c r="E368" s="6" t="inlineStr">
@@ -10978,22 +10978,22 @@
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>问财金融投研AI</t>
+          <t>PDF文档AI</t>
         </is>
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>300033</t>
+          <t>688095</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>同花顺</t>
+          <t>福昕软件</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
+          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
         </is>
       </c>
       <c r="E369" s="6" t="inlineStr">
@@ -11005,22 +11005,22 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>保险IT AI应用</t>
+          <t>问财金融投研AI</t>
         </is>
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>603927</t>
+          <t>300033</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>中科软</t>
+          <t>同花顺</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
+          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
         </is>
       </c>
       <c r="E370" s="6" t="inlineStr">
@@ -11032,22 +11032,22 @@
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>AI多媒体创作平台</t>
+          <t>保险IT AI应用</t>
         </is>
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>300624</t>
+          <t>603927</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>万兴科技</t>
+          <t>中科软</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
+          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
         </is>
       </c>
       <c r="E371" s="6" t="inlineStr">
@@ -11059,22 +11059,22 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>AI+CAx工业设计软件</t>
+          <t>AI多媒体创作平台</t>
         </is>
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>688083</t>
+          <t>300624</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>中望软件</t>
+          <t>万兴科技</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
+          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
         </is>
       </c>
       <c r="E372" s="6" t="inlineStr">
@@ -11086,22 +11086,22 @@
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>物理AI工业仿真</t>
+          <t>AI+CAx工业设计软件</t>
         </is>
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>688507</t>
+          <t>688083</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>索辰科技</t>
+          <t>中望软件</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
+          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
         </is>
       </c>
       <c r="E373" s="6" t="inlineStr">
@@ -11113,22 +11113,22 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>流程工业AI</t>
+          <t>物理AI工业仿真</t>
         </is>
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>688777</t>
+          <t>688507</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>中控技术</t>
+          <t>索辰科技</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
+          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
         </is>
       </c>
       <c r="E374" s="6" t="inlineStr">
@@ -11140,22 +11140,22 @@
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>激光加工AI工艺优化</t>
+          <t>流程工业AI</t>
         </is>
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>688188</t>
+          <t>688777</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>柏楚电子</t>
+          <t>中控技术</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
+          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
         </is>
       </c>
       <c r="E375" s="6" t="inlineStr">
@@ -11167,22 +11167,22 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>AI分子砌块设计</t>
+          <t>激光加工AI工艺优化</t>
         </is>
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>300725</t>
+          <t>688188</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>药石科技</t>
+          <t>柏楚电子</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
+          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
         </is>
       </c>
       <c r="E376" s="6" t="inlineStr">
@@ -11194,22 +11194,22 @@
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>AI片段分子库</t>
+          <t>AI分子砌块设计</t>
         </is>
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>688131</t>
+          <t>300725</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>皓元医药</t>
+          <t>药石科技</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
+          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
         </is>
       </c>
       <c r="E377" s="6" t="inlineStr">
@@ -11221,22 +11221,22 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>AI药物发现</t>
+          <t>AI片段分子库</t>
         </is>
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>688222</t>
+          <t>688131</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>成都先导</t>
+          <t>皓元医药</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
+          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
         </is>
       </c>
       <c r="E378" s="6" t="inlineStr">
@@ -11248,22 +11248,22 @@
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>AI辅助药物设计</t>
+          <t>AI药物发现</t>
         </is>
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>301230</t>
+          <t>688222</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>泓博医药</t>
+          <t>成都先导</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
+          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
         </is>
       </c>
       <c r="E379" s="6" t="inlineStr">
@@ -11275,22 +11275,22 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>AI患者追踪系统</t>
+          <t>AI辅助药物设计</t>
         </is>
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>300451</t>
+          <t>301230</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>创业慧康</t>
+          <t>泓博医药</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
+          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
         </is>
       </c>
       <c r="E380" s="6" t="inlineStr">
@@ -11302,22 +11302,22 @@
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>AI医学影像设备</t>
+          <t>AI患者追踪系统</t>
         </is>
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>688271</t>
+          <t>300451</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>联影医疗</t>
+          <t>创业慧康</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
+          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
         </is>
       </c>
       <c r="E381" s="6" t="inlineStr">
@@ -11329,22 +11329,22 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>医疗信息化大模型</t>
+          <t>AI医学影像设备</t>
         </is>
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>300253</t>
+          <t>688271</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>卫宁健康</t>
+          <t>联影医疗</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
         </is>
       </c>
       <c r="E382" s="6" t="inlineStr">
@@ -11356,25 +11356,52 @@
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
+          <t>医疗信息化大模型</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>300253</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>卫宁健康</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+        </is>
+      </c>
+      <c r="E383" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
           <t>医学检验AI服务</t>
         </is>
       </c>
-      <c r="B383" s="3" t="inlineStr">
+      <c r="B384" s="3" t="inlineStr">
         <is>
           <t>603108</t>
         </is>
       </c>
-      <c r="C383" s="2" t="inlineStr">
+      <c r="C384" s="2" t="inlineStr">
         <is>
           <t>润达医疗</t>
         </is>
       </c>
-      <c r="D383" s="2" t="inlineStr">
+      <c r="D384" s="2" t="inlineStr">
         <is>
           <t>证据中强但业绩弱：2025年报披露公司推出大模型产品CDx良医晓慧，覆盖数据基座、医生助理和健康智能体，已在华西、南方、齐鲁等医院落地；核心仍是IVD流通/实验室服务，主板块由IVD检验AI细化为医学检验AI服务。</t>
         </is>
       </c>
-      <c r="E383" s="6" t="inlineStr">
+      <c r="E384" s="6" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>

</xml_diff>

<commit_message>
docs: update asia components research records
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1089,7 +1089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E384"/>
+  <dimension ref="A1:E385"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3180,12 +3180,12 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>高频高速覆铜板主线，AI服务器/光模块用高速板材料明确，M8/M9/M10升级看客户认证、订单能见度和涨价传导；封装基板材料并入备注，不再单列主板块。证据B。</t>
+          <t>高频高速覆铜板主线，AI服务器/光模块用高速板材料明确，M8/M9/M10升级看客户认证、订单能见度和涨价传导；封装基板材料并入备注，不再单列主板块。证据B。2026-06-16 JPM补充：报告提示HPC CCL/PCB TAM由AI server、常规server、LEO共同推升，CCL TAM可按2.5-3倍近似外推PCB TAM，M9升级和载板用Q glass是新增验证方向；仍按B级卖方估算处理，需看分产品lead time、涨价、客户认证和收入毛利。</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -3207,12 +3207,12 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>大陆CCL龙头，高速覆铜板、封装材料和客户覆盖最完整，是AI服务器高速PCB与M9/M10材料升级的稳健映射；主板块保留高端高速CCL，封装基板材料放备注，风险是周期、价格传导和高端占比。证据A/B。</t>
+          <t>大陆CCL龙头，高速覆铜板、封装材料和客户覆盖最完整，是AI服务器高速PCB与M9/M10材料升级的稳健映射；主板块保留高端高速CCL，封装基板材料放备注，风险是周期、价格传导和高端占比。证据A/B。2026-06-16 JPM补充：报告强化M8/M9高端CCL、HPC CCL与载板用CCL/Q glass需求，支持高端高速CCL soft_bottleneck+；但不能替代公司分产品订单、涨价和客户锁料证据。</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -3288,12 +3288,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>高速通信/AI服务器PCB主线，数据中心交换机、服务器、加速卡等高多层高速板客户和产品验证最直接；主板块保留AI服务器高速PCB，风险是大客户节奏、毛利年降和扩产良率。证据A。</t>
+          <t>高速通信/AI服务器PCB主线，数据中心交换机、服务器、加速卡等高多层高速板客户和产品验证最直接；主板块保留AI服务器高速PCB，风险是大客户节奏、毛利年降和扩产良率。证据A。2026-06-16 JPM补充：报告强调AI switch层数提升、HDI良率下降和M9升级可能使高层高速PCB供给落后需求，强化需求侧和复杂度证据；仍不证明具体客户订单或交期失控。</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -3315,12 +3315,12 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>PCB综合龙头，通信、数据中心和封装基板平台完整，AI服务器/高速互连PCB与FC-BGA/BT载板能力共振；主板块保留AI服务器高速PCB，封装基板行并入备注，不再单列，风险是收入占比和客户放量节奏。证据A/B。</t>
+          <t>PCB综合龙头，AI服务器/高速互连PCB与FC-BGA/BT载板能力共振；2026-06-16 ABF/IC载板复核后定位为“基本面质量锚”：深南电路具备数据中心PCB、封装基板平台和FC-BGA研发/打样能力，但不能直接写成NVIDIA/AMD高端GPU ABF载板订单。主板块保留AI服务器高速PCB，ABF/IC载板放备注跟踪，风险是封装基板收入占比、24层及以上进度、客户放量和毛利兑现。证据A/B。2026-06-16 JPM补充：报告估算IC载板UTR在2027e超过100%、AI server &amp; switch面积需求2028e占比75%，强化FC-BGA/ABF独立跟踪；深南仍需24层以上FC-BGA进展、大客户订单、收入和毛利验证。</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -3342,12 +3342,12 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>高多层PCB、HDI和AI服务器/交换机PCB是最直接主线，年报披露AI服务器相关HDI及18层以上多层板高景气，并强调深度绑定国际头部客户；主板块保留AI服务器高速PCB，风险是大客户集中、扩产良率和海外交付节奏。证据A/B。</t>
+          <t>高多层PCB、HDI和AI服务器/交换机PCB是最直接主线，年报披露AI服务器相关HDI及18层以上多层板高景气，并强调深度绑定国际头部客户；主板块保留AI服务器高速PCB，风险是大客户集中、扩产良率和海外交付节奏。证据A/B。2026-06-16 JPM补充：报告从AI switch、midplane/HDI和高层PCB良率角度强化AI PCB价值量与制造难度，支持胜宏高层高速板需求侧；风险仍是扩产良率、客户集中和毛利年降。</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -3369,12 +3369,12 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>AI服务器、OAM、UBB等高端PCB已大规模量产，2025年AI算力相关产品同比高增，是PCB环节纯度较高的标的；主板块保留AI服务器高速PCB，BT载板并入备注后不单列，风险是客户集中、产能爬坡和高端良率。证据A。</t>
+          <t>AI服务器、OAM、UBB等高端PCB已大规模量产，2025年AI算力相关产品同比高增，是PCB环节纯度较高的标的；主板块保留AI服务器高速PCB，BT载板并入备注后不单列，风险是客户集中、产能爬坡和高端良率。证据A。2026-06-16 JPM补充：报告强化AI server/switch PCB复杂度与高端CCL需求，对生益电子的AI服务器、OAM、UBB等高端PCB形成需求侧佐证；仍需跟踪客户、毛利和产能爬坡。</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -4202,12 +4202,12 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>电力电子平台，2025年报披露数据中心通用及AI服务器电源和系统产品拓展顺利，并聚焦AI算力基础设施供电系统；网络电源可支持通信、交换机、通用服务器和AI服务器场景。主板块保留数据中心电源，风险是AI电源研发投入压制利润、海外客户导入节奏和800VDC/BBU/Power Shelf规模收入验证。证据A/B。</t>
+          <t>电力电子平台，2026-06-16 800VDC复核后定位为“watch+ / catalyst_watch”：NVIDIA官方800VDC生态中可确认位于Power system components，公司年报/IR有推荐提供商、800VDC/SST/Sidecar/Power Shelf产品体系、小批量送测/试产和部分北美项目线索；但不能证明NVIDIA或Google直采订单。主板块保留数据中心电源，风险是AI电源研发投入、800VDC规模收入、订单金额、收入占比、毛利率和交付节奏兑现。证据A/B/C。</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核</t>
         </is>
       </c>
     </row>
@@ -5228,12 +5228,12 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>电子陶瓷材料平台，年报披露MLCC需求增长并继续突破超高容大尺寸产品、加深服务器等客户合作；光通信陶瓷插芯、MT插芯和陶瓷管壳受数据中心光器件需求带动，但相对MLCC主业降级为备注。主板块改为MLCC，风险是高容MLCC客户认证、价格竞争和光通信小件占比。证据A/B。</t>
+          <t>电子陶瓷材料平台，2026-06-16 MLCC复核后定位为AI server高端MLCC“main_candidate / 主受益候选”：年报披露数据中心领域多尺寸高容MLCC和48V电源系统高容MLCC，2026Q1盈利质量较强，光通信陶瓷件也有增量。风险是未披露AI server客户名单、具体高端MLCC ASP涨价、AI server收入拆分，估值已反映部分景气。证据A/B。2026-06-16 JPM补充：报告估算AI server MLCC TAM 150%+ CAGR，并指出高端MLCC产能消耗会挤压低阶/中阶供给；三环仍需用高容/高压/高可靠MLCC客户、ASP、收入占比和毛利率验证。</t>
         </is>
       </c>
       <c r="E154" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -5255,12 +5255,12 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露新能源汽车、AI算力、智能机器人等赛道扩容，公司推动MLCC向极限高容突破，并提到AI算力等领域应用；但公司仍属综合被动元件平台，AI服务器客户和收入弹性需继续验证。</t>
+          <t>高端MLCC国产替代标的，2026-06-16 MLCC复核后定位为“watch+ / event_trade”：公司披露极限高容MLCC应用于AI服务器等领域，多个MLCC产品完成客户编码认定并批量交付，但已明确目前尚未直接供货英伟达。交易弹性高于基本面确定性，需跟踪AI服务器MLCC批量规模、涨价执行、客户编码数量和净利率改善。证据A/B。2026-06-16 JPM补充：报告强化AI server高端MLCC需求和低阶供给挤压，但海外锚主要是YAGEO/Murata/Samsung；风华仍按watch+ / event_trade处理，需验证AI服务器MLCC批量规模、涨价执行和客户编码。</t>
         </is>
       </c>
       <c r="E155" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -5903,12 +5903,12 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>证据中强：IC封装基板收入高增，FCBGA项目面向服务器、AI芯片、交换机晶片等应用，正在提升高密植球大尺寸FCBGA能力；删减BT载板、IC测试板重复行，保留最能解释AI弹性的FC-BGA载板，风险是FCBGA尚未大批量生产且毛利仍承压。</t>
+          <t>证据中强：IC封装基板收入高增，FCBGA/ABF项目面向服务器、AI芯片、交换机晶片等应用并处小批量生产/客户导入阶段；2026-06-16 ABF复核后定位为“watch+ / event_trade_option”，更像订单突破期权而非当前基本面主受益。风险是大批量量产取决于客户进展和供应商管理策略，FCBGA过去仍拖累利润，需跟踪客户层级、单季收入和毛利改善。证据A/B。2026-06-16 JPM补充：报告估算载板UTR在2027e超过100%，AI server &amp; switch面积需求从2024年2,448 bn mm2升至2028e 21,522 bn mm2，占比升至75%；兴森仍是FC-BGA/ABF订单突破期权，需大客户、量产、收入和毛利验证。</t>
         </is>
       </c>
       <c r="E179" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -7056,12 +7056,12 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/公开资料显示公司已形成测试机、分选机、探针台、AOI等平台型产品矩阵，测试机成为核心收入来源，AI芯片复杂度提升、存储扩产和国产替代共同拉动高端测试设备需求；合并并删减“半导体测试分选机”重复行。</t>
+          <t>证据强：2025年报/公开资料显示公司已形成测试机、分选机、探针台、AOI等平台型产品矩阵，测试机成为核心收入来源，AI芯片复杂度提升、存储扩产和国产替代共同拉动高端测试设备需求；合并并删减“半导体测试分选机”重复行。2026-06-16 JPM补充：报告把GPU FT/SLT测试时间延长、TDP提升列为测试设备需求驱动，海外锚为Chroma；长川受益需验证高端SoC/SLT平台订单和AI客户收入，不泛化为所有测试机。</t>
         </is>
       </c>
       <c r="E222" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -7149,49 +7149,49 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>半导体测试探针</t>
+          <t>AI系统级测试设备</t>
         </is>
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>688661</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>和林微纳</t>
+          <t>暂无成熟A股纯标的（海外锚：致茂电子 2360.TW）</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/公开资料显示半导体测试探针业务成为增长引擎，收入同比高增并带动扭亏；公开证据更直接指向测试探针平台，HBM专用探针客户和收入未充分披露，故将“HBM测试探针”降级为半导体测试探针。</t>
+          <t>J.P. Morgan Asia Components 2026-06 中文整理版把Chroma的SLT、光通信/CPO、数据中心电源测试标注为三条100%+ CAGR方向；A股映射需拆到长川科技、华峰测控、华兴源创、伟测科技、精智达等子环节逐项验证，当前仅作new_watch，不等同普通半导体测试设备受益。证据B。</t>
         </is>
       </c>
       <c r="E226" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>新增；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>晶圆探针台</t>
+          <t>半导体测试探针</t>
         </is>
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>301629</t>
+          <t>688661</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>矽电股份</t>
+          <t>和林微纳</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司是中国大陆首家实现12英寸晶圆探针台产业化应用的厂商，产品面向SOC、Memory、CIS、功率器件等测试领域；AI/HBM是行业需求驱动而非已披露专用探针收入，原“HBM测试探针”修正为晶圆探针台。</t>
+          <t>证据中强：2025年报/公开资料显示半导体测试探针业务成为增长引擎，收入同比高增并带动扭亏；公开证据更直接指向测试探针平台，HBM专用探针客户和收入未充分披露，故将“HBM测试探针”降级为半导体测试探针。</t>
         </is>
       </c>
       <c r="E227" s="6" t="inlineStr">
@@ -7203,22 +7203,22 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>半导体测试分选设备</t>
+          <t>晶圆探针台</t>
         </is>
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>603061</t>
+          <t>301629</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>金海通</t>
+          <t>矽电股份</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司专注半导体芯片测试设备，三温测试分选机及大平台超多工位测试分选机需求持续增长、产品销量提升；AI算力芯片和先进封装属于复杂测试应用场景，主板块保留半导体测试分选机。</t>
+          <t>证据强：2025年报披露公司是中国大陆首家实现12英寸晶圆探针台产业化应用的厂商，产品面向SOC、Memory、CIS、功率器件等测试领域；AI/HBM是行业需求驱动而非已披露专用探针收入，原“HBM测试探针”修正为晶圆探针台。</t>
         </is>
       </c>
       <c r="E228" s="6" t="inlineStr">
@@ -7235,17 +7235,17 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>688328</t>
+          <t>603061</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>深科达</t>
+          <t>金海通</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/公告显示公司半导体设备业务增长，转塔式和平移式测试分选机实现批量订单交付，子公司深科达半导体贡献利润；未见TCB热压键合为核心收入，故由TCB修正为半导体测试分选设备。</t>
+          <t>证据强：2025年报披露公司专注半导体芯片测试设备，三温测试分选机及大平台超多工位测试分选机需求持续增长、产品销量提升；AI算力芯片和先进封装属于复杂测试应用场景，主板块保留半导体测试分选机。</t>
         </is>
       </c>
       <c r="E229" s="6" t="inlineStr">
@@ -7257,22 +7257,22 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>半导体检测量测设备</t>
+          <t>半导体测试分选设备</t>
         </is>
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>688361</t>
+          <t>688328</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>中科飞测</t>
+          <t>深科达</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露检测设备和量测设备收入增长，暗场纳米图形晶圆缺陷检测、无图形晶圆缺陷检测、套刻精度量测等产品贡献提升，并拓展电子束/X光技术；先进封装X-Ray作为能力补充并入备注，删除重复行。</t>
+          <t>证据中：2025年报/公告显示公司半导体设备业务增长，转塔式和平移式测试分选机实现批量订单交付，子公司深科达半导体贡献利润；未见TCB热压键合为核心收入，故由TCB修正为半导体测试分选设备。</t>
         </is>
       </c>
       <c r="E230" s="6" t="inlineStr">
@@ -7284,22 +7284,22 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>半导体测试服务</t>
+          <t>半导体检测量测设备</t>
         </is>
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>688135</t>
+          <t>688361</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>利扬芯片</t>
+          <t>中科飞测</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司主业为集成电路测试方案开发、晶圆测试和成品测试服务，营收创新高且亏损收窄，增长受高算力、存储、汽车电子等芯片测试需求和新客户/新产品导入带动；AI链条为后道测试服务弹性，客户与AI芯片收入未单列。</t>
+          <t>证据强：2025年报披露检测设备和量测设备收入增长，暗场纳米图形晶圆缺陷检测、无图形晶圆缺陷检测、套刻精度量测等产品贡献提升，并拓展电子束/X光技术；先进封装X-Ray作为能力补充并入备注，删除重复行。</t>
         </is>
       </c>
       <c r="E231" s="6" t="inlineStr">
@@ -7316,17 +7316,17 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>430139</t>
+          <t>688135</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>华岭股份</t>
+          <t>利扬芯片</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报显示测试服务仍为核心收入来源，并建设高算力应用芯片开放式测试创新服务平台；但公司2025年亏损扩大，AI/高算力测试仍处研发和客户拓展阶段，主线保留半导体测试服务，备注降级AI兑现强度。</t>
+          <t>证据中强：2025年报显示公司主业为集成电路测试方案开发、晶圆测试和成品测试服务，营收创新高且亏损收窄，增长受高算力、存储、汽车电子等芯片测试需求和新客户/新产品导入带动；AI链条为后道测试服务弹性，客户与AI芯片收入未单列。</t>
         </is>
       </c>
       <c r="E232" s="6" t="inlineStr">
@@ -7343,17 +7343,17 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>688372</t>
+          <t>430139</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>伟测科技</t>
+          <t>华岭股份</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报明确公司聚焦中高端晶圆及成品测试，拓展高算力产品测试，服务CPU/GPU/AI/FPGA、SoC/Chiplet/SiP等测试需求，并披露TSV工艺高性能AI产品整体测试方案研发；主板块由泛半导体测试收敛为高算力芯片测试服务。</t>
+          <t>证据中：2025年报显示测试服务仍为核心收入来源，并建设高算力应用芯片开放式测试创新服务平台；但公司2025年亏损扩大，AI/高算力测试仍处研发和客户拓展阶段，主线保留半导体测试服务，备注降级AI兑现强度。</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
@@ -7365,22 +7365,22 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>存储芯片测试设备</t>
+          <t>半导体测试服务</t>
         </is>
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>688627</t>
+          <t>688372</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>精智达</t>
+          <t>伟测科技</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/公开资料显示半导体存储测试设备业务快速放量，并签订两笔约3.2亿元级半导体重大订单；公司推进高速FT测试机、老化测试修复设备、探针卡及HBM测试设备研发，HBM BI属于未来强化方向，主板块收敛为存储芯片测试设备。</t>
+          <t>证据强：2025年报明确公司聚焦中高端晶圆及成品测试，拓展高算力产品测试，服务CPU/GPU/AI/FPGA、SoC/Chiplet/SiP等测试需求，并披露TSV工艺高性能AI产品整体测试方案研发；主板块由泛半导体测试收敛为高算力芯片测试服务。</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
@@ -7392,22 +7392,22 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>半导体洁净室</t>
+          <t>存储芯片测试设备</t>
         </is>
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>603929</t>
+          <t>688627</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>亚翔集成</t>
+          <t>精智达</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司为IC半导体、光电、云计算中心等建厂工程提供洁净室、机电和建筑工程服务，净利润同比高增；AI受益路径来自半导体/存储扩产与厂务资本开支，属于配套基础设施而非芯片产品直接弹性。</t>
+          <t>证据强：2025年报/公开资料显示半导体存储测试设备业务快速放量，并签订两笔约3.2亿元级半导体重大订单；公司推进高速FT测试机、老化测试修复设备、探针卡及HBM测试设备研发，HBM BI属于未来强化方向，主板块收敛为存储芯片测试设备。</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
@@ -7424,17 +7424,17 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>601133</t>
+          <t>603929</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>柏诚股份</t>
+          <t>亚翔集成</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/摘要显示公司主要从事高等级洁净系统集成服务，覆盖半导体及泛半导体、新型显示、生命科学等；2025营收和利润承压且应收/合同资产占比较高，AI链条为晶圆厂扩产配套，保留半导体洁净室但降低弹性强度。</t>
+          <t>证据中强：2025年报披露公司为IC半导体、光电、云计算中心等建厂工程提供洁净室、机电和建筑工程服务，净利润同比高增；AI受益路径来自半导体/存储扩产与厂务资本开支，属于配套基础设施而非芯片产品直接弹性。</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
@@ -7451,17 +7451,17 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>603163</t>
+          <t>601133</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>圣晖集成</t>
+          <t>柏诚股份</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示公司继续专注洁净室系统集成工程，覆盖设计、采购、施工和维护全链条，主要客户集中在半导体、电子等高科技行业，营收和利润高增；AI受益路径来自晶圆厂/先进封装/存储扩产的厂务资本开支。</t>
+          <t>证据中：2025年报/摘要显示公司主要从事高等级洁净系统集成服务，覆盖半导体及泛半导体、新型显示、生命科学等；2025营收和利润承压且应收/合同资产占比较高，AI链条为晶圆厂扩产配套，保留半导体洁净室但降低弹性强度。</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
@@ -7473,22 +7473,22 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>洁净过滤材料</t>
+          <t>半导体洁净室</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>603601</t>
+          <t>603163</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>再升科技</t>
+          <t>圣晖集成</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司干净空气材料包括高效空气滤材、PTFE膜等，是FFU、新风系统等核心部件，用于工业电子、生物医药等洁净场景；半导体洁净室链条为间接受益，且2025收入利润承压，故由半导体洁净过滤降级为洁净过滤材料。</t>
+          <t>证据强：2025年报显示公司继续专注洁净室系统集成工程，覆盖设计、采购、施工和维护全链条，主要客户集中在半导体、电子等高科技行业，营收和利润高增；AI受益路径来自晶圆厂/先进封装/存储扩产的厂务资本开支。</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
@@ -7500,22 +7500,22 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>半导体洁净过滤</t>
+          <t>洁净过滤材料</t>
         </is>
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>688376</t>
+          <t>603601</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>美埃科技</t>
+          <t>再升科技</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦工业级超洁净技术，风机过滤单元、过滤器和空气净化设备用于半导体等洁净厂房，并通过收购延伸洁净室墙壁和天花板系统；但2025净利润下滑，半导体项目延期压制业绩弹性。</t>
+          <t>证据中：2025年报披露公司干净空气材料包括高效空气滤材、PTFE膜等，是FFU、新风系统等核心部件，用于工业电子、生物医药等洁净场景；半导体洁净室链条为间接受益，且2025收入利润承压，故由半导体洁净过滤降级为洁净过滤材料。</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
@@ -7527,22 +7527,22 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>半导体高纯工艺系统</t>
+          <t>半导体洁净过滤</t>
         </is>
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>300260</t>
+          <t>688376</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>新莱应材</t>
+          <t>美埃科技</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露泛半导体/高纯及超高纯应用材料收入增长，真空和UHP等级管道、管件、阀门、腔体、精密零部件用于半导体制程及厂务；液冷管路属于新布局且规模仍小，合并删减“液冷管路”重复行。</t>
+          <t>证据中强：2025年报披露公司聚焦工业级超洁净技术，风机过滤单元、过滤器和空气净化设备用于半导体等洁净厂房，并通过收购延伸洁净室墙壁和天花板系统；但2025净利润下滑，半导体项目延期压制业绩弹性。</t>
         </is>
       </c>
       <c r="E240" s="6" t="inlineStr">
@@ -7559,17 +7559,17 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>603690</t>
+          <t>300260</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>至纯科技</t>
+          <t>新莱应材</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露公司业务围绕高纯工艺系统、制程设备、电子材料、零部件和专业服务，服务晶圆厂建设投产和运营量产；AI链条来自半导体扩产，但2025归母亏损扩大，湿法设备和高纯系统订单修复需继续验证。</t>
+          <t>证据中强：2025年报披露泛半导体/高纯及超高纯应用材料收入增长，真空和UHP等级管道、管件、阀门、腔体、精密零部件用于半导体制程及厂务；液冷管路属于新布局且规模仍小，合并删减“液冷管路”重复行。</t>
         </is>
       </c>
       <c r="E241" s="6" t="inlineStr">
@@ -7586,17 +7586,17 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>688596</t>
+          <t>603690</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>正帆科技</t>
+          <t>至纯科技</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司稳固“制程关键系统、核心工艺材料与零组件、专业服务”三位一体定位，制程关键系统覆盖多数国内一线晶圆厂，GasBox等设备零部件获头部设备厂商采用；合并删减“半导体核心零部件”重复行。</t>
+          <t>证据中：2025年报摘要披露公司业务围绕高纯工艺系统、制程设备、电子材料、零部件和专业服务，服务晶圆厂建设投产和运营量产；AI链条来自半导体扩产，但2025归母亏损扩大，湿法设备和高纯系统订单修复需继续验证。</t>
         </is>
       </c>
       <c r="E242" s="6" t="inlineStr">
@@ -7608,22 +7608,22 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>半导体工艺废气处理</t>
+          <t>半导体高纯工艺系统</t>
         </is>
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>603324</t>
+          <t>688596</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>盛剑环境</t>
+          <t>正帆科技</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>证据中：公开简称盛剑科技，2025年报显示公司围绕半导体等泛半导体客户提供工艺废气治理、湿电子化学品供应与绿色厂务系统服务；AI受益来自晶圆厂扩产和厂务环保配套，非芯片设备直接弹性。</t>
+          <t>证据中强：2025年报披露公司稳固“制程关键系统、核心工艺材料与零组件、专业服务”三位一体定位，制程关键系统覆盖多数国内一线晶圆厂，GasBox等设备零部件获头部设备厂商采用；合并删减“半导体核心零部件”重复行。</t>
         </is>
       </c>
       <c r="E243" s="6" t="inlineStr">
@@ -7640,17 +7640,17 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>301030</t>
+          <t>603324</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>仕净科技</t>
+          <t>盛剑环境</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>证据弱中：公司有泛半导体/光伏等制程污染防控与废气处理经验，但2025年受光伏客户和资产减值拖累出现大额亏损，半导体AI链条订单和收入证据不足；保留工艺废气处理，但在备注中降级为观察型厂务环保标的。</t>
+          <t>证据中：公开简称盛剑科技，2025年报显示公司围绕半导体等泛半导体客户提供工艺废气治理、湿电子化学品供应与绿色厂务系统服务；AI受益来自晶圆厂扩产和厂务环保配套，非芯片设备直接弹性。</t>
         </is>
       </c>
       <c r="E244" s="6" t="inlineStr">
@@ -7662,22 +7662,22 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>高纯湿电子化学品</t>
+          <t>半导体工艺废气处理</t>
         </is>
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>688549</t>
+          <t>301030</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>中巨芯-U</t>
+          <t>仕净科技</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报显示公司同时覆盖电子湿化学品、电子特种气体和前驱体材料，其中电子湿化学品收入占比约72.5%，电子特气及前驱体占比约23.9%；公司仍亏损，故由ALD-CVD前驱体修正为电子湿化学品。</t>
+          <t>证据弱中：公司有泛半导体/光伏等制程污染防控与废气处理经验，但2025年受光伏客户和资产减值拖累出现大额亏损，半导体AI链条订单和收入证据不足；保留工艺废气处理，但在备注中降级为观察型厂务环保标的。</t>
         </is>
       </c>
       <c r="E245" s="6" t="inlineStr">
@@ -7694,17 +7694,17 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>300655</t>
+          <t>688549</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>晶瑞电材</t>
+          <t>中巨芯-U</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司扭亏并净利润大幅增长，业绩改善主要来自高纯湿化学品量价齐升，光刻胶业务稳健发展且KrF产品已有订单；原半导体光刻胶标签偏窄，收敛为更能解释业绩的高纯湿电子化学品。</t>
+          <t>证据中：2025年报显示公司同时覆盖电子湿化学品、电子特种气体和前驱体材料，其中电子湿化学品收入占比约72.5%，电子特气及前驱体占比约23.9%；公司仍亏损，故由ALD-CVD前驱体修正为电子湿化学品。</t>
         </is>
       </c>
       <c r="E246" s="6" t="inlineStr">
@@ -7716,22 +7716,22 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>光刻胶上游材料</t>
+          <t>高纯湿电子化学品</t>
         </is>
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>300429</t>
+          <t>300655</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>强力新材</t>
+          <t>晶瑞电材</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>公司核心是PCB/LCD/半导体光刻胶光引发剂等电子材料，PSPI先进封装材料项目提供AI先进封装可选弹性；主板块由干膜改为光刻胶上游材料，PSPI并入备注，先进封装电镀液证据不足降级删除。风险是PSPI量产节奏、库存减值、下游竞争和盈利修复。证据B/C。</t>
+          <t>证据中强：2025年报显示公司扭亏并净利润大幅增长，业绩改善主要来自高纯湿化学品量价齐升，光刻胶业务稳健发展且KrF产品已有订单；原半导体光刻胶标签偏窄，收敛为更能解释业绩的高纯湿电子化学品。</t>
         </is>
       </c>
       <c r="E247" s="6" t="inlineStr">
@@ -7743,22 +7743,22 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>半导体光刻胶</t>
+          <t>光刻胶上游材料</t>
         </is>
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>603650</t>
+          <t>300429</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>彤程新材</t>
+          <t>强力新材</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露半导体光刻胶业务高速增长，ArF光刻胶收入实现超800%突破，同时显示光刻胶规模优势稳固；RDL-Bumping属于先进封装光刻材料延伸，合并删减重复行。</t>
+          <t>公司核心是PCB/LCD/半导体光刻胶光引发剂等电子材料，PSPI先进封装材料项目提供AI先进封装可选弹性；主板块由干膜改为光刻胶上游材料，PSPI并入备注，先进封装电镀液证据不足降级删除。风险是PSPI量产节奏、库存减值、下游竞争和盈利修复。证据B/C。</t>
         </is>
       </c>
       <c r="E248" s="6" t="inlineStr">
@@ -7770,22 +7770,22 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>CMP抛光材料</t>
+          <t>半导体光刻胶</t>
         </is>
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>688019</t>
+          <t>603650</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>安集科技</t>
+          <t>彤程新材</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司围绕CMP抛光液、功能性湿电子化学品、电镀液及核心原材料形成“3+1”平台，先进封装用TSV、混合键合、聚合物等抛光液在国内客户中作为首选供应商并销售上量；主板块由泛先进封装工艺材料收敛为CMP抛光材料。</t>
+          <t>证据强：2025年报披露半导体光刻胶业务高速增长，ArF光刻胶收入实现超800%突破，同时显示光刻胶规模优势稳固；RDL-Bumping属于先进封装光刻材料延伸，合并删减重复行。</t>
         </is>
       </c>
       <c r="E249" s="6" t="inlineStr">
@@ -7797,22 +7797,22 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>半导体电子特气</t>
+          <t>CMP抛光材料</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>688268</t>
+          <t>688019</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>华特气体</t>
+          <t>安集科技</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报摘要披露公司特种气体品种数量位居国内前列，已实现57个产品进口替代，覆盖国内8/12英寸集成电路制造厂商超90%客户，并切入全球顶尖半导体供应链；先进封装需求体现在电子特气增量，合并删减泛“先进封装工艺材料”重复行。</t>
+          <t>证据强：2025年报披露公司围绕CMP抛光液、功能性湿电子化学品、电镀液及核心原材料形成“3+1”平台，先进封装用TSV、混合键合、聚合物等抛光液在国内客户中作为首选供应商并销售上量；主板块由泛先进封装工艺材料收敛为CMP抛光材料。</t>
         </is>
       </c>
       <c r="E250" s="6" t="inlineStr">
@@ -7829,17 +7829,17 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>688146</t>
+          <t>688268</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>中船特气</t>
+          <t>华特气体</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司超高纯WF6用于集成电路CVD并具备2000吨/年产能，招股书披露产品纯度达6N以上、可满足不同制程需求，客户覆盖台积电、美光、SK海力士等海内外晶圆厂；AI链条来自先进芯片/存储扩产对CVD钨沉积电子特气需求的拉动。高端确定性强于一般电子特气平台，需跟踪海外新增订单公告、6N/7N价格、钨粉成本及成熟品竞争。</t>
+          <t>证据强：2025年报摘要披露公司特种气体品种数量位居国内前列，已实现57个产品进口替代，覆盖国内8/12英寸集成电路制造厂商超90%客户，并切入全球顶尖半导体供应链；先进封装需求体现在电子特气增量，合并删减泛“先进封装工艺材料”重复行。</t>
         </is>
       </c>
       <c r="E251" s="6" t="inlineStr">
@@ -7856,22 +7856,22 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>600378</t>
+          <t>688146</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>昊华科技</t>
+          <t>中船特气</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>证据中强：昊华气体官网披露电子级六氟化钨5N产品，公开互动口径称WF6产能约600吨/年；AI链条来自先进制程/存储芯片CVD钨沉积用电子特气需求，确定性和客户验证透明度弱于中船特气，需跟踪6N升级、客户认证、出口订单和钨粉成本传导。</t>
+          <t>2026-06-16 WF6复核后列为“main_candidate / 主受益候选”：公司具备直接WF6合成产能、6N产品能力、较高产能利用率和2027年新增产能规划，AI链条来自3D NAND/HBM/先进逻辑CVD钨沉积需求以及钨出口许可、APT/钨粉、WF6价格链。边界是Kanto Denka/Central Glass“2026-07-01永久停产”未获官方确认，公司也提示未签署新的长期或大额实质性订单，不能把WF6涨价线性外推为业绩。证据A/B/C。</t>
         </is>
       </c>
       <c r="E252" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核</t>
         </is>
       </c>
     </row>
@@ -7883,17 +7883,17 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>688106</t>
+          <t>600378</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>金宏气体</t>
+          <t>昊华科技</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露电子特种气体国内市占率约2.81%，电子大宗载气提纯、现场制气及多个半导体/显示项目持续导入；但公司2025年增收不增利、应收较高，主板块由单一电子特气扩为半导体电子气体。</t>
+          <t>证据中强：昊华气体官网披露电子级六氟化钨5N产品，公开互动口径称WF6产能约600吨/年；AI链条来自先进制程/存储芯片CVD钨沉积用电子特气需求，确定性和客户验证透明度弱于中船特气，需跟踪6N升级、客户认证、出口订单和钨粉成本传导。</t>
         </is>
       </c>
       <c r="E253" s="6" t="inlineStr">
@@ -7905,22 +7905,22 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>半导体前驱体材料</t>
+          <t>半导体电子特气</t>
         </is>
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>300346</t>
+          <t>688106</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>南大光电</t>
+          <t>金宏气体</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司围绕先进前驱体、电子特气、光刻胶及配套材料三大核心半导体材料发展，业绩连续增长；光刻胶有产业化突破但收入规模仍需跟踪，主线从光刻胶/ALD-CVD前驱体重复标签收敛为半导体前驱体材料。</t>
+          <t>证据中强：2025年报披露电子特种气体国内市占率约2.81%，电子大宗载气提纯、现场制气及多个半导体/显示项目持续导入；但公司2025年增收不增利、应收较高，主板块由单一电子特气扩为半导体电子气体。</t>
         </is>
       </c>
       <c r="E254" s="6" t="inlineStr">
@@ -7932,22 +7932,22 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>半导体高纯金属靶材</t>
+          <t>半导体前驱体材料</t>
         </is>
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>300666</t>
+          <t>300346</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>江丰电子</t>
+          <t>南大光电</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示公司核心产品为超高纯金属溅射靶材，覆盖先进制程及存储、逻辑、功率等客户，半导体靶材收入占比高；HBM TSV金属材料属于先进封装/存储升级延伸，证据仍弱于靶材主业，合并删减“HBM TSV金属材料”重复行。</t>
+          <t>证据中强：2025年报显示公司围绕先进前驱体、电子特气、光刻胶及配套材料三大核心半导体材料发展，业绩连续增长；光刻胶有产业化突破但收入规模仍需跟踪，主线从光刻胶/ALD-CVD前驱体重复标签收敛为半导体前驱体材料。</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
@@ -7964,17 +7964,17 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>600206</t>
+          <t>300666</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>有研新材</t>
+          <t>江丰电子</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦电子薄膜及贵金属材料等新材料，集成电路及半导体薄膜材料国产化需求持续；高纯金属靶材是更确定主线，HBM TSV金属材料属于先进存储/封装延伸，当前公开证据不足以作为主板块。</t>
+          <t>证据强：2025年报显示公司核心产品为超高纯金属溅射靶材，覆盖先进制程及存储、逻辑、功率等客户，半导体靶材收入占比高；HBM TSV金属材料属于先进封装/存储升级延伸，证据仍弱于靶材主业，合并删减“HBM TSV金属材料”重复行。</t>
         </is>
       </c>
       <c r="E256" s="6" t="inlineStr">
@@ -7986,22 +7986,22 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>半导体先进陶瓷部件</t>
+          <t>半导体高纯金属靶材</t>
         </is>
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>301611</t>
+          <t>600206</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>珂玛科技</t>
+          <t>有研新材</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以半导体先进陶瓷零部件为核心，陶瓷加热器已大批量交付，静电卡盘8/12英寸产品通过客户验证并小规模量产；静电卡盘弹性清晰但收入仍小，主板块由单一静电卡盘修正为半导体先进陶瓷部件。</t>
+          <t>证据中强：2025年报披露公司聚焦电子薄膜及贵金属材料等新材料，集成电路及半导体薄膜材料国产化需求持续；高纯金属靶材是更确定主线，HBM TSV金属材料属于先进存储/封装延伸，当前公开证据不足以作为主板块。</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
@@ -8013,22 +8013,22 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>碳化硅衬底</t>
+          <t>半导体先进陶瓷部件</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>688234</t>
+          <t>301611</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>天岳先进</t>
+          <t>珂玛科技</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营碳化硅衬底，导电型SiC衬底全球份额27.6%、8英寸份额51.3%；AI数据中心拉动SiC材料应用是中长期变量，但2025收入下滑并亏损，需跟踪价格和产能利用率。</t>
+          <t>证据中强：2025年报披露公司以半导体先进陶瓷零部件为核心，陶瓷加热器已大批量交付，静电卡盘8/12英寸产品通过客户验证并小规模量产；静电卡盘弹性清晰但收入仍小，主板块由单一静电卡盘修正为半导体先进陶瓷部件。</t>
         </is>
       </c>
       <c r="E258" s="6" t="inlineStr">
@@ -8040,22 +8040,22 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>内存接口芯片</t>
+          <t>碳化硅衬底</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>688008</t>
+          <t>688234</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>澜起科技</t>
+          <t>天岳先进</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>DDR5 RCD/DB、MRCD/MDB、CKD是AI服务器高带宽内存互连核心节点，PCIe Retimer、CXL MXC扩展高速互连第二曲线；主板块收敛为内存接口芯片，HBM、DDR5 SPD、SOCAMM、CXL和CXL内存扩展模组均并入备注或删除，避免误当存储模组/HBM厂商。风险是海外竞争、服务器平台迭代和新品放量节奏。证据A。</t>
+          <t>证据强：2025年报披露公司主营碳化硅衬底，导电型SiC衬底全球份额27.6%、8英寸份额51.3%；AI数据中心拉动SiC材料应用是中长期变量，但2025收入下滑并亏损，需跟踪价格和产能利用率。</t>
         </is>
       </c>
       <c r="E259" s="6" t="inlineStr">
@@ -8067,22 +8067,22 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>DDR5 SPD</t>
+          <t>内存接口芯片</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>688123</t>
+          <t>688008</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>聚辰股份</t>
+          <t>澜起科技</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>公司具备DDR2/3/4/5内存模组配套SPD、TS等芯片产品，DDR5 SPD受益AI服务器内存模组数量提升，是明确的小芯片弹性节点；主板块保留DDR5 SPD，SOCAMM作为下游内存模组形态并入备注，不单列。风险是DDR5渗透节奏、客户导入、EEPROM周期和价格竞争。证据A。</t>
+          <t>DDR5 RCD/DB、MRCD/MDB、CKD是AI服务器高带宽内存互连核心节点，PCIe Retimer、CXL MXC扩展高速互连第二曲线；主板块收敛为内存接口芯片，HBM、DDR5 SPD、SOCAMM、CXL和CXL内存扩展模组均并入备注或删除，避免误当存储模组/HBM厂商。风险是海外竞争、服务器平台迭代和新品放量节奏。证据A。</t>
         </is>
       </c>
       <c r="E260" s="6" t="inlineStr">
@@ -8094,22 +8094,22 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>高端存储分销</t>
+          <t>DDR5 SPD</t>
         </is>
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>300475</t>
+          <t>688123</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>香农芯创</t>
+          <t>聚辰股份</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>公司以SK海力士核心代理分销为基本盘，向国内云服务器龙头和大型ODM提供存储解决方案；HBM/DDR5紧缺带来强周期弹性，但本质不是HBM制造商。自主海普存储企业级SSD/DRAM开始贡献增量。主板块由HBM改为高端存储分销，风险是存储价格周期、供应商授权、分销毛利和库存。证据A/B。</t>
+          <t>公司具备DDR2/3/4/5内存模组配套SPD、TS等芯片产品，DDR5 SPD受益AI服务器内存模组数量提升，是明确的小芯片弹性节点；主板块保留DDR5 SPD，SOCAMM作为下游内存模组形态并入备注，不单列。风险是DDR5渗透节奏、客户导入、EEPROM周期和价格竞争。证据A。</t>
         </is>
       </c>
       <c r="E261" s="6" t="inlineStr">
@@ -8121,22 +8121,22 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>企业级存储模组</t>
+          <t>高端存储分销</t>
         </is>
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>688525</t>
+          <t>300475</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>佰维存储</t>
+          <t>香农芯创</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>公司企业级存储方案覆盖PCIe/SATA SSD、DDR4/DDR5 RDIMM和CXL内存扩展模组，服务数据中心、服务器和AI工作负载；主板块由DDR5 SPD改为企业级存储模组，SOCAMM、企业级SSD、SSD主控、UFS、晶圆级封测和CXL并入备注或降级。风险是NAND/DRAM价格周期、库存、客户认证和自研控制器/封测兑现。证据B。</t>
+          <t>公司以SK海力士核心代理分销为基本盘，向国内云服务器龙头和大型ODM提供存储解决方案；HBM/DDR5紧缺带来强周期弹性，但本质不是HBM制造商。自主海普存储企业级SSD/DRAM开始贡献增量。主板块由HBM改为高端存储分销，风险是存储价格周期、供应商授权、分销毛利和库存。证据A/B。</t>
         </is>
       </c>
       <c r="E262" s="6" t="inlineStr">
@@ -8153,17 +8153,17 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>301308</t>
+          <t>688525</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>江波龙</t>
+          <t>佰维存储</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>公司企业级eSSD和RDIMM已在互联网、运营商等客户完成验证并批量出货，SOCAMM2、CXL内存扩展、MRDIMM等构成AI服务器存储升级可选项；主板块由SOCAMM改为企业级存储模组，端侧UFS、eMMC、SSD主控、SPU、HLC-iSA、mSSD和CXL并入备注。SOCAMM2仍需收入贡献验证。证据A/B。</t>
+          <t>公司企业级存储方案覆盖PCIe/SATA SSD、DDR4/DDR5 RDIMM和CXL内存扩展模组，服务数据中心、服务器和AI工作负载；主板块由DDR5 SPD改为企业级存储模组，SOCAMM、企业级SSD、SSD主控、UFS、晶圆级封测和CXL并入备注或降级。风险是NAND/DRAM价格周期、库存、客户认证和自研控制器/封测兑现。证据B。</t>
         </is>
       </c>
       <c r="E263" s="6" t="inlineStr">
@@ -8175,22 +8175,22 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD</t>
+          <t>企业级存储模组</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>001309</t>
+          <t>301308</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>德明利</t>
+          <t>江波龙</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露AI浪潮下公司加快向高容量、高性能固态硬盘拓展，重点聚焦QLC NAND企业级应用方向；自研主控是能力基础，但表格保留最贴近收入承载的“企业级SSD”，删减企业级SSD主控、QLC SSD、AI场景化存储方案重复行。风险是存储价格周期和经营现金流波动。</t>
+          <t>公司企业级eSSD和RDIMM已在互联网、运营商等客户完成验证并批量出货，SOCAMM2、CXL内存扩展、MRDIMM等构成AI服务器存储升级可选项；主板块由SOCAMM改为企业级存储模组，端侧UFS、eMMC、SSD主控、SPU、HLC-iSA、mSSD和CXL并入备注。SOCAMM2仍需收入贡献验证。证据A/B。</t>
         </is>
       </c>
       <c r="E264" s="6" t="inlineStr">
@@ -8202,22 +8202,22 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD主控</t>
+          <t>企业级SSD</t>
         </is>
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>300672</t>
+          <t>001309</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>国科微</t>
+          <t>德明利</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>证据中偏弱：公司固态存储主控芯片实现国产替代，同时布局端侧AI、车载电子、智慧视觉等多条芯片线；AI数据中心企业级SSD客户、收入占比和订单仍未充分披露，保留为SSD主控国产替代观察，基本面需关注2025亏损后毛利修复和研发投入转化。</t>
+          <t>证据中强：2025年报摘要披露AI浪潮下公司加快向高容量、高性能固态硬盘拓展，重点聚焦QLC NAND企业级应用方向；自研主控是能力基础，但表格保留最贴近收入承载的“企业级SSD”，删减企业级SSD主控、QLC SSD、AI场景化存储方案重复行。风险是存储价格周期和经营现金流波动。</t>
         </is>
       </c>
       <c r="E265" s="6" t="inlineStr">
@@ -8234,17 +8234,17 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>688449</t>
+          <t>300672</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>联芸科技</t>
+          <t>国科微</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露SSD主控覆盖SATA、PCIe3.0/4.0/5.0，企业级PCIe Gen5 SSD主控已进入量产测试阶段，并规划PCIe Gen6/Gen7切入数据中心；删减UFS主控重复行，UFS偏终端嵌入式，AI算力弹性以企业级SSD主控为主。</t>
+          <t>证据中偏弱：公司固态存储主控芯片实现国产替代，同时布局端侧AI、车载电子、智慧视觉等多条芯片线；AI数据中心企业级SSD客户、收入占比和订单仍未充分披露，保留为SSD主控国产替代观察，基本面需关注2025亏损后毛利修复和研发投入转化。</t>
         </is>
       </c>
       <c r="E266" s="6" t="inlineStr">
@@ -8256,22 +8256,22 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>AI存储</t>
+          <t>企业级SSD主控</t>
         </is>
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>300302</t>
+          <t>688449</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>同有科技</t>
+          <t>联芸科技</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露高端存储在AI智算中心、高性能计算等核心场景推进，NVMe/RDMA高性能分布式文件存储用于智算领域高并发、低延迟需求；主板块保留AI存储，跟踪标杆方案复制、国产化替代和毛利率。</t>
+          <t>证据强：2025年报披露SSD主控覆盖SATA、PCIe3.0/4.0/5.0，企业级PCIe Gen5 SSD主控已进入量产测试阶段，并规划PCIe Gen6/Gen7切入数据中心；删减UFS主控重复行，UFS偏终端嵌入式，AI算力弹性以企业级SSD主控为主。</t>
         </is>
       </c>
       <c r="E267" s="6" t="inlineStr">
@@ -8283,30 +8283,34 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>HBF高带宽闪存</t>
+          <t>AI存储</t>
         </is>
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>300302</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>同有科技</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>德明利2025半年报提到闪迪HBF结合3D NAND与HBM、适合读取密集型AI推理任务；A股暂无成熟高带宽闪存纯标的。</t>
-        </is>
-      </c>
-      <c r="E268" s="6" t="n"/>
+          <t>证据强：2025年报披露高端存储在AI智算中心、高性能计算等核心场景推进，NVMe/RDMA高性能分布式文件存储用于智算领域高并发、低延迟需求；主板块保留AI存储，跟踪标杆方案复制、国产化替代和毛利率。</t>
+        </is>
+      </c>
+      <c r="E268" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>Nearline HDD</t>
+          <t>HBF高带宽闪存</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr">
@@ -8321,7 +8325,7 @@
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>希捷和西部数据官方披露AI数据增长推动数据中心exabyte级低成本存储需求；近线HDD仍主要由海外双寡头主导。</t>
+          <t>德明利2025半年报提到闪迪HBF结合3D NAND与HBM、适合读取密集型AI推理任务；A股暂无成熟高带宽闪存纯标的。</t>
         </is>
       </c>
       <c r="E269" s="6" t="n"/>
@@ -8329,7 +8333,7 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>HAMR-ePMR高容量HDD</t>
+          <t>Nearline HDD</t>
         </is>
       </c>
       <c r="B270" s="3" t="inlineStr">
@@ -8344,7 +8348,7 @@
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>希捷披露HAMR Mozaic放量，西部数据披露40TB UltraSMR ePMR验证和HAMR 100TB路线；A股暂无成熟HDD主线标的。</t>
+          <t>希捷和西部数据官方披露AI数据增长推动数据中心exabyte级低成本存储需求；近线HDD仍主要由海外双寡头主导。</t>
         </is>
       </c>
       <c r="E270" s="6" t="n"/>
@@ -8352,7 +8356,7 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>高带宽HDD</t>
+          <t>HAMR-ePMR高容量HDD</t>
         </is>
       </c>
       <c r="B271" s="3" t="inlineStr">
@@ -8367,7 +8371,7 @@
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>西部数据2026 Innovation Day披露High Bandwidth Drive与Dual Pivot提升HDD带宽/IO，服务AI温冷数据层，A股暂无对应纯标的。</t>
+          <t>希捷披露HAMR Mozaic放量，西部数据披露40TB UltraSMR ePMR验证和HAMR 100TB路线；A股暂无成熟HDD主线标的。</t>
         </is>
       </c>
       <c r="E271" s="6" t="n"/>
@@ -8375,7 +8379,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>CXL</t>
+          <t>高带宽HDD</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
@@ -8390,7 +8394,7 @@
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
+          <t>西部数据2026 Innovation Day披露High Bandwidth Drive与Dual Pivot提升HDD带宽/IO，服务AI温冷数据层，A股暂无对应纯标的。</t>
         </is>
       </c>
       <c r="E272" s="6" t="n"/>
@@ -8398,22 +8402,22 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>CXL内存扩展模组</t>
+          <t>CXL</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
           <t>暂无成熟A股纯标的</t>
         </is>
       </c>
-      <c r="C273" s="2" t="inlineStr">
-        <is>
-          <t>CXL Switch暂无成熟A股纯标的</t>
-        </is>
-      </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>CXL交换/池化控制仍主要由Marvell等海外厂商推进，A股目前缺成熟CXL Switch纯标的。</t>
+          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
         </is>
       </c>
       <c r="E273" s="6" t="n"/>
@@ -8421,49 +8425,45 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>HBM BI</t>
+          <t>CXL内存扩展模组</t>
         </is>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>300567</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>精测电子</t>
+          <t>CXL Switch暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>检测设备平台，2025年报摘要披露推出JH5520 HBM BI测试系统以满足HBM高端存储测试需求，半导体量检测覆盖前道、后道电测和先进封装；主板块改为HBM BI，PCB AOI、半导体量测和先进封装X-Ray并入备注，风险是半导体业务收入占比、客户认证和设备订单兑现。证据A/B。</t>
-        </is>
-      </c>
-      <c r="E274" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>CXL交换/池化控制仍主要由Marvell等海外厂商推进，A股目前缺成熟CXL Switch纯标的。</t>
+        </is>
+      </c>
+      <c r="E274" s="6" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>AI服务器整机</t>
+          <t>HBM BI</t>
         </is>
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>603019</t>
+          <t>300567</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>中科曙光</t>
+          <t>精测电子</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心是高端计算机、智能计算和算力服务，2025年报披露继续围绕AI算力、液冷散热、高速互联等核心领域投入；AI存储和推理板卡只是配套能力，删减AI存储、AI推理板卡、AI服务器ODM重复行，保留更准确的AI服务器整机/智算底座定位。</t>
+          <t>检测设备平台，2025年报摘要披露推出JH5520 HBM BI测试系统以满足HBM高端存储测试需求，半导体量检测覆盖前道、后道电测和先进封装；主板块改为HBM BI，PCB AOI、半导体量测和先进封装X-Ray并入备注，风险是半导体业务收入占比、客户认证和设备订单兑现。证据A/B。</t>
         </is>
       </c>
       <c r="E275" s="6" t="inlineStr">
@@ -8480,17 +8480,17 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>000977</t>
+          <t>603019</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>浪潮信息</t>
+          <t>中科曙光</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露总营收1647.82亿元、同比增长43.25%，主要由服务器产品销售增长驱动；存储交换类收入占比小，删减AI存储重复行，主板块改为AI服务器整机。风险是服务器高增但毛利率偏低，GPU/核心器件供应和价格压力影响利润弹性。</t>
+          <t>证据中强：公司核心是高端计算机、智能计算和算力服务，2025年报披露继续围绕AI算力、液冷散热、高速互联等核心领域投入；AI存储和推理板卡只是配套能力，删减AI存储、AI推理板卡、AI服务器ODM重复行，保留更准确的AI服务器整机/智算底座定位。</t>
         </is>
       </c>
       <c r="E276" s="6" t="inlineStr">
@@ -8507,17 +8507,17 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>000034</t>
+          <t>000977</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>神州数码</t>
+          <t>浪潮信息</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露AI相关业务收入330.3亿元、同比增长47.7%，神州鲲泰服务器基于鲲鹏CPU+昇腾NPU支持DeepSeek等大模型私有化部署，并开放国产技术栈AI智算OpenLab；主线是国产算力整机和方案。</t>
+          <t>证据强：2025年报披露总营收1647.82亿元、同比增长43.25%，主要由服务器产品销售增长驱动；存储交换类收入占比小，删减AI存储重复行，主板块改为AI服务器整机。风险是服务器高增但毛利率偏低，GPU/核心器件供应和价格压力影响利润弹性。</t>
         </is>
       </c>
       <c r="E277" s="6" t="inlineStr">
@@ -8534,17 +8534,17 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>002261</t>
+          <t>000034</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>拓维信息</t>
+          <t>神州数码</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露公司基于“鲲鹏+昇腾AI”算力底座，推出中心侧高性能服务器、推理服务器和边端终端侧产品；主板块从国产AI服务器收敛为昇腾AI服务器，风险是收入下滑、利润体量仍小。</t>
+          <t>证据中强：2025年报披露AI相关业务收入330.3亿元、同比增长47.7%，神州鲲泰服务器基于鲲鹏CPU+昇腾NPU支持DeepSeek等大模型私有化部署，并开放国产技术栈AI智算OpenLab；主线是国产算力整机和方案。</t>
         </is>
       </c>
       <c r="E278" s="6" t="inlineStr">
@@ -8556,22 +8556,22 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>AI服务器ODM</t>
+          <t>AI服务器整机</t>
         </is>
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>601138</t>
+          <t>002261</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>拓维信息</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司与全球头部客户协同下一代AI服务器及液冷技术，云服务商AI服务器收入同比大增，GPU与ASIC方案产品快速增长；删减“AI服务器机柜”重复行，机柜/液冷作为ODM系统能力纳入备注。</t>
+          <t>证据中：2025年报摘要披露公司基于“鲲鹏+昇腾AI”算力底座，推出中心侧高性能服务器、推理服务器和边端终端侧产品；主板块从国产AI服务器收敛为昇腾AI服务器，风险是收入下滑、利润体量仍小。</t>
         </is>
       </c>
       <c r="E279" s="6" t="inlineStr">
@@ -8588,17 +8588,17 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>603296</t>
+          <t>601138</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>华勤技术</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露华勤数据中心业务形成AI服务器、通用服务器、交换机等全栈产品组合，数据中心业务收入754.75亿元、同比增长51.93%；主板块保留AI服务器ODM，AI PC和终端ODM作为附属受益。</t>
+          <t>证据强：2025年报披露公司与全球头部客户协同下一代AI服务器及液冷技术，云服务商AI服务器收入同比大增，GPU与ASIC方案产品快速增长；删减“AI服务器机柜”重复行，机柜/液冷作为ODM系统能力纳入备注。</t>
         </is>
       </c>
       <c r="E280" s="6" t="inlineStr">
@@ -8610,22 +8610,22 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>算力服务器结构件</t>
+          <t>AI服务器ODM</t>
         </is>
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>002965</t>
+          <t>603296</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>祥鑫科技</t>
+          <t>华勤技术</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>证据中弱：2025年报披露公司在通信设备领域可供应通讯插箱、交换机箱、算力服务器等产品和服务，但汽车业务仍占收入主体且净利润下滑；主板块由AI服务器机柜收敛为算力服务器结构件，AI订单强度需继续验证。</t>
+          <t>证据强：2025年报披露华勤数据中心业务形成AI服务器、通用服务器、交换机等全栈产品组合，数据中心业务收入754.75亿元、同比增长51.93%；主板块保留AI服务器ODM，AI PC和终端ODM作为附属受益。</t>
         </is>
       </c>
       <c r="E281" s="6" t="inlineStr">
@@ -8637,22 +8637,22 @@
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>智能算力产品及服务</t>
+          <t>算力服务器结构件</t>
         </is>
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>300857</t>
+          <t>002965</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>协创数据</t>
+          <t>祥鑫科技</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露智能算力产品及服务收入27.61亿元、同比增长1727.17%、占总收入22.57%，成为第二大收入支柱；原IDC标签不准确，改为智能算力产品及服务。</t>
+          <t>证据中弱：2025年报披露公司在通信设备领域可供应通讯插箱、交换机箱、算力服务器等产品和服务，但汽车业务仍占收入主体且净利润下滑；主板块由AI服务器机柜收敛为算力服务器结构件，AI订单强度需继续验证。</t>
         </is>
       </c>
       <c r="E282" s="6" t="inlineStr">
@@ -8664,22 +8664,22 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>国产AI加速芯片</t>
+          <t>智能算力产品及服务</t>
         </is>
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>688256</t>
+          <t>300857</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>寒武纪</t>
+          <t>协创数据</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司云边端智能芯片及板卡矩阵，云端产品线面向服务器和数据中心AI处理，收入大增并首次全年盈利；删减“AI推理板卡”重复行，板卡是产品形态，主板块归入国产AI加速芯片。</t>
+          <t>证据强：2025年报披露智能算力产品及服务收入27.61亿元、同比增长1727.17%、占总收入22.57%，成为第二大收入支柱；原IDC标签不准确，改为智能算力产品及服务。</t>
         </is>
       </c>
       <c r="E283" s="6" t="inlineStr">
@@ -8691,22 +8691,22 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>国产CPU-DCU芯片</t>
+          <t>国产AI加速芯片</t>
         </is>
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>688041</t>
+          <t>688256</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>海光信息</t>
+          <t>寒武纪</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及公开资料显示海光坚持CPU+DCU双芯战略，DCU软件栈适配大模型训练推理并在多行业场景落地；删减“AI推理板卡”重复行，核心价值在国产高端处理器和DCU算力平台。</t>
+          <t>证据强：2025年报披露公司云边端智能芯片及板卡矩阵，云端产品线面向服务器和数据中心AI处理，收入大增并首次全年盈利；删减“AI推理板卡”重复行，板卡是产品形态，主板块归入国产AI加速芯片。</t>
         </is>
       </c>
       <c r="E284" s="6" t="inlineStr">
@@ -8718,22 +8718,22 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>国产GPU芯片</t>
+          <t>国产CPU-DCU芯片</t>
         </is>
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>300474</t>
+          <t>688041</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>景嘉微</t>
+          <t>海光信息</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司推进“高性能GPU+边端侧AI SoC芯片”双轮驱动，景宏系列智算模块及整机产品瞄准AI训练和推理；删减“AI推理板卡”重复行，当前仍以国产GPU芯片为主线，亏损和商业化规模是主要风险。</t>
+          <t>证据强：2025年报及公开资料显示海光坚持CPU+DCU双芯战略，DCU软件栈适配大模型训练推理并在多行业场景落地；删减“AI推理板卡”重复行，核心价值在国产高端处理器和DCU算力平台。</t>
         </is>
       </c>
       <c r="E285" s="6" t="inlineStr">
@@ -8745,22 +8745,22 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>AI推理芯片</t>
+          <t>国产GPU芯片</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>688343</t>
+          <t>300474</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>云天励飞</t>
+          <t>景嘉微</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司构建应用、算法、芯片全栈能力，自研AI推理芯片适配国产大模型、操作系统和推理框架，并推出大模型一体机；一体机为产品化形态，主板块保留AI推理芯片。</t>
+          <t>证据中：2025年报披露公司推进“高性能GPU+边端侧AI SoC芯片”双轮驱动，景宏系列智算模块及整机产品瞄准AI训练和推理；删减“AI推理板卡”重复行，当前仍以国产GPU芯片为主线，亏损和商业化规模是主要风险。</t>
         </is>
       </c>
       <c r="E286" s="6" t="inlineStr">
@@ -8772,22 +8772,22 @@
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>智算网络设备</t>
+          <t>AI推理芯片</t>
         </is>
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>000938</t>
+          <t>688343</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>紫光股份</t>
+          <t>云天励飞</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>证据强：新华三深度覆盖云、网、安、算、存、端，但公司披露中国数据中心交换机份额居前，并在智算网络、800G/CPO交换机和AI算力基础设施上持续推进；删减AI存储、AI服务器ODM重复行，主板块保留最能体现差异化和份额优势的智算交换机。</t>
+          <t>证据中强：2025年报披露公司构建应用、算法、芯片全栈能力，自研AI推理芯片适配国产大模型、操作系统和推理框架，并推出大模型一体机；一体机为产品化形态，主板块保留AI推理芯片。</t>
         </is>
       </c>
       <c r="E287" s="6" t="inlineStr">
@@ -8804,17 +8804,17 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>301165</t>
+          <t>000938</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>锐捷网络</t>
+          <t>紫光股份</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI智算中心网络方案已服务中国移动、阿里、字节、百度、腾讯等训练/推理大模型场景，数据中心交换机订单加速交付；IDC数据显示中国数据中心交换机市占率第三。</t>
+          <t>证据强：新华三深度覆盖云、网、安、算、存、端，但公司披露中国数据中心交换机份额居前，并在智算网络、800G/CPO交换机和AI算力基础设施上持续推进；删减AI存储、AI服务器ODM重复行，主板块保留最能体现差异化和份额优势的智算交换机。</t>
         </is>
       </c>
       <c r="E288" s="6" t="inlineStr">
@@ -8831,17 +8831,17 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>000063</t>
+          <t>301165</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>中兴通讯</t>
+          <t>锐捷网络</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及公司新闻披露算力业务收入同比约150%，服务器及存储同比超200%，数据中心产品同比增长；公司以自研AI大容量交换芯片支撑智算超节点和万卡级智算中心，主板块从交换机扩展为智算网络设备。</t>
+          <t>证据强：2025年报披露AI智算中心网络方案已服务中国移动、阿里、字节、百度、腾讯等训练/推理大模型场景，数据中心交换机订单加速交付；IDC数据显示中国数据中心交换机市占率第三。</t>
         </is>
       </c>
       <c r="E289" s="6" t="inlineStr">
@@ -8853,22 +8853,22 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>以太网交换芯片</t>
+          <t>智算网络设备</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>688702</t>
+          <t>000063</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>盛科通信-U</t>
+          <t>中兴通讯</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营以太网交换芯片及配套产品，交换芯片收入8.31亿元、占营收72.26%，交换机收入占比较低；删减“智算交换机”重复行，保留最能体现价值量的以太网交换芯片，风险是亏损扩大和高端产品放量节奏。</t>
+          <t>证据强：2025年报及公司新闻披露算力业务收入同比约150%，服务器及存储同比超200%，数据中心产品同比增长；公司以自研AI大容量交换芯片支撑智算超节点和万卡级智算中心，主板块从交换机扩展为智算网络设备。</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
@@ -8880,22 +8880,22 @@
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>以太网PHY-交换芯片</t>
+          <t>以太网交换芯片</t>
         </is>
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>688515</t>
+          <t>688702</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>裕太微</t>
+          <t>盛科通信-U</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注高速有线通信芯片，网通PHY、交换机芯片、网卡芯片已规模量产，网通类产品销量约1.4亿颗，并向数据中心与基站等高价值场景延伸；AI数据中心直接收入仍需跟踪。</t>
+          <t>证据中强：2025年报披露公司主营以太网交换芯片及配套产品，交换芯片收入8.31亿元、占营收72.26%，交换机收入占比较低；删减“智算交换机”重复行，保留最能体现价值量的以太网交换芯片，风险是亏损扩大和高端产品放量节奏。</t>
         </is>
       </c>
       <c r="E291" s="6" t="inlineStr">
@@ -8907,30 +8907,34 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>PCIe Switch</t>
+          <t>以太网PHY-交换芯片</t>
         </is>
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>688515</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>裕太微</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>GPU集群内PCIe Switch、NVSwitch和高端交换ASIC主要由NVIDIA、Broadcom、Microchip、Astera等海外厂商主导，A股不硬凑。</t>
-        </is>
-      </c>
-      <c r="E292" s="6" t="n"/>
+          <t>证据中：2025年报披露公司专注高速有线通信芯片，网通PHY、交换机芯片、网卡芯片已规模量产，网通类产品销量约1.4亿颗，并向数据中心与基站等高价值场景延伸；AI数据中心直接收入仍需跟踪。</t>
+        </is>
+      </c>
+      <c r="E292" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>BMC</t>
+          <t>PCIe Switch</t>
         </is>
       </c>
       <c r="B293" s="3" t="inlineStr">
@@ -8945,7 +8949,7 @@
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>AI服务器BMC/远程管理芯片以海外和台湾厂商为主，A股目前缺成熟纯标的，先列系统级空白。</t>
+          <t>GPU集群内PCIe Switch、NVSwitch和高端交换ASIC主要由NVIDIA、Broadcom、Microchip、Astera等海外厂商主导，A股不硬凑。</t>
         </is>
       </c>
       <c r="E293" s="6" t="n"/>
@@ -8953,49 +8957,45 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>Edge BMC管理芯片</t>
+          <t>BMC</t>
         </is>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>688595</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>芯海科技</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露面向边缘计算及服务器市场的轻量级edge BMC管理芯片已上市并量产销售，同时EC芯片在AI PC量产；保留BMC但改为Edge BMC管理芯片，风险是公司仍亏损且BMC收入规模未单列。</t>
-        </is>
-      </c>
-      <c r="E294" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>AI服务器BMC/远程管理芯片以海外和台湾厂商为主，A股目前缺成熟纯标的，先列系统级空白。</t>
+        </is>
+      </c>
+      <c r="E294" s="6" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>低抖动时钟源</t>
+          <t>Edge BMC管理芯片</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>603738</t>
+          <t>688595</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>泰晶科技</t>
+          <t>芯海科技</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露公司开发面向AI数据中心基础设施的312.5MHz差分输出温补振荡器和低抖动可编程振荡器，满足AI数据中心、3.2T光模块、AI算力等需求；主板块保留低抖动时钟源。</t>
+          <t>证据中：2025年报摘要披露面向边缘计算及服务器市场的轻量级edge BMC管理芯片已上市并量产销售，同时EC芯片在AI PC量产；保留BMC但改为Edge BMC管理芯片，风险是公司仍亏损且BMC收入规模未单列。</t>
         </is>
       </c>
       <c r="E295" s="6" t="inlineStr">
@@ -9007,22 +9007,22 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>高频晶振</t>
+          <t>低抖动时钟源</t>
         </is>
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>300460</t>
+          <t>603738</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>惠伦晶体</t>
+          <t>泰晶科技</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>证据弱：2025半年报披露公司主营石英晶体元器件，高频产品和服务器等领域方案商认证具备基础支撑价值；但2025年仍亏损且未见明确AI服务器低抖动订单，主板块由低抖动时钟源降级为高频晶振观察。</t>
+          <t>证据中强：2025年报/半年报披露公司开发面向AI数据中心基础设施的312.5MHz差分输出温补振荡器和低抖动可编程振荡器，满足AI数据中心、3.2T光模块、AI算力等需求；主板块保留低抖动时钟源。</t>
         </is>
       </c>
       <c r="E296" s="6" t="inlineStr">
@@ -9034,22 +9034,22 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>IDC</t>
+          <t>高频晶振</t>
         </is>
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>600845</t>
+          <t>300460</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>宝信软件</t>
+          <t>惠伦晶体</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>工业软件和IDC双主业，宝之云IDC、华北基地、人工智能算力资源池等资产构成算力基础设施运营侧真实映射；DCIM不是公司最核心的AI受益解释。主板块由DCIM改为IDC，原IDC重复行合并删除。风险是钢铁行业软件需求承压、IDC资本开支和上架率、电力成本、AI算力资源池回报周期。证据A/B。</t>
+          <t>证据弱：2025半年报披露公司主营石英晶体元器件，高频产品和服务器等领域方案商认证具备基础支撑价值；但2025年仍亏损且未见明确AI服务器低抖动订单，主板块由低抖动时钟源降级为高频晶振观察。</t>
         </is>
       </c>
       <c r="E297" s="6" t="inlineStr">
@@ -9061,22 +9061,22 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>AIDC智算中心</t>
+          <t>IDC</t>
         </is>
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>300442</t>
+          <t>600845</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>宝信软件</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示AIDC收入25.1亿元、占总收入44.24%，新增交付算力规模220MW且含单体100MW智算中心；合并IDC/算力中心运维，主线改为AIDC智算中心。</t>
+          <t>工业软件和IDC双主业，宝之云IDC、华北基地、人工智能算力资源池等资产构成算力基础设施运营侧真实映射；DCIM不是公司最核心的AI受益解释。主板块由DCIM改为IDC，原IDC重复行合并删除。风险是钢铁行业软件需求承压、IDC资本开支和上架率、电力成本、AI算力资源池回报周期。证据A/B。</t>
         </is>
       </c>
       <c r="E298" s="6" t="inlineStr">
@@ -9088,22 +9088,22 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>IDC及算力租赁</t>
+          <t>AIDC智算中心</t>
         </is>
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>300738</t>
+          <t>300442</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>奥飞数据</t>
+          <t>润泽科技</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露业务为IDC及互联网综合服务，报告期新项目投产并继续推进算力租赁和相关设备销售；AI链受益来自机柜上架和算力需求，保留IDC及算力租赁。</t>
+          <t>证据强：2025年报显示AIDC收入25.1亿元、占总收入44.24%，新增交付算力规模220MW且含单体100MW智算中心；合并IDC/算力中心运维，主线改为AIDC智算中心。</t>
         </is>
       </c>
       <c r="E299" s="6" t="inlineStr">
@@ -9115,22 +9115,22 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>IDC云计算基础设施</t>
+          <t>IDC及算力租赁</t>
         </is>
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>300383</t>
+          <t>300738</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>光环新网</t>
+          <t>奥飞数据</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露主营仍是IDC及云计算，AI爆发带动数据中心与云计算需求，并与格灵深瞳合作AI+行业智算云；直接算力运营收入未充分拆分，保留IDC云计算基础设施。</t>
+          <t>证据中：2025年报披露业务为IDC及互联网综合服务，报告期新项目投产并继续推进算力租赁和相关设备销售；AI链受益来自机柜上架和算力需求，保留IDC及算力租赁。</t>
         </is>
       </c>
       <c r="E300" s="6" t="inlineStr">
@@ -9142,22 +9142,22 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>算力中心运维</t>
+          <t>IDC云计算基础设施</t>
         </is>
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>002929</t>
+          <t>300383</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>润建股份</t>
+          <t>光环新网</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露算力网络业务增长、算力中心管理运维和智算云服务推进，但AI及算力收入占比仍较小且归母净利下滑；保留算力中心运维并下调盈利确定性。</t>
+          <t>证据中：2025年报披露主营仍是IDC及云计算，AI爆发带动数据中心与云计算需求，并与格灵深瞳合作AI+行业智算云；直接算力运营收入未充分拆分，保留IDC云计算基础设施。</t>
         </is>
       </c>
       <c r="E301" s="6" t="inlineStr">
@@ -9169,22 +9169,22 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>算力设备交付运维</t>
+          <t>算力中心运维</t>
         </is>
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>301085</t>
+          <t>002929</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>亚康股份</t>
+          <t>润建股份</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露向富士康、英业达、华勤、浪潮等算力服务器制造商提供交付及售后维保，并从传统数据中心向AI智算中心运维升级；公司亏损，主线为算力设备交付运维。</t>
+          <t>证据中：2025年报披露算力网络业务增长、算力中心管理运维和智算云服务推进，但AI及算力收入占比仍较小且归母净利下滑；保留算力中心运维并下调盈利确定性。</t>
         </is>
       </c>
       <c r="E302" s="6" t="inlineStr">
@@ -9196,22 +9196,22 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>AI智能终端ODM</t>
+          <t>算力设备交付运维</t>
         </is>
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>603341</t>
+          <t>301085</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>龙旗科技</t>
+          <t>亚康股份</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露AI PC实现全平台产品设计与量产落地并获得全球头部客户订单，智能眼镜实现多场景、多品类规模化量产，AIoT业务覆盖智能手表/手环和智能眼镜；主板块从智能终端ODM细化为AI智能终端ODM。风险是手机/平板仍占大盘，新业务弹性需看AI PC、智能眼镜收入占比和毛利。</t>
+          <t>证据中：2025年报摘要披露向富士康、英业达、华勤、浪潮等算力服务器制造商提供交付及售后维保，并从传统数据中心向AI智算中心运维升级；公司亏损，主线为算力设备交付运维。</t>
         </is>
       </c>
       <c r="E303" s="6" t="inlineStr">
@@ -9223,22 +9223,22 @@
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>端侧AI SoC</t>
+          <t>AI智能终端ODM</t>
         </is>
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>603893</t>
+          <t>603341</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>瑞芯微</t>
+          <t>龙旗科技</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/半年报披露智能应用处理器为核心收入来源，RK3588/RK3576等SoC和自研NPU支持端侧模型、AIoT多场景落地；主板块从“端侧AI处理器”规范为“端侧AI SoC”，跟踪高端SoC新品、客户导入和AIoT需求持续性。</t>
+          <t>证据中强：2025年报披露AI PC实现全平台产品设计与量产落地并获得全球头部客户订单，智能眼镜实现多场景、多品类规模化量产，AIoT业务覆盖智能手表/手环和智能眼镜；主板块从智能终端ODM细化为AI智能终端ODM。风险是手机/平板仍占大盘，新业务弹性需看AI PC、智能眼镜收入占比和毛利。</t>
         </is>
       </c>
       <c r="E304" s="6" t="inlineStr">
@@ -9255,17 +9255,17 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>300458</t>
+          <t>603893</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>全志科技</t>
+          <t>瑞芯微</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司实现CPU、GPU、NPU、DSP及RISC-V协处理器复杂异构芯片规模化量产，智能终端应用处理器是核心业务；删减AI眼镜应用处理器重复行，AI眼镜只是下游应用之一，主板块保留端侧AI SoC。</t>
+          <t>证据强：2025年报/半年报披露智能应用处理器为核心收入来源，RK3588/RK3576等SoC和自研NPU支持端侧模型、AIoT多场景落地；主板块从“端侧AI处理器”规范为“端侧AI SoC”，跟踪高端SoC新品、客户导入和AIoT需求持续性。</t>
         </is>
       </c>
       <c r="E305" s="6" t="inlineStr">
@@ -9282,17 +9282,17 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>688099</t>
+          <t>300458</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>晶晨股份</t>
+          <t>全志科技</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露智能多媒体及显示SoC仍是核心收入来源，AIoT SoC收入16.40亿元、同比增长8.50%，AIoT SoC集成NPU、DSP、视觉处理单元、ISP及编解码器并获Google EDLA认证；主板块从端侧AIoT SoC收敛为端侧AI SoC，跟踪端侧大模型适配、头部客户新品和经营现金流修复。</t>
+          <t>证据中强：2025年报披露公司实现CPU、GPU、NPU、DSP及RISC-V协处理器复杂异构芯片规模化量产，智能终端应用处理器是核心业务；删减AI眼镜应用处理器重复行，AI眼镜只是下游应用之一，主板块保留端侧AI SoC。</t>
         </is>
       </c>
       <c r="E306" s="6" t="inlineStr">
@@ -9304,22 +9304,22 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜主控SoC</t>
+          <t>端侧AI SoC</t>
         </is>
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>688608</t>
+          <t>688099</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>恒玄科技</t>
+          <t>晶晨股份</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
+          <t>证据中强：2025年报披露智能多媒体及显示SoC仍是核心收入来源，AIoT SoC收入16.40亿元、同比增长8.50%，AIoT SoC集成NPU、DSP、视觉处理单元、ISP及编解码器并获Google EDLA认证；主板块从端侧AIoT SoC收敛为端侧AI SoC，跟踪端侧大模型适配、头部客户新品和经营现金流修复。</t>
         </is>
       </c>
       <c r="E307" s="6" t="inlineStr">
@@ -9331,22 +9331,22 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>智能穿戴SoC</t>
+          <t>AI眼镜主控SoC</t>
         </is>
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>688049</t>
+          <t>688608</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>炬芯科技</t>
+          <t>恒玄科技</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
+          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
         </is>
       </c>
       <c r="E308" s="6" t="inlineStr">
@@ -9358,22 +9358,22 @@
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>端侧音视频SoC</t>
+          <t>智能穿戴SoC</t>
         </is>
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>688332</t>
+          <t>688049</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>中科蓝讯</t>
+          <t>炬芯科技</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
+          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
         </is>
       </c>
       <c r="E309" s="6" t="inlineStr">
@@ -9385,22 +9385,22 @@
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>端侧AI MCU</t>
+          <t>端侧音视频SoC</t>
         </is>
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>688018</t>
+          <t>688332</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>乐鑫科技</t>
+          <t>中科蓝讯</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
+          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
         </is>
       </c>
       <c r="E310" s="6" t="inlineStr">
@@ -9412,22 +9412,22 @@
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>端侧AI蜂窝模组</t>
+          <t>端侧AI MCU</t>
         </is>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>603236</t>
+          <t>688018</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>移远通信</t>
+          <t>乐鑫科技</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
+          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
         </is>
       </c>
       <c r="E311" s="6" t="inlineStr">
@@ -9439,22 +9439,22 @@
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>高算力智能模组</t>
+          <t>端侧AI蜂窝模组</t>
         </is>
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>002881</t>
+          <t>603236</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>美格智能</t>
+          <t>移远通信</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
+          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
         </is>
       </c>
       <c r="E312" s="6" t="inlineStr">
@@ -9466,22 +9466,22 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>端侧AI模组</t>
+          <t>高算力智能模组</t>
         </is>
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>300638</t>
+          <t>002881</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>广和通</t>
+          <t>美格智能</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
+          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
         </is>
       </c>
       <c r="E313" s="6" t="inlineStr">
@@ -9493,22 +9493,22 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>AIOS端侧智能</t>
+          <t>端侧AI模组</t>
         </is>
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>300496</t>
+          <t>300638</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>中科创达</t>
+          <t>广和通</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
+          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
         </is>
       </c>
       <c r="E314" s="6" t="inlineStr">
@@ -9520,22 +9520,22 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>AR光波导</t>
+          <t>AIOS端侧智能</t>
         </is>
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>002273</t>
+          <t>300496</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>水晶光电</t>
+          <t>中科创达</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
+          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
         </is>
       </c>
       <c r="E315" s="6" t="inlineStr">
@@ -9547,22 +9547,22 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜光学模组</t>
+          <t>AR光波导</t>
         </is>
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>300433</t>
+          <t>002273</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>蓝思科技</t>
+          <t>水晶光电</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
+          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
         </is>
       </c>
       <c r="E316" s="6" t="inlineStr">
@@ -9574,22 +9574,22 @@
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>AR投影光机</t>
+          <t>AI眼镜光学模组</t>
         </is>
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>688010</t>
+          <t>300433</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>福光股份</t>
+          <t>蓝思科技</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
+          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
         </is>
       </c>
       <c r="E317" s="6" t="inlineStr">
@@ -9601,22 +9601,22 @@
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>硅基OLED微显示</t>
+          <t>AR投影光机</t>
         </is>
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>688496</t>
+          <t>688010</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>清越科技</t>
+          <t>福光股份</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
+          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
         </is>
       </c>
       <c r="E318" s="6" t="inlineStr">
@@ -9628,22 +9628,22 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED光机</t>
+          <t>硅基OLED微显示</t>
         </is>
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>300296</t>
+          <t>688496</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>利亚德</t>
+          <t>清越科技</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
+          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
         </is>
       </c>
       <c r="E319" s="6" t="inlineStr">
@@ -9655,22 +9655,22 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED微显示</t>
+          <t>AI眼镜MicroLED光机</t>
         </is>
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>300323</t>
+          <t>300296</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>京东方华灿</t>
+          <t>利亚德</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
+          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
         </is>
       </c>
       <c r="E320" s="6" t="inlineStr">
@@ -9682,22 +9682,22 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MicroLED芯片</t>
+          <t>AI眼镜MicroLED微显示</t>
         </is>
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>600703</t>
+          <t>300323</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>三安光电</t>
+          <t>京东方华灿</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
+          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
         </is>
       </c>
       <c r="E321" s="6" t="inlineStr">
@@ -9709,22 +9709,22 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>OLED-MicroLED显示</t>
+          <t>MicroLED芯片</t>
         </is>
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>002387</t>
+          <t>600703</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>维信诺</t>
+          <t>三安光电</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
+          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
         </is>
       </c>
       <c r="E322" s="6" t="inlineStr">
@@ -9736,22 +9736,22 @@
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜CIS</t>
+          <t>OLED-MicroLED显示</t>
         </is>
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>688213</t>
+          <t>002387</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>思特威</t>
+          <t>维信诺</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
+          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
         </is>
       </c>
       <c r="E323" s="6" t="inlineStr">
@@ -9768,17 +9768,17 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>688728</t>
+          <t>688213</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>格科微</t>
+          <t>思特威</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
+          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
         </is>
       </c>
       <c r="E324" s="6" t="inlineStr">
@@ -9790,22 +9790,22 @@
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜视觉算法</t>
+          <t>AI眼镜CIS</t>
         </is>
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>688088</t>
+          <t>688728</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>虹软科技</t>
+          <t>格科微</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
+          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
         </is>
       </c>
       <c r="E325" s="6" t="inlineStr">
@@ -9817,22 +9817,22 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜模拟芯片</t>
+          <t>AI眼镜视觉算法</t>
         </is>
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>688798</t>
+          <t>688088</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>艾为电子</t>
+          <t>虹软科技</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
+          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
         </is>
       </c>
       <c r="E326" s="6" t="inlineStr">
@@ -9844,22 +9844,22 @@
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜声学传感器</t>
+          <t>AI眼镜模拟芯片</t>
         </is>
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>688286</t>
+          <t>688798</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>敏芯股份</t>
+          <t>艾为电子</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
+          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
         </is>
       </c>
       <c r="E327" s="6" t="inlineStr">
@@ -9871,22 +9871,22 @@
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>消费锂电池</t>
+          <t>AI眼镜声学传感器</t>
         </is>
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>688772</t>
+          <t>688286</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>珠海冠宇</t>
+          <t>敏芯股份</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
+          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
         </is>
       </c>
       <c r="E328" s="6" t="inlineStr">
@@ -9898,22 +9898,22 @@
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜电池</t>
+          <t>消费锂电池</t>
         </is>
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>001283</t>
+          <t>688772</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>豪鹏科技</t>
+          <t>珠海冠宇</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
+          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
         </is>
       </c>
       <c r="E329" s="6" t="inlineStr">
@@ -9925,22 +9925,22 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜结构件</t>
+          <t>AI智能眼镜电池</t>
         </is>
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>300115</t>
+          <t>001283</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>长盈精密</t>
+          <t>豪鹏科技</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
+          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
         </is>
       </c>
       <c r="E330" s="6" t="inlineStr">
@@ -9952,22 +9952,22 @@
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜整机</t>
+          <t>AI眼镜结构件</t>
         </is>
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>002241</t>
+          <t>300115</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>歌尔股份</t>
+          <t>长盈精密</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
+          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
         </is>
       </c>
       <c r="E331" s="6" t="inlineStr">
@@ -9979,22 +9979,22 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>AI终端精密功能件</t>
+          <t>AI智能眼镜整机</t>
         </is>
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>002600</t>
+          <t>002241</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>领益智造</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
+          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
         </is>
       </c>
       <c r="E332" s="6" t="inlineStr">
@@ -10006,22 +10006,22 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>机器人3D视觉</t>
+          <t>AI终端精密功能件</t>
         </is>
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>688322</t>
+          <t>002600</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>奥比中光</t>
+          <t>领益智造</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
+          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
         </is>
       </c>
       <c r="E333" s="6" t="inlineStr">
@@ -10033,22 +10033,22 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>机器人力传感器</t>
+          <t>机器人3D视觉</t>
         </is>
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>603662</t>
+          <t>688322</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>柯力传感</t>
+          <t>奥比中光</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
+          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
         </is>
       </c>
       <c r="E334" s="6" t="inlineStr">
@@ -10065,17 +10065,17 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>301413</t>
+          <t>603662</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>安培龙</t>
+          <t>柯力传感</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
+          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
         </is>
       </c>
       <c r="E335" s="6" t="inlineStr">
@@ -10092,17 +10092,17 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>300354</t>
+          <t>301413</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>东华测试</t>
+          <t>安培龙</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
+          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
         </is>
       </c>
       <c r="E336" s="6" t="inlineStr">
@@ -10114,22 +10114,22 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>机器人电子皮肤</t>
+          <t>机器人力传感器</t>
         </is>
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>300007</t>
+          <t>300354</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>汉威科技</t>
+          <t>东华测试</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
+          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
         </is>
       </c>
       <c r="E337" s="6" t="inlineStr">
@@ -10141,22 +10141,22 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>机器人谐波减速器</t>
+          <t>机器人电子皮肤</t>
         </is>
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>688017</t>
+          <t>300007</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>绿的谐波</t>
+          <t>汉威科技</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
+          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
         </is>
       </c>
       <c r="E338" s="6" t="inlineStr">
@@ -10168,22 +10168,22 @@
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>机器人精密减速器</t>
+          <t>机器人谐波减速器</t>
         </is>
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>002896</t>
+          <t>688017</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>中大力德</t>
+          <t>绿的谐波</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
+          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
         </is>
       </c>
       <c r="E339" s="6" t="inlineStr">
@@ -10200,17 +10200,17 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>002472</t>
+          <t>002896</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>双环传动</t>
+          <t>中大力德</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
+          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
         </is>
       </c>
       <c r="E340" s="6" t="inlineStr">
@@ -10222,22 +10222,22 @@
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>行星滚柱丝杠</t>
+          <t>机器人精密减速器</t>
         </is>
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>603667</t>
+          <t>002472</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>五洲新春</t>
+          <t>双环传动</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
+          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
         </is>
       </c>
       <c r="E341" s="6" t="inlineStr">
@@ -10254,17 +10254,17 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>601100</t>
+          <t>603667</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>恒立液压</t>
+          <t>五洲新春</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
+          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
         </is>
       </c>
       <c r="E342" s="6" t="inlineStr">
@@ -10281,17 +10281,17 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>688678</t>
+          <t>601100</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>福立旺</t>
+          <t>恒立液压</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
+          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
         </is>
       </c>
       <c r="E343" s="6" t="inlineStr">
@@ -10308,17 +10308,17 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>603009</t>
+          <t>688678</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>北特科技</t>
+          <t>福立旺</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
+          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
         </is>
       </c>
       <c r="E344" s="6" t="inlineStr">
@@ -10330,22 +10330,22 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>机器人执行器</t>
+          <t>行星滚柱丝杠</t>
         </is>
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>601689</t>
+          <t>603009</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>拓普集团</t>
+          <t>北特科技</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
+          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
         </is>
       </c>
       <c r="E345" s="6" t="inlineStr">
@@ -10357,22 +10357,22 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>机器人伺服驱动</t>
+          <t>机器人执行器</t>
         </is>
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>300124</t>
+          <t>601689</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>汇川技术</t>
+          <t>拓普集团</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
+          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
         </is>
       </c>
       <c r="E346" s="6" t="inlineStr">
@@ -10384,22 +10384,22 @@
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>机器人驱控系统</t>
+          <t>机器人伺服驱动</t>
         </is>
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>002979</t>
+          <t>300124</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>雷赛智能</t>
+          <t>汇川技术</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
+          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
         </is>
       </c>
       <c r="E347" s="6" t="inlineStr">
@@ -10411,22 +10411,22 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>空心杯电机</t>
+          <t>机器人驱控系统</t>
         </is>
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>603728</t>
+          <t>002979</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>鸣志电器</t>
+          <t>雷赛智能</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
+          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
         </is>
       </c>
       <c r="E348" s="6" t="inlineStr">
@@ -10438,22 +10438,22 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>行业大模型+Agent平台</t>
+          <t>空心杯电机</t>
         </is>
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>300229</t>
+          <t>603728</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>拓尔思</t>
+          <t>鸣志电器</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
+          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
         </is>
       </c>
       <c r="E349" s="6" t="inlineStr">
@@ -10465,22 +10465,22 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>行业大模型训推一体</t>
+          <t>行业大模型+Agent平台</t>
         </is>
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>688327</t>
+          <t>300229</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>云从科技</t>
+          <t>拓尔思</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
+          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
         </is>
       </c>
       <c r="E350" s="6" t="inlineStr">
@@ -10492,22 +10492,22 @@
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>国产算力大模型底座</t>
+          <t>行业大模型训推一体</t>
         </is>
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>002230</t>
+          <t>688327</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>科大讯飞</t>
+          <t>云从科技</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
         </is>
       </c>
       <c r="E351" s="6" t="inlineStr">
@@ -10519,22 +10519,22 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>企业AI平台</t>
+          <t>国产算力大模型底座</t>
         </is>
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>600588</t>
+          <t>002230</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>用友网络</t>
+          <t>科大讯飞</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
+          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
         </is>
       </c>
       <c r="E352" s="6" t="inlineStr">
@@ -10546,22 +10546,22 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>企业级AI应用平台</t>
+          <t>企业AI平台</t>
         </is>
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>300170</t>
+          <t>600588</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>汉得信息</t>
+          <t>用友网络</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
+          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
         </is>
       </c>
       <c r="E353" s="6" t="inlineStr">
@@ -10573,22 +10573,22 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>行业AI智能体平台</t>
+          <t>企业级AI应用平台</t>
         </is>
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>301236</t>
+          <t>300170</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>软通动力</t>
+          <t>汉得信息</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
         </is>
       </c>
       <c r="E354" s="6" t="inlineStr">
@@ -10600,22 +10600,22 @@
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>制造业AI智能体平台</t>
+          <t>行业AI智能体平台</t>
         </is>
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>300378</t>
+          <t>301236</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>鼎捷数智</t>
+          <t>软通动力</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
         </is>
       </c>
       <c r="E355" s="6" t="inlineStr">
@@ -10627,22 +10627,22 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>行业AI交付</t>
+          <t>制造业AI智能体平台</t>
         </is>
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>002649</t>
+          <t>300378</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>博彦科技</t>
+          <t>鼎捷数智</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
+          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
         </is>
       </c>
       <c r="E356" s="6" t="inlineStr">
@@ -10654,22 +10654,22 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>AI数据基础设施软件</t>
+          <t>行业AI交付</t>
         </is>
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>688031</t>
+          <t>002649</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>星环科技</t>
+          <t>博彦科技</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
         </is>
       </c>
       <c r="E357" s="6" t="inlineStr">
@@ -10681,22 +10681,22 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>向量数据库</t>
+          <t>AI数据基础设施软件</t>
         </is>
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>603138</t>
+          <t>688031</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>海量数据</t>
+          <t>星环科技</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
+          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
         </is>
       </c>
       <c r="E358" s="6" t="inlineStr">
@@ -10708,22 +10708,22 @@
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>AI数据库</t>
+          <t>向量数据库</t>
         </is>
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>688692</t>
+          <t>603138</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>达梦数据</t>
+          <t>海量数据</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
+          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
         </is>
       </c>
       <c r="E359" s="6" t="inlineStr">
@@ -10735,22 +10735,22 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>多模态训练数据</t>
+          <t>AI数据库</t>
         </is>
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>688787</t>
+          <t>688692</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>海天瑞声</t>
+          <t>达梦数据</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
+          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
         </is>
       </c>
       <c r="E360" s="6" t="inlineStr">
@@ -10762,22 +10762,22 @@
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>中文数据语料</t>
+          <t>多模态训练数据</t>
         </is>
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>688228</t>
+          <t>688787</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>开普云</t>
+          <t>海天瑞声</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
+          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
         </is>
       </c>
       <c r="E361" s="6" t="inlineStr">
@@ -10789,22 +10789,22 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>AI安全</t>
+          <t>中文数据语料</t>
         </is>
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>002439</t>
+          <t>688228</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>启明星辰</t>
+          <t>开普云</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
+          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
         </is>
       </c>
       <c r="E362" s="6" t="inlineStr">
@@ -10821,17 +10821,17 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>300454</t>
+          <t>002439</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>深信服</t>
+          <t>启明星辰</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
+          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
         </is>
       </c>
       <c r="E363" s="6" t="inlineStr">
@@ -10848,17 +10848,17 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>688561</t>
+          <t>300454</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>奇安信</t>
+          <t>深信服</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
+          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
         </is>
       </c>
       <c r="E364" s="6" t="inlineStr">
@@ -10875,17 +10875,17 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>688023</t>
+          <t>688561</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>安恒信息</t>
+          <t>奇安信</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
+          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
         </is>
       </c>
       <c r="E365" s="6" t="inlineStr">
@@ -10902,17 +10902,17 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>601360</t>
+          <t>688023</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>三六零</t>
+          <t>安恒信息</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
+          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
         </is>
       </c>
       <c r="E366" s="6" t="inlineStr">
@@ -10929,17 +10929,17 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>300369</t>
+          <t>601360</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>绿盟科技</t>
+          <t>三六零</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
+          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
         </is>
       </c>
       <c r="E367" s="6" t="inlineStr">
@@ -10951,22 +10951,22 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>AI办公Agent</t>
+          <t>AI安全</t>
         </is>
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>688111</t>
+          <t>300369</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>金山办公</t>
+          <t>绿盟科技</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
+          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
         </is>
       </c>
       <c r="E368" s="6" t="inlineStr">
@@ -10978,22 +10978,22 @@
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>PDF文档AI</t>
+          <t>AI办公Agent</t>
         </is>
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>688095</t>
+          <t>688111</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>福昕软件</t>
+          <t>金山办公</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
+          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
         </is>
       </c>
       <c r="E369" s="6" t="inlineStr">
@@ -11005,22 +11005,22 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>问财金融投研AI</t>
+          <t>PDF文档AI</t>
         </is>
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>300033</t>
+          <t>688095</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>同花顺</t>
+          <t>福昕软件</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
+          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
         </is>
       </c>
       <c r="E370" s="6" t="inlineStr">
@@ -11032,22 +11032,22 @@
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>保险IT AI应用</t>
+          <t>问财金融投研AI</t>
         </is>
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>603927</t>
+          <t>300033</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>中科软</t>
+          <t>同花顺</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
+          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
         </is>
       </c>
       <c r="E371" s="6" t="inlineStr">
@@ -11059,22 +11059,22 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>AI多媒体创作平台</t>
+          <t>保险IT AI应用</t>
         </is>
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>300624</t>
+          <t>603927</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>万兴科技</t>
+          <t>中科软</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
+          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
         </is>
       </c>
       <c r="E372" s="6" t="inlineStr">
@@ -11086,22 +11086,22 @@
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>AI+CAx工业设计软件</t>
+          <t>AI多媒体创作平台</t>
         </is>
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>688083</t>
+          <t>300624</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>中望软件</t>
+          <t>万兴科技</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
+          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
         </is>
       </c>
       <c r="E373" s="6" t="inlineStr">
@@ -11113,22 +11113,22 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>物理AI工业仿真</t>
+          <t>AI+CAx工业设计软件</t>
         </is>
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>688507</t>
+          <t>688083</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>索辰科技</t>
+          <t>中望软件</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
+          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
         </is>
       </c>
       <c r="E374" s="6" t="inlineStr">
@@ -11140,22 +11140,22 @@
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>流程工业AI</t>
+          <t>物理AI工业仿真</t>
         </is>
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>688777</t>
+          <t>688507</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>中控技术</t>
+          <t>索辰科技</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
+          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
         </is>
       </c>
       <c r="E375" s="6" t="inlineStr">
@@ -11167,22 +11167,22 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>激光加工AI工艺优化</t>
+          <t>流程工业AI</t>
         </is>
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>688188</t>
+          <t>688777</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>柏楚电子</t>
+          <t>中控技术</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
+          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
         </is>
       </c>
       <c r="E376" s="6" t="inlineStr">
@@ -11194,22 +11194,22 @@
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>AI分子砌块设计</t>
+          <t>激光加工AI工艺优化</t>
         </is>
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>300725</t>
+          <t>688188</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>药石科技</t>
+          <t>柏楚电子</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
+          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
         </is>
       </c>
       <c r="E377" s="6" t="inlineStr">
@@ -11221,22 +11221,22 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>AI片段分子库</t>
+          <t>AI分子砌块设计</t>
         </is>
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>688131</t>
+          <t>300725</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>皓元医药</t>
+          <t>药石科技</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
+          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
         </is>
       </c>
       <c r="E378" s="6" t="inlineStr">
@@ -11248,22 +11248,22 @@
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>AI药物发现</t>
+          <t>AI片段分子库</t>
         </is>
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>688222</t>
+          <t>688131</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>成都先导</t>
+          <t>皓元医药</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
+          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
         </is>
       </c>
       <c r="E379" s="6" t="inlineStr">
@@ -11275,22 +11275,22 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>AI辅助药物设计</t>
+          <t>AI药物发现</t>
         </is>
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>301230</t>
+          <t>688222</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>泓博医药</t>
+          <t>成都先导</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
+          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
         </is>
       </c>
       <c r="E380" s="6" t="inlineStr">
@@ -11302,22 +11302,22 @@
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>AI患者追踪系统</t>
+          <t>AI辅助药物设计</t>
         </is>
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>300451</t>
+          <t>301230</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>创业慧康</t>
+          <t>泓博医药</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
+          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
         </is>
       </c>
       <c r="E381" s="6" t="inlineStr">
@@ -11329,22 +11329,22 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>AI医学影像设备</t>
+          <t>AI患者追踪系统</t>
         </is>
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>688271</t>
+          <t>300451</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>联影医疗</t>
+          <t>创业慧康</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
+          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
         </is>
       </c>
       <c r="E382" s="6" t="inlineStr">
@@ -11356,22 +11356,22 @@
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>医疗信息化大模型</t>
+          <t>AI医学影像设备</t>
         </is>
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>300253</t>
+          <t>688271</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>卫宁健康</t>
+          <t>联影医疗</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
         </is>
       </c>
       <c r="E383" s="6" t="inlineStr">
@@ -11383,25 +11383,52 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
+          <t>医疗信息化大模型</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>300253</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>卫宁健康</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+        </is>
+      </c>
+      <c r="E384" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
           <t>医学检验AI服务</t>
         </is>
       </c>
-      <c r="B384" s="3" t="inlineStr">
+      <c r="B385" s="3" t="inlineStr">
         <is>
           <t>603108</t>
         </is>
       </c>
-      <c r="C384" s="2" t="inlineStr">
+      <c r="C385" s="2" t="inlineStr">
         <is>
           <t>润达医疗</t>
         </is>
       </c>
-      <c r="D384" s="2" t="inlineStr">
+      <c r="D385" s="2" t="inlineStr">
         <is>
           <t>证据中强但业绩弱：2025年报披露公司推出大模型产品CDx良医晓慧，覆盖数据基座、医生助理和健康智能体，已在华西、南方、齐鲁等医院落地；核心仍是IVD流通/实验室服务，主板块由IVD检验AI细化为医学检验AI服务。</t>
         </is>
       </c>
-      <c r="E384" s="6" t="inlineStr">
+      <c r="E385" s="6" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>

</xml_diff>

<commit_message>
docs: backup ai chain tracking artifacts
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -2829,12 +2829,12 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>高端电子布纯度高，港交所申请版本披露低Dk/Df、低CTE和石英布路线，并进入GPU/CPU等核心供应链；主线保留低介电电子布，石英布作为未来项，风险是估值拥挤和客户脱敏。证据A。</t>
+          <t>高端电子布纯度高，港交所申请版本披露低Dk/Df、低CTE和石英布路线，并进入GPU/CPU等核心供应链；主线保留低介电电子布，石英布作为未来项，风险是估值拥挤和客户脱敏。证据A。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/高优先观察”，不是基本面主受益；公司Low Dk/Low CTE电子布相关度高，但NVIDIA直签、寄售、提前一年锁产能未获A证据，需分布种收入、客户认证、交期/allocation和毛利兑现。</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-17证据分层</t>
         </is>
       </c>
     </row>
@@ -2937,12 +2937,12 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>PCB级RTF/HVLP进展最直接，年报披露RTF-3/4认证并批量供货、HVLP1-3批量供货、HVLP4小规模放量、HVLP5完成样品认证并推进导入；主板块由高端铜箔细化为HVLP铜箔，风险是HVLP5多客户、收入和毛利率仍需量化。证据A/B。</t>
+          <t>PCB级RTF/HVLP进展最直接，年报披露RTF-3/4认证并批量供货、HVLP1-3批量供货、HVLP4小规模放量、HVLP5完成样品认证并推进导入；主板块由高端铜箔细化为HVLP铜箔，风险是HVLP5多客户、收入和毛利率仍需量化。证据A/B。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/条件式HVLP期权”；HVLP4/5从纯watch提高到watch_to_soft验证优先级，但需多客户批量、加工费、电子电路铜箔收入占比和毛利证据，不能混同锂电铜箔修复。</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-17证据分层</t>
         </is>
       </c>
     </row>
@@ -3207,12 +3207,12 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>大陆CCL龙头，高速覆铜板、封装材料和客户覆盖最完整，是AI服务器高速PCB与M9/M10材料升级的稳健映射；主板块保留高端高速CCL，封装基板材料放备注，风险是周期、价格传导和高端占比。证据A/B。2026-06-16 JPM补充：报告强化M8/M9高端CCL、HPC CCL与载板用CCL/Q glass需求，支持高端高速CCL soft_bottleneck+；但不能替代公司分产品订单、涨价和客户锁料证据。</t>
+          <t>大陆CCL龙头，高速覆铜板、封装材料和客户覆盖最完整，是AI服务器高速PCB与M9/M10材料升级的稳健映射；主板块保留高端高速CCL，封装基板材料放备注，风险是周期、价格传导和高端占比。证据A/B。2026-06-16 JPM补充：报告强化M8/M9高端CCL、HPC CCL与载板用CCL/Q glass需求，支持高端高速CCL soft_bottleneck+；但不能替代公司分产品订单、涨价和客户锁料证据。 2026-06-17 HVLP4/T-glass复核：放“基本面主受益/质量锚”；高速CCL/prepreg是板级PCB材料主线最稳映射，但NVIDIA M9独家/直供等说法仍需公司、客户或正式供应链文件确认。</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>已处理；2026-06-16 JPM补充</t>
+          <t>已处理；2026-06-16 JPM补充；2026-06-17证据分层</t>
         </is>
       </c>
     </row>
@@ -3261,12 +3261,12 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>小市值高频高速覆铜板标的，AI服务器高速PCB/CCL需求可带来弹性；主板块保留高端高速CCL，核心看量产规模、客户结构和盈利修复，证据强度弱于生益/南亚。证据B/C。</t>
+          <t>小市值高频高速覆铜板标的，AI服务器高速PCB/CCL需求可带来弹性；主板块保留高端高速CCL，核心看量产规模、客户结构和盈利修复，证据强度弱于生益/南亚。证据B/C。 2026-06-17 HVLP4/T-glass复核：放“仅观察/PTFE-M10相邻线索”；PTFE高频覆铜板不属于HVLP4铜箔或T-glass直签锁产能主线，需AI server/M9-M10客户认证、量产收入和毛利证据后再上调。</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-17证据分层</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ai pcb lock capacity evidence
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -2829,12 +2829,12 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>高端电子布纯度高，港交所申请版本披露低Dk/Df、低CTE和石英布路线，并进入GPU/CPU等核心供应链；主线保留低介电电子布，石英布作为未来项，风险是估值拥挤和客户脱敏。证据A。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/高优先观察”，不是基本面主受益；公司Low Dk/Low CTE电子布相关度高，但NVIDIA直签、寄售、提前一年锁产能未获A证据，需分布种收入、客户认证、交期/allocation和毛利兑现。</t>
+          <t>高端电子布纯度高，港交所申请版本披露低Dk/Df、低CTE和石英布路线，并进入GPU/CPU等核心供应链；主线保留低介电电子布，石英布作为未来项，风险是估值拥挤和客户脱敏。证据A。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/高优先观察”，不是基本面主受益；公司Low Dk/Low CTE电子布相关度高，但官方追杀后，NVIDIA直签/寄售/提前一年锁产能仍未闭环；DIGITIMES只支持NVIDIA接洽Co-Tech讨论长期产能规划，仍需分布种收入、客户认证、交期/allocation和毛利兑现。</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>已处理；2026-06-17证据分层</t>
+          <t>已处理；2026-06-17证据分层；2026-06-17官方锁产追杀仍未闭环</t>
         </is>
       </c>
     </row>
@@ -2937,12 +2937,12 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>PCB级RTF/HVLP进展最直接，年报披露RTF-3/4认证并批量供货、HVLP1-3批量供货、HVLP4小规模放量、HVLP5完成样品认证并推进导入；主板块由高端铜箔细化为HVLP铜箔，风险是HVLP5多客户、收入和毛利率仍需量化。证据A/B。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/条件式HVLP期权”；HVLP4/5从纯watch提高到watch_to_soft验证优先级，但需多客户批量、加工费、电子电路铜箔收入占比和毛利证据，不能混同锂电铜箔修复。</t>
+          <t>PCB级RTF/HVLP进展最直接，年报披露RTF-3/4认证并批量供货、HVLP1-3批量供货、HVLP4小规模放量、HVLP5完成样品认证并推进导入；主板块由高端铜箔细化为HVLP铜箔，风险是HVLP5多客户、收入和毛利率仍需量化。证据A/B。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/条件式HVLP期权”；HVLP4/5从纯watch提高到watch_to_soft验证优先级，但需多客户批量、加工费、电子电路铜箔收入占比和毛利证据，不能混同锂电铜箔修复；官方追杀后，NVIDIA锁产/寄售/LTA/prepayment仍未闭环。</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>已处理；2026-06-17证据分层</t>
+          <t>已处理；2026-06-17证据分层；2026-06-17官方锁产追杀仍未闭环</t>
         </is>
       </c>
     </row>
@@ -3207,12 +3207,12 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>大陆CCL龙头，高速覆铜板、封装材料和客户覆盖最完整，是AI服务器高速PCB与M9/M10材料升级的稳健映射；主板块保留高端高速CCL，封装基板材料放备注，风险是周期、价格传导和高端占比。证据A/B。2026-06-16 JPM补充：报告强化M8/M9高端CCL、HPC CCL与载板用CCL/Q glass需求，支持高端高速CCL soft_bottleneck+；但不能替代公司分产品订单、涨价和客户锁料证据。 2026-06-17 HVLP4/T-glass复核：放“基本面主受益/质量锚”；高速CCL/prepreg是板级PCB材料主线最稳映射，但NVIDIA M9独家/直供等说法仍需公司、客户或正式供应链文件确认。</t>
+          <t>大陆CCL龙头，高速覆铜板、封装材料和客户覆盖最完整，是AI服务器高速PCB与M9/M10材料升级的稳健映射；主板块保留高端高速CCL，封装基板材料放备注，风险是周期、价格传导和高端占比。证据A/B。2026-06-16 JPM补充：报告强化M8/M9高端CCL、HPC CCL与载板用CCL/Q glass需求，支持高端高速CCL soft_bottleneck+；但不能替代公司分产品订单、涨价和客户锁料证据。 2026-06-17 HVLP4/T-glass复核：放“基本面主受益/质量锚”；高速CCL/prepreg是板级PCB材料主线最稳映射，但NVIDIA M9独家/直供/锁产等说法在官方追杀后仍未闭环，仍需公司、客户或正式供应链文件确认。</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>已处理；2026-06-16 JPM补充；2026-06-17证据分层</t>
+          <t>已处理；2026-06-16 JPM补充；2026-06-17证据分层；2026-06-17官方锁产追杀仍未闭环</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>已处理；2026-06-17证据分层</t>
+          <t>已处理；2026-06-17证据分层；2026-06-17官方锁产追杀仍未闭环</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: full backup 2026-07-25
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -1089,7 +1089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E391"/>
+  <dimension ref="A1:E392"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9493,49 +9493,49 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜主控SoC</t>
+          <t>端侧AI SoC</t>
         </is>
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>688608</t>
+          <t>301536</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>恒玄科技</t>
+          <t>星宸科技</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
+          <t>证据强：2025年报及2026年半年度业绩预告显示，公司以视觉AI SoC为核心，产品集成ISP、NPU、编解码、音频、显示及3D感知等能力，覆盖IPC/NVR智能安防、家用服务机器人、智能家居/办公/工业控制和车载DMS/OMS/CMS等场景；2025年智能安防、智能物联、智能车载收入占比分别为65.10%、22.14%、10.69%，SSR670已实现大规模商用，2026H1预告收入26.2—27.2亿元、扣非净利润7.0—7.8亿元。主板块归入端侧AI SoC；风险是高毛利与价量增长持续性、存货和经营现金流，以及AI眼镜、3D感知和车载前装仍处不同商业化阶段。</t>
         </is>
       </c>
       <c r="E314" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>新增；2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>智能穿戴SoC</t>
+          <t>AI眼镜主控SoC</t>
         </is>
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>688049</t>
+          <t>688608</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>炬芯科技</t>
+          <t>恒玄科技</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
+          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
         </is>
       </c>
       <c r="E315" s="6" t="inlineStr">
@@ -9547,22 +9547,22 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>端侧音视频SoC</t>
+          <t>智能穿戴SoC</t>
         </is>
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>688332</t>
+          <t>688049</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>中科蓝讯</t>
+          <t>炬芯科技</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
+          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
         </is>
       </c>
       <c r="E316" s="6" t="inlineStr">
@@ -9574,22 +9574,22 @@
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>端侧AI MCU</t>
+          <t>端侧音视频SoC</t>
         </is>
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>688018</t>
+          <t>688332</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>乐鑫科技</t>
+          <t>中科蓝讯</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
+          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
         </is>
       </c>
       <c r="E317" s="6" t="inlineStr">
@@ -9601,22 +9601,22 @@
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>端侧AI蜂窝模组</t>
+          <t>端侧AI MCU</t>
         </is>
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>603236</t>
+          <t>688018</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>移远通信</t>
+          <t>乐鑫科技</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
+          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
         </is>
       </c>
       <c r="E318" s="6" t="inlineStr">
@@ -9628,22 +9628,22 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>高算力智能模组</t>
+          <t>端侧AI蜂窝模组</t>
         </is>
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>002881</t>
+          <t>603236</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>美格智能</t>
+          <t>移远通信</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
+          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
         </is>
       </c>
       <c r="E319" s="6" t="inlineStr">
@@ -9655,22 +9655,22 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>端侧AI模组</t>
+          <t>高算力智能模组</t>
         </is>
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>300638</t>
+          <t>002881</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>广和通</t>
+          <t>美格智能</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
+          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
         </is>
       </c>
       <c r="E320" s="6" t="inlineStr">
@@ -9682,22 +9682,22 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>AIOS端侧智能</t>
+          <t>端侧AI模组</t>
         </is>
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>300496</t>
+          <t>300638</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>中科创达</t>
+          <t>广和通</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
+          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
         </is>
       </c>
       <c r="E321" s="6" t="inlineStr">
@@ -9709,22 +9709,22 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>AR光波导</t>
+          <t>AIOS端侧智能</t>
         </is>
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>002273</t>
+          <t>300496</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>水晶光电</t>
+          <t>中科创达</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
+          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
         </is>
       </c>
       <c r="E322" s="6" t="inlineStr">
@@ -9736,22 +9736,22 @@
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜光学模组</t>
+          <t>AR光波导</t>
         </is>
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>300433</t>
+          <t>002273</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>蓝思科技</t>
+          <t>水晶光电</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
+          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
         </is>
       </c>
       <c r="E323" s="6" t="inlineStr">
@@ -9763,22 +9763,22 @@
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>AR投影光机</t>
+          <t>AI眼镜光学模组</t>
         </is>
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>688010</t>
+          <t>300433</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>福光股份</t>
+          <t>蓝思科技</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
+          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
         </is>
       </c>
       <c r="E324" s="6" t="inlineStr">
@@ -9790,22 +9790,22 @@
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>硅基OLED微显示</t>
+          <t>AR投影光机</t>
         </is>
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>688496</t>
+          <t>688010</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>清越科技</t>
+          <t>福光股份</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
+          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
         </is>
       </c>
       <c r="E325" s="6" t="inlineStr">
@@ -9817,22 +9817,22 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED光机</t>
+          <t>硅基OLED微显示</t>
         </is>
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>300296</t>
+          <t>688496</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>利亚德</t>
+          <t>清越科技</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
+          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
         </is>
       </c>
       <c r="E326" s="6" t="inlineStr">
@@ -9844,22 +9844,22 @@
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED微显示</t>
+          <t>AI眼镜MicroLED光机</t>
         </is>
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>300323</t>
+          <t>300296</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>京东方华灿</t>
+          <t>利亚德</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
+          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
         </is>
       </c>
       <c r="E327" s="6" t="inlineStr">
@@ -9871,22 +9871,22 @@
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MicroLED芯片</t>
+          <t>AI眼镜MicroLED微显示</t>
         </is>
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>600703</t>
+          <t>300323</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>三安光电</t>
+          <t>京东方华灿</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
+          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
         </is>
       </c>
       <c r="E328" s="6" t="inlineStr">
@@ -9898,22 +9898,22 @@
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>OLED-MicroLED显示</t>
+          <t>MicroLED芯片</t>
         </is>
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>002387</t>
+          <t>600703</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>维信诺</t>
+          <t>三安光电</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
+          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
         </is>
       </c>
       <c r="E329" s="6" t="inlineStr">
@@ -9925,22 +9925,22 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜CIS</t>
+          <t>OLED-MicroLED显示</t>
         </is>
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>688213</t>
+          <t>002387</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>思特威</t>
+          <t>维信诺</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
+          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
         </is>
       </c>
       <c r="E330" s="6" t="inlineStr">
@@ -9957,17 +9957,17 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>688728</t>
+          <t>688213</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>格科微</t>
+          <t>思特威</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
+          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
         </is>
       </c>
       <c r="E331" s="6" t="inlineStr">
@@ -9979,22 +9979,22 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜视觉算法</t>
+          <t>AI眼镜CIS</t>
         </is>
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>688088</t>
+          <t>688728</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>虹软科技</t>
+          <t>格科微</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
+          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
         </is>
       </c>
       <c r="E332" s="6" t="inlineStr">
@@ -10006,22 +10006,22 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜模拟芯片</t>
+          <t>AI眼镜视觉算法</t>
         </is>
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>688798</t>
+          <t>688088</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>艾为电子</t>
+          <t>虹软科技</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
+          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
         </is>
       </c>
       <c r="E333" s="6" t="inlineStr">
@@ -10033,22 +10033,22 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜声学传感器</t>
+          <t>AI眼镜模拟芯片</t>
         </is>
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>688286</t>
+          <t>688798</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>敏芯股份</t>
+          <t>艾为电子</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
+          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
         </is>
       </c>
       <c r="E334" s="6" t="inlineStr">
@@ -10060,22 +10060,22 @@
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>消费锂电池</t>
+          <t>AI眼镜声学传感器</t>
         </is>
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>688772</t>
+          <t>688286</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>珠海冠宇</t>
+          <t>敏芯股份</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
+          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
         </is>
       </c>
       <c r="E335" s="6" t="inlineStr">
@@ -10087,22 +10087,22 @@
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜电池</t>
+          <t>消费锂电池</t>
         </is>
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>001283</t>
+          <t>688772</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>豪鹏科技</t>
+          <t>珠海冠宇</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
+          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
         </is>
       </c>
       <c r="E336" s="6" t="inlineStr">
@@ -10114,22 +10114,22 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜结构件</t>
+          <t>AI智能眼镜电池</t>
         </is>
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>300115</t>
+          <t>001283</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>长盈精密</t>
+          <t>豪鹏科技</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
+          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
         </is>
       </c>
       <c r="E337" s="6" t="inlineStr">
@@ -10141,22 +10141,22 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜整机</t>
+          <t>AI眼镜结构件</t>
         </is>
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>002241</t>
+          <t>300115</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>歌尔股份</t>
+          <t>长盈精密</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
+          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
         </is>
       </c>
       <c r="E338" s="6" t="inlineStr">
@@ -10168,22 +10168,22 @@
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>AI终端精密功能件</t>
+          <t>AI智能眼镜整机</t>
         </is>
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>002600</t>
+          <t>002241</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>领益智造</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
+          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
         </is>
       </c>
       <c r="E339" s="6" t="inlineStr">
@@ -10195,22 +10195,22 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>机器人3D视觉</t>
+          <t>AI终端精密功能件</t>
         </is>
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>688322</t>
+          <t>002600</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>奥比中光</t>
+          <t>领益智造</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
+          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
         </is>
       </c>
       <c r="E340" s="6" t="inlineStr">
@@ -10222,22 +10222,22 @@
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>机器人力传感器</t>
+          <t>机器人3D视觉</t>
         </is>
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>603662</t>
+          <t>688322</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>柯力传感</t>
+          <t>奥比中光</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
+          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
         </is>
       </c>
       <c r="E341" s="6" t="inlineStr">
@@ -10254,17 +10254,17 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>301413</t>
+          <t>603662</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>安培龙</t>
+          <t>柯力传感</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
+          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
         </is>
       </c>
       <c r="E342" s="6" t="inlineStr">
@@ -10281,17 +10281,17 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>300354</t>
+          <t>301413</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>东华测试</t>
+          <t>安培龙</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
+          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
         </is>
       </c>
       <c r="E343" s="6" t="inlineStr">
@@ -10303,22 +10303,22 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>机器人电子皮肤</t>
+          <t>机器人力传感器</t>
         </is>
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>300007</t>
+          <t>300354</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>汉威科技</t>
+          <t>东华测试</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
+          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
         </is>
       </c>
       <c r="E344" s="6" t="inlineStr">
@@ -10330,22 +10330,22 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>机器人谐波减速器</t>
+          <t>机器人电子皮肤</t>
         </is>
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>688017</t>
+          <t>300007</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>绿的谐波</t>
+          <t>汉威科技</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
+          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
         </is>
       </c>
       <c r="E345" s="6" t="inlineStr">
@@ -10357,22 +10357,22 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>机器人精密减速器</t>
+          <t>机器人谐波减速器</t>
         </is>
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>002896</t>
+          <t>688017</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>中大力德</t>
+          <t>绿的谐波</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
+          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
         </is>
       </c>
       <c r="E346" s="6" t="inlineStr">
@@ -10389,17 +10389,17 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>002472</t>
+          <t>002896</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>双环传动</t>
+          <t>中大力德</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
+          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
         </is>
       </c>
       <c r="E347" s="6" t="inlineStr">
@@ -10411,22 +10411,22 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>行星滚柱丝杠</t>
+          <t>机器人精密减速器</t>
         </is>
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>603667</t>
+          <t>002472</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>五洲新春</t>
+          <t>双环传动</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
+          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
         </is>
       </c>
       <c r="E348" s="6" t="inlineStr">
@@ -10443,17 +10443,17 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>601100</t>
+          <t>603667</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>恒立液压</t>
+          <t>五洲新春</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
+          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
         </is>
       </c>
       <c r="E349" s="6" t="inlineStr">
@@ -10470,17 +10470,17 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>688678</t>
+          <t>601100</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>福立旺</t>
+          <t>恒立液压</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
+          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
         </is>
       </c>
       <c r="E350" s="6" t="inlineStr">
@@ -10497,17 +10497,17 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>603009</t>
+          <t>688678</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>北特科技</t>
+          <t>福立旺</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
+          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
         </is>
       </c>
       <c r="E351" s="6" t="inlineStr">
@@ -10519,22 +10519,22 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>机器人执行器</t>
+          <t>行星滚柱丝杠</t>
         </is>
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>601689</t>
+          <t>603009</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>拓普集团</t>
+          <t>北特科技</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
+          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
         </is>
       </c>
       <c r="E352" s="6" t="inlineStr">
@@ -10546,22 +10546,22 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>机器人伺服驱动</t>
+          <t>机器人执行器</t>
         </is>
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>300124</t>
+          <t>601689</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>汇川技术</t>
+          <t>拓普集团</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
+          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
         </is>
       </c>
       <c r="E353" s="6" t="inlineStr">
@@ -10573,22 +10573,22 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>机器人驱控系统</t>
+          <t>机器人伺服驱动</t>
         </is>
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>002979</t>
+          <t>300124</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>雷赛智能</t>
+          <t>汇川技术</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
+          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
         </is>
       </c>
       <c r="E354" s="6" t="inlineStr">
@@ -10600,22 +10600,22 @@
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>空心杯电机</t>
+          <t>机器人驱控系统</t>
         </is>
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>603728</t>
+          <t>002979</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>鸣志电器</t>
+          <t>雷赛智能</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
+          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
         </is>
       </c>
       <c r="E355" s="6" t="inlineStr">
@@ -10627,22 +10627,22 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>行业大模型+Agent平台</t>
+          <t>空心杯电机</t>
         </is>
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>300229</t>
+          <t>603728</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>拓尔思</t>
+          <t>鸣志电器</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
+          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
         </is>
       </c>
       <c r="E356" s="6" t="inlineStr">
@@ -10654,22 +10654,22 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>行业大模型训推一体</t>
+          <t>行业大模型+Agent平台</t>
         </is>
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>688327</t>
+          <t>300229</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>云从科技</t>
+          <t>拓尔思</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
+          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
         </is>
       </c>
       <c r="E357" s="6" t="inlineStr">
@@ -10681,22 +10681,22 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>国产算力大模型底座</t>
+          <t>行业大模型训推一体</t>
         </is>
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>002230</t>
+          <t>688327</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>科大讯飞</t>
+          <t>云从科技</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
         </is>
       </c>
       <c r="E358" s="6" t="inlineStr">
@@ -10708,22 +10708,22 @@
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>企业AI平台</t>
+          <t>国产算力大模型底座</t>
         </is>
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>600588</t>
+          <t>002230</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>用友网络</t>
+          <t>科大讯飞</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
+          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
         </is>
       </c>
       <c r="E359" s="6" t="inlineStr">
@@ -10735,22 +10735,22 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>企业级AI应用平台</t>
+          <t>企业AI平台</t>
         </is>
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>300170</t>
+          <t>600588</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>汉得信息</t>
+          <t>用友网络</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
+          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
         </is>
       </c>
       <c r="E360" s="6" t="inlineStr">
@@ -10762,22 +10762,22 @@
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>行业AI智能体平台</t>
+          <t>企业级AI应用平台</t>
         </is>
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>301236</t>
+          <t>300170</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>软通动力</t>
+          <t>汉得信息</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
         </is>
       </c>
       <c r="E361" s="6" t="inlineStr">
@@ -10789,22 +10789,22 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>制造业AI智能体平台</t>
+          <t>行业AI智能体平台</t>
         </is>
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>300378</t>
+          <t>301236</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>鼎捷数智</t>
+          <t>软通动力</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
         </is>
       </c>
       <c r="E362" s="6" t="inlineStr">
@@ -10816,22 +10816,22 @@
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>行业AI交付</t>
+          <t>制造业AI智能体平台</t>
         </is>
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>002649</t>
+          <t>300378</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>博彦科技</t>
+          <t>鼎捷数智</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
+          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
         </is>
       </c>
       <c r="E363" s="6" t="inlineStr">
@@ -10843,22 +10843,22 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>AI数据基础设施软件</t>
+          <t>行业AI交付</t>
         </is>
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>688031</t>
+          <t>002649</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>星环科技</t>
+          <t>博彦科技</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
         </is>
       </c>
       <c r="E364" s="6" t="inlineStr">
@@ -10870,22 +10870,22 @@
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>向量数据库</t>
+          <t>AI数据基础设施软件</t>
         </is>
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>603138</t>
+          <t>688031</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>海量数据</t>
+          <t>星环科技</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
+          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
         </is>
       </c>
       <c r="E365" s="6" t="inlineStr">
@@ -10897,22 +10897,22 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>AI数据库</t>
+          <t>向量数据库</t>
         </is>
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>688692</t>
+          <t>603138</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>达梦数据</t>
+          <t>海量数据</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
+          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
         </is>
       </c>
       <c r="E366" s="6" t="inlineStr">
@@ -10924,22 +10924,22 @@
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>多模态训练数据</t>
+          <t>AI数据库</t>
         </is>
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>688787</t>
+          <t>688692</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>海天瑞声</t>
+          <t>达梦数据</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
+          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
         </is>
       </c>
       <c r="E367" s="6" t="inlineStr">
@@ -10951,22 +10951,22 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>中文数据语料</t>
+          <t>多模态训练数据</t>
         </is>
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>688228</t>
+          <t>688787</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>开普云</t>
+          <t>海天瑞声</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
+          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
         </is>
       </c>
       <c r="E368" s="6" t="inlineStr">
@@ -10978,22 +10978,22 @@
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>AI安全</t>
+          <t>中文数据语料</t>
         </is>
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>002439</t>
+          <t>688228</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>启明星辰</t>
+          <t>开普云</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
+          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
         </is>
       </c>
       <c r="E369" s="6" t="inlineStr">
@@ -11010,17 +11010,17 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>300454</t>
+          <t>002439</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>深信服</t>
+          <t>启明星辰</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
+          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
         </is>
       </c>
       <c r="E370" s="6" t="inlineStr">
@@ -11037,17 +11037,17 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>688561</t>
+          <t>300454</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>奇安信</t>
+          <t>深信服</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
+          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
         </is>
       </c>
       <c r="E371" s="6" t="inlineStr">
@@ -11064,17 +11064,17 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>688023</t>
+          <t>688561</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>安恒信息</t>
+          <t>奇安信</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
+          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
         </is>
       </c>
       <c r="E372" s="6" t="inlineStr">
@@ -11091,17 +11091,17 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>601360</t>
+          <t>688023</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>三六零</t>
+          <t>安恒信息</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
+          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
         </is>
       </c>
       <c r="E373" s="6" t="inlineStr">
@@ -11118,17 +11118,17 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>300369</t>
+          <t>601360</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>绿盟科技</t>
+          <t>三六零</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
+          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
         </is>
       </c>
       <c r="E374" s="6" t="inlineStr">
@@ -11140,22 +11140,22 @@
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>AI办公Agent</t>
+          <t>AI安全</t>
         </is>
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>688111</t>
+          <t>300369</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>金山办公</t>
+          <t>绿盟科技</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
+          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
         </is>
       </c>
       <c r="E375" s="6" t="inlineStr">
@@ -11167,22 +11167,22 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>PDF文档AI</t>
+          <t>AI办公Agent</t>
         </is>
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>688095</t>
+          <t>688111</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>福昕软件</t>
+          <t>金山办公</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
+          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
         </is>
       </c>
       <c r="E376" s="6" t="inlineStr">
@@ -11194,22 +11194,22 @@
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>问财金融投研AI</t>
+          <t>PDF文档AI</t>
         </is>
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>300033</t>
+          <t>688095</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>同花顺</t>
+          <t>福昕软件</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
+          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
         </is>
       </c>
       <c r="E377" s="6" t="inlineStr">
@@ -11221,22 +11221,22 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>保险IT AI应用</t>
+          <t>问财金融投研AI</t>
         </is>
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>603927</t>
+          <t>300033</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>中科软</t>
+          <t>同花顺</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
+          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
         </is>
       </c>
       <c r="E378" s="6" t="inlineStr">
@@ -11248,22 +11248,22 @@
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>AI多媒体创作平台</t>
+          <t>保险IT AI应用</t>
         </is>
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>300624</t>
+          <t>603927</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>万兴科技</t>
+          <t>中科软</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
+          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
         </is>
       </c>
       <c r="E379" s="6" t="inlineStr">
@@ -11275,22 +11275,22 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>AI+CAx工业设计软件</t>
+          <t>AI多媒体创作平台</t>
         </is>
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>688083</t>
+          <t>300624</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>中望软件</t>
+          <t>万兴科技</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
+          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
         </is>
       </c>
       <c r="E380" s="6" t="inlineStr">
@@ -11302,22 +11302,22 @@
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>物理AI工业仿真</t>
+          <t>AI+CAx工业设计软件</t>
         </is>
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>688507</t>
+          <t>688083</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>索辰科技</t>
+          <t>中望软件</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
+          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
         </is>
       </c>
       <c r="E381" s="6" t="inlineStr">
@@ -11329,22 +11329,22 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>流程工业AI</t>
+          <t>物理AI工业仿真</t>
         </is>
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>688777</t>
+          <t>688507</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>中控技术</t>
+          <t>索辰科技</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
+          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
         </is>
       </c>
       <c r="E382" s="6" t="inlineStr">
@@ -11356,22 +11356,22 @@
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>激光加工AI工艺优化</t>
+          <t>流程工业AI</t>
         </is>
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>688188</t>
+          <t>688777</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>柏楚电子</t>
+          <t>中控技术</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
+          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
         </is>
       </c>
       <c r="E383" s="6" t="inlineStr">
@@ -11383,22 +11383,22 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>AI分子砌块设计</t>
+          <t>激光加工AI工艺优化</t>
         </is>
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>300725</t>
+          <t>688188</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>药石科技</t>
+          <t>柏楚电子</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
+          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
         </is>
       </c>
       <c r="E384" s="6" t="inlineStr">
@@ -11410,22 +11410,22 @@
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>AI片段分子库</t>
+          <t>AI分子砌块设计</t>
         </is>
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>688131</t>
+          <t>300725</t>
         </is>
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>皓元医药</t>
+          <t>药石科技</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
+          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
         </is>
       </c>
       <c r="E385" s="6" t="inlineStr">
@@ -11437,22 +11437,22 @@
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>AI药物发现</t>
+          <t>AI片段分子库</t>
         </is>
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>688222</t>
+          <t>688131</t>
         </is>
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>成都先导</t>
+          <t>皓元医药</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
+          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
         </is>
       </c>
       <c r="E386" s="6" t="inlineStr">
@@ -11464,22 +11464,22 @@
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>AI辅助药物设计</t>
+          <t>AI药物发现</t>
         </is>
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>301230</t>
+          <t>688222</t>
         </is>
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>泓博医药</t>
+          <t>成都先导</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
+          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
         </is>
       </c>
       <c r="E387" s="6" t="inlineStr">
@@ -11491,22 +11491,22 @@
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>AI患者追踪系统</t>
+          <t>AI辅助药物设计</t>
         </is>
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>300451</t>
+          <t>301230</t>
         </is>
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>创业慧康</t>
+          <t>泓博医药</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
+          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
         </is>
       </c>
       <c r="E388" s="6" t="inlineStr">
@@ -11518,22 +11518,22 @@
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>AI医学影像设备</t>
+          <t>AI患者追踪系统</t>
         </is>
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>688271</t>
+          <t>300451</t>
         </is>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>联影医疗</t>
+          <t>创业慧康</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
+          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
         </is>
       </c>
       <c r="E389" s="6" t="inlineStr">
@@ -11545,22 +11545,22 @@
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>医疗信息化大模型</t>
+          <t>AI医学影像设备</t>
         </is>
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>300253</t>
+          <t>688271</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>卫宁健康</t>
+          <t>联影医疗</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
         </is>
       </c>
       <c r="E390" s="6" t="inlineStr">
@@ -11572,25 +11572,52 @@
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
+          <t>医疗信息化大模型</t>
+        </is>
+      </c>
+      <c r="B391" s="3" t="inlineStr">
+        <is>
+          <t>300253</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>卫宁健康</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+        </is>
+      </c>
+      <c r="E391" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
           <t>医学检验AI服务</t>
         </is>
       </c>
-      <c r="B391" s="3" t="inlineStr">
+      <c r="B392" s="3" t="inlineStr">
         <is>
           <t>603108</t>
         </is>
       </c>
-      <c r="C391" s="2" t="inlineStr">
+      <c r="C392" s="2" t="inlineStr">
         <is>
           <t>润达医疗</t>
         </is>
       </c>
-      <c r="D391" s="2" t="inlineStr">
+      <c r="D392" s="2" t="inlineStr">
         <is>
           <t>证据中强但业绩弱：2025年报披露公司推出大模型产品CDx良医晓慧，覆盖数据基座、医生助理和健康智能体，已在华西、南方、齐鲁等医院落地；核心仍是IVD流通/实验室服务，主板块由IVD检验AI细化为医学检验AI服务。</t>
         </is>
       </c>
-      <c r="E391" s="6" t="inlineStr">
+      <c r="E392" s="6" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>

</xml_diff>

<commit_message>
docs: update Rockchip AI chain entry
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -9427,12 +9427,12 @@
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/半年报披露智能应用处理器为核心收入来源，RK3588/RK3576等SoC和自研NPU支持端侧模型、AIoT多场景落地；主板块从“端侧AI处理器”规范为“端侧AI SoC”，跟踪高端SoC新品、客户导入和AIoT需求持续性。</t>
+          <t>证据强：2026年一季报及2026年半年度业绩预告显示，公司采用“AIoT SoC算力平台+AI协处理器”双轨路线，RK3588、RK3576、RV11系列持续高速增长，RK182X已量产并预计下半年开始放量；以RK3588为例，芯片集成CPU、GPU、6TOPS自研NPU、ISP及8K音视频编解码能力，终端覆盖机器人、机器视觉/安防、工业控制、智能座舱、商显/办公、智能家居及教育娱乐等消费电子。2026H1预告营收28.70—29.10亿元、归母净利润8.50—9.10亿元、扣非净利润8.30—8.90亿元（均未经审计）。主板块归入端侧AI SoC；风险是存储及载板等原材料涨价/短缺、消费类终端承压，以及新品导入和放量不及预期。</t>
         </is>
       </c>
       <c r="E311" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>更新；2026-07-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: full backup research updates 2026-07-25
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -9508,12 +9508,12 @@
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及2026年半年度业绩预告显示，公司以视觉AI SoC为核心，产品集成ISP、NPU、编解码、音频、显示及3D感知等能力，覆盖IPC/NVR智能安防、家用服务机器人、智能家居/办公/工业控制和车载DMS/OMS/CMS等场景；2025年智能安防、智能物联、智能车载收入占比分别为65.10%、22.14%、10.69%，SSR670已实现大规模商用，2026H1预告收入26.2—27.2亿元、扣非净利润7.0—7.8亿元。主板块归入端侧AI SoC；风险是高毛利与价量增长持续性、存货和经营现金流，以及AI眼镜、3D感知和车载前装仍处不同商业化阶段。</t>
+          <t>证据强（截至2026-07-25）：公司以视觉AI SoC为核心，核心芯片集成ISP、NPU、编解码、音频/显示等IP；主要产品/目标终端包括IPC/NVR（SSR670G）、家用服务及户外等机器人、智能家居/办公/工业、智能穿戴和车载记录仪/DMS/OMS/CMS/L0-L2辅助驾驶，另布局SPAD 3D感知与蓝牙。已形成收入：2025年智能安防19.35亿元/65.10%、智能物联6.58亿元/22.14%、智能车载3.18亿元/10.69%；2026H1预告收入26.2—27.2亿元、归母8.2—9.0亿元、扣非7.0—7.8亿元（未经审计；7月22日公告称无需修正），SSR670系列公司称已大规模商用。商业化边界：AI眼镜SSC309QL仅小规模量产，另有5—6家客户开发中，订单/独立收入N/A；机器人2025年出货超1,000万颗但独立收入N/A，具身“小脑/大脑”仍在研；SS901公司IR称已在国内一线自主品牌主力车型量产上车，其他车载/3D项目的导入或规划不等于订单/收入。PE(TTM，用户口径)=24.4—28.4x：总市值555.82亿元（东方财富，2026-07-24收盘）÷[(2026H1扣非预告7.0—7.8亿元−2026Q1扣非2.0998亿元)×4]，非标准近四季PE。证据状态：财务/分部=confirmed_official；产品/客户进展=company_claim；估值=market_data_vendor；annualized_core_gap_status=insufficient、formal_surprise_status=N/A（缺公告前FY归母点时共识）。风险：半年度预告待8月27日正式半年报验证，毛利率、现金流、存货、价量与新品放量持续性待核。</t>
         </is>
       </c>
       <c r="E314" s="6" t="inlineStr">
         <is>
-          <t>新增；2026-07-24</t>
+          <t>更新；2026-07-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: full backup 2026-07-31 company tracking
</commit_message>
<xml_diff>
--- a/AI产业链.xlsx
+++ b/AI产业链.xlsx
@@ -801,6 +801,32 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>OpenAI Codex</author>
+  </authors>
+  <commentList>
+    <comment ref="D21" authorId="0" shapeId="0">
+      <text>
+        <t>更新日期：2026-07-31
+证据等级：A，均为公司、交易所正式披露。
+来源：
+1. 2026年半年度业绩预告（2026-07-07）：
+https://static.cninfo.com.cn/finalpage/2026-07-07/1225412846.PDF
+2. 2025年度募集资金存放与实际使用情况专项报告（TFLN阶段，2026-03-24）：
+https://static.cninfo.com.cn/finalpage/2026-03-24/1225026100.PDF
+3. 发行股份、可转换公司债券及支付现金购买资产并募集配套资金暨关联交易报告书（草案，2026-06-25）：
+https://static.cninfo.com.cn/finalpage/2026-06-25/1225388287.PDF
+4. 深交所重组项目动态（项目ID 1004186，查询日2026-07-31）：
+https://listing.szse.cn/api/ras/projectrends/details?id=1004186
+口径：数据中心/AI集群PAM4 TFLN仍为验证送样；安捷讯项目当前“已问询”，尚未完成交割，不作为已确认并表收入。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1641,7 +1667,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>光通讯器件收入2025年高增，产品覆盖隔离器、WDM、FAU/MT、CPO光纤阵列及薄膜铌酸锂调制器/芯片；主板块改为TFLN，法拉第旋光片、AWG、OCS、薄膜滤波片、光纤连接和PM光纤并入备注，风险是TFLN量产收入、OCS代工占比低和重大资产重组不确定。证据B。</t>
+          <t>光通信器件是当前业绩主线：2026H1归母预告1.40–1.50亿元、同比+170%–190%（未经审计；Q1增长含武汉光库并表）。TFLN为高端调制器路线：骨干网CDM芯片已批量出货、模块小批量；DCI及数据中心/AI集群PAM4仍验证送样且进度延后，不能按800G/1.6T量产收入计。安捷讯拟收购补高速模块组件及机房光互联，MT/FAU/MPO类存在产品重叠；截至2026-07-31深交所项目状态为“已问询”，交割后方能并表，若2026H2交割，完整年度贡献最早看2027。主板块保留TFLN，风险是验证转量产、项目效益/利用率、审批交割及数通产品降价。证据A（截至2026-07-31）。</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -11626,5 +11652,6 @@
   </sheetData>
   <autoFilter ref="A1:D605"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>